<commit_message>
ssh_connection moved to TestSuiteSetup.py under Test_Setup directory
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -95,73 +95,73 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_BQR</t>
   </si>
   <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_Filters_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Filters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_ChargeSlip_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_ChargeSlip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_AutoLogin_Disabled_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_AutoLogin_Enabled_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_SendReceipt_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_SendReceipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_PrintReceipt_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_PrintReceipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_English_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Multilanguage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_English_to_Hindi_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_to_English_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_Lang_selection_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Upfront_Mobile_Number_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sample</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_Filters_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Filters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_ChargeSlip_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_ChargeSlip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_AutoLogin_Disabled_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_AutoLogin_Enabled_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_SendReceipt_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_SendReceipt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_PrintReceipt_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_PrintReceipt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_English_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Multilanguage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_English_to_Hindi_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_to_English_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_Lang_selection_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Upfront_Mobile_Number_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sample</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -411,14 +411,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -547,15 +546,15 @@
         <v>6</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>24</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>6</v>
@@ -566,10 +565,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>6</v>
@@ -580,10 +579,10 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>6</v>
@@ -594,10 +593,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>6</v>
@@ -608,10 +607,10 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>6</v>
@@ -622,10 +621,10 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>6</v>
@@ -636,10 +635,10 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>36</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
@@ -651,10 +650,10 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>6</v>
@@ -665,10 +664,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>6</v>
@@ -679,10 +678,10 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>6</v>
@@ -693,10 +692,10 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>6</v>
@@ -707,10 +706,10 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>6</v>
@@ -721,16 +720,16 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="C22" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -759,7 +758,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -792,7 +791,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -825,7 +824,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -858,7 +857,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -917,7 +916,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -950,7 +949,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -983,7 +982,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
methods and variables cleanup - First commit
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="49">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_success_2</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -182,7 +185,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -232,6 +235,13 @@
       <family val="3"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF00627A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -288,7 +298,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -330,6 +340,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -411,7 +425,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -732,8 +746,19 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D23" s="5"/>
+    <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -758,7 +783,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -791,7 +816,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -824,7 +849,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -857,7 +882,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -881,13 +906,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -916,7 +941,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -949,7 +974,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -982,7 +1007,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Methods and Variables cleanup 2nd commit
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -50,15 +50,18 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_Signature_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Signature</t>
+  </si>
+  <si>
     <t xml:space="preserve">False</t>
   </si>
   <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_Signature_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Signature</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_UI_SA_TxnHistory_Void_01</t>
   </si>
   <si>
@@ -159,9 +162,6 @@
   </si>
   <si>
     <t xml:space="preserve">test_sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_success_2</t>
@@ -425,11 +425,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.95"/>
   </cols>
@@ -473,7 +472,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F3" s="6"/>
       <c r="H3" s="7"/>
@@ -481,269 +480,269 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>35</v>
-      </c>
       <c r="C17" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -751,13 +750,13 @@
         <v>45</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -783,7 +782,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -816,7 +815,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -849,7 +848,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -882,7 +881,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -915,7 +914,7 @@
         <v>48</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -941,7 +940,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -974,7 +973,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1007,7 +1006,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Latest code with changes from Nivin, Avinash and Vineeth
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -50,118 +50,118 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
+    <t xml:space="preserve">False</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_Signature_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Signature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_Void_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Void</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Promo_Displayed_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Promo_Displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Logout_Success_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Logout_Success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Login_Invalid_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Login_Invalid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_CheckStatus_UPI_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_UPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_CheckStatus_BQR_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_BQR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_Filters_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Filters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_ChargeSlip_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_ChargeSlip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_AutoLogin_Disabled_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_AutoLogin_Enabled_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_SendReceipt_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_SendReceipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_PrintReceipt_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_PrintReceipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_English_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Multilanguage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_English_to_Hindi_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_to_English_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Multilanguage_Lang_selection_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_Upfront_Mobile_Number_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sample</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_Signature_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Signature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">False</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_Void_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Void</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Promo_Displayed_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Promo_Displayed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Logout_Success_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Logout_Success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Login_Invalid_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Login_Invalid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_CheckStatus_UPI_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_UPI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_CheckStatus_BQR_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_BQR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_Filters_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Filters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_ChargeSlip_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_ChargeSlip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_AutoLogin_Disabled_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_AutoLogin_Enabled_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_AutoLogin_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_SendReceipt_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_SendReceipt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_PrintReceipt_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_PrintReceipt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_English_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Multilanguage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_English_to_Hindi_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_Hindi_to_English_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Multilanguage_Lang_selection_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_SA_Upfront_Mobile_Number_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sample</t>
   </si>
   <si>
     <t xml:space="preserve">test_success_2</t>
@@ -425,7 +425,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -472,7 +472,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F3" s="6"/>
       <c r="H3" s="7"/>
@@ -480,269 +480,269 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>12</v>
-      </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>20</v>
-      </c>
       <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>26</v>
-      </c>
       <c r="C11" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="C12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="C13" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="C14" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="C15" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>36</v>
-      </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>42</v>
-      </c>
       <c r="C21" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="C22" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -750,13 +750,13 @@
         <v>45</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +782,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -815,7 +815,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -848,7 +848,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -881,7 +881,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -914,7 +914,7 @@
         <v>48</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -940,7 +940,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -973,7 +973,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1006,7 +1006,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Methods and variables cleanup -4th commit
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -89,6 +89,9 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_UPI</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_UI_SA_CheckStatus_BQR_01</t>
   </si>
   <si>
@@ -159,9 +162,6 @@
   </si>
   <si>
     <t xml:space="preserve">test_sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_success_2</t>
@@ -425,7 +425,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -545,15 +545,15 @@
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>6</v>
@@ -564,10 +564,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>6</v>
@@ -578,10 +578,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>6</v>
@@ -592,10 +592,10 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>6</v>
@@ -606,10 +606,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>6</v>
@@ -620,10 +620,10 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>6</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>6</v>
@@ -648,10 +648,10 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
@@ -663,10 +663,10 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>6</v>
@@ -677,10 +677,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>6</v>
@@ -691,10 +691,10 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>6</v>
@@ -705,10 +705,10 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>6</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>6</v>
@@ -733,16 +733,16 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -750,13 +750,13 @@
         <v>45</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +782,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -815,7 +815,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -848,7 +848,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -881,7 +881,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -940,7 +940,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -973,7 +973,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1006,7 +1006,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
end of cleanup activity
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -50,15 +50,18 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_SA_TxnHistory_Signature_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Signature</t>
+  </si>
+  <si>
     <t xml:space="preserve">False</t>
   </si>
   <si>
-    <t xml:space="preserve">test_UI_SA_TxnHistory_Signature_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_TxnHistory_Signature</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_UI_SA_TxnHistory_Void_01</t>
   </si>
   <si>
@@ -87,9 +90,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_CheckStatus_UPI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_UI_SA_CheckStatus_BQR_01</t>
@@ -425,7 +425,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="14.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -472,7 +472,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F3" s="6"/>
       <c r="H3" s="7"/>
@@ -480,38 +480,38 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>6</v>
@@ -522,30 +522,30 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -559,7 +559,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -573,7 +573,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -587,7 +587,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -601,7 +601,7 @@
         <v>6</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -615,7 +615,7 @@
         <v>6</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -629,7 +629,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -643,7 +643,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -672,7 +672,7 @@
         <v>6</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -686,7 +686,7 @@
         <v>6</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -700,7 +700,7 @@
         <v>6</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -714,7 +714,7 @@
         <v>6</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -728,7 +728,7 @@
         <v>6</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -742,7 +742,7 @@
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -756,7 +756,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +782,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -815,7 +815,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -848,7 +848,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -881,7 +881,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -914,7 +914,7 @@
         <v>48</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -940,7 +940,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -973,7 +973,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1006,7 +1006,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
cleared all temp files
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="48">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -155,49 +155,13 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_102_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Generate_BQR_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_011</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_success</t>
   </si>
   <si>
     <t xml:space="preserve">test_sample</t>
   </si>
   <si>
-    <t xml:space="preserve">test_common_100_102_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
+    <t xml:space="preserve">test_success_2</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -269,10 +233,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF067D17"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
+      <sz val="13.5"/>
+      <color rgb="FF00627A"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -400,7 +364,7 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF067D17"/>
+      <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
@@ -457,8 +421,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="15.90234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr defaultColWidth="15.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -778,8 +742,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+    <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="0" t="s">
@@ -792,51 +756,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D26" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D23" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -857,7 +779,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -890,7 +812,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -922,14 +844,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
-  </cols>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -945,69 +861,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D5" type="list">
-      <formula1>"True,False"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1024,7 +878,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1048,13 +902,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1083,7 +937,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1116,7 +970,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1149,7 +1003,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Before start of bqr scripting
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -422,7 +422,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="15.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.61328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -779,7 +779,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -812,7 +812,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -845,7 +845,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -878,7 +878,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -937,7 +937,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -970,7 +970,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1003,7 +1003,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Callback plus client side tcs
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="65">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -176,13 +176,43 @@
     <t xml:space="preserve">test_UI_MPOS_PM_UPI_Failure_HDFC_02</t>
   </si>
   <si>
-    <t xml:space="preserve">test_UI_MPOS_PM_UPI_Pending_HDFC_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_UI_MPOS_PM_UPI_Refund_HDFC_04</t>
+    <t xml:space="preserve">test_UI_MPOS_PM_UPI_Pending_HDFC_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_MPOS_PM_UPI_Refund_HDFC_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_MPOS_PM_UPI_Expire_HDFC_06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_Callback_Success_HDFC_07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/ezetap/EzeAuto/TestCases/Functional/UI/Common/test_UPI_Payment_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
   </si>
   <si>
     <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_Callback_Failed_HDFC_09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_RefundByAPI_HDFC_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_UPG_Authorized_HDFC_11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_UPG_Auth_Refunded_HDFC_12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_UPG_Failed_HDFC_13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_Callback_Success_AfterExpiry_HDFC_04</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -443,7 +473,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="15.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.47265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -799,8 +829,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -820,8 +850,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
         <v>45</v>
       </c>
       <c r="B2" s="0" t="s">
@@ -834,8 +864,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="0" t="s">
@@ -873,12 +903,46 @@
         <v>47</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
         <v>51</v>
       </c>
+      <c r="B6" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D5" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D10" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -899,7 +963,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -931,8 +995,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -948,7 +1016,111 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D8" type="list">
+      <formula1>"True,False"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -965,7 +1137,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -989,13 +1161,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1024,7 +1196,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1057,7 +1229,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1090,7 +1262,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
renaming the test case name to test_UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -185,7 +185,7 @@
     <t xml:space="preserve">test_UI_MPOS_PM_UPI_Expire_HDFC_06</t>
   </si>
   <si>
-    <t xml:space="preserve">test_UI_Common_PM_UPI_Callback_Success_HDFC_07</t>
+    <t xml:space="preserve">test_UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">/home/ezetap/EzeAuto/TestCases/Functional/UI/Common/test_UPI_Payment_01</t>
@@ -233,7 +233,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -286,6 +286,13 @@
     <font>
       <sz val="13.5"/>
       <color rgb="FF00627A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -346,7 +353,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -392,6 +399,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -473,7 +484,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="15.47265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -830,7 +841,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -963,7 +974,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -996,7 +1007,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1017,7 +1028,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="0" t="s">
@@ -1137,7 +1148,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1196,7 +1207,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1229,7 +1240,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1262,7 +1273,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
changes before logger and api
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="58">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -155,13 +155,43 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
   </si>
   <si>
-    <t xml:space="preserve">test_success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_success_2</t>
+    <t xml:space="preserve">test_sa_100_102_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Generate_BQR_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -233,10 +263,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="13.5"/>
-      <color rgb="FF00627A"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <color rgb="FF067D17"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -364,7 +394,7 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF067D17"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
@@ -421,8 +451,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="15.61328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L25"/>
+  <sheetFormatPr defaultColWidth="15.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -739,12 +769,12 @@
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>43</v>
@@ -753,12 +783,40 @@
         <v>6</v>
       </c>
       <c r="D23" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D23" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D25" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -779,7 +837,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -812,7 +870,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -844,8 +902,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -861,7 +925,69 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D5" type="list">
+      <formula1>"True,False"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -878,7 +1004,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -902,13 +1028,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -937,7 +1063,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -970,7 +1096,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1003,7 +1129,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Integration of execution logger and api parametrization
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="69">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -158,12 +158,15 @@
     <t xml:space="preserve">test_success</t>
   </si>
   <si>
+    <t xml:space="preserve">/home/ezetap/EzeAuto/TestCases/test_sample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_success_2</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sample</t>
   </si>
   <si>
-    <t xml:space="preserve">test_success_2</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_sa_100_101_001</t>
   </si>
   <si>
@@ -173,6 +176,9 @@
     <t xml:space="preserve">UI/MPOS</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_101_002</t>
   </si>
   <si>
@@ -191,9 +197,6 @@
     <t xml:space="preserve">test_sa_100_101_003</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_com_100_101_005</t>
   </si>
   <si>
@@ -216,6 +219,12 @@
   </si>
   <si>
     <t xml:space="preserve">test_com_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_SubFeatureCode_CNP_TXN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/ezetap/EzeAuto/TestCases/Functional/UI/Common/test_cnp_testCase</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -236,7 +245,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -300,6 +309,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF9B703F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -356,7 +372,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -406,6 +422,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -431,7 +451,7 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF9B703F"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF00627A"/>
       <rgbColor rgb="FFB4C7DC"/>
@@ -487,12 +507,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="15.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -812,7 +831,7 @@
         <v>44</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>6</v>
@@ -844,7 +863,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -866,27 +885,27 @@
     </row>
     <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -894,13 +913,13 @@
     </row>
     <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -908,13 +927,13 @@
     </row>
     <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -922,13 +941,13 @@
     </row>
     <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>7</v>
@@ -936,13 +955,13 @@
     </row>
     <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>7</v>
@@ -950,16 +969,16 @@
     </row>
     <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>54</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -995,7 +1014,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1027,8 +1046,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1050,13 +1069,13 @@
     </row>
     <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1064,13 +1083,13 @@
     </row>
     <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -1078,13 +1097,13 @@
     </row>
     <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1092,13 +1111,13 @@
     </row>
     <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -1106,13 +1125,13 @@
     </row>
     <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>7</v>
@@ -1120,21 +1139,35 @@
     </row>
     <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D7" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D8" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1155,7 +1188,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1179,13 +1212,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1214,7 +1247,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1247,7 +1280,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1280,7 +1313,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Commit after refund test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="66">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -161,12 +161,12 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_sa_100_102_008</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_009</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_102_010</t>
   </si>
   <si>
@@ -176,22 +176,46 @@
     <t xml:space="preserve">test_sa_100_102_011</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_102_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
+    <t xml:space="preserve">test_common_100_102_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_006</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -451,13 +475,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
-  <sheetFormatPr defaultColWidth="15.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr defaultColWidth="16.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -769,12 +792,12 @@
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>43</v>
@@ -783,15 +806,15 @@
         <v>6</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>6</v>
@@ -802,7 +825,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>47</v>
@@ -814,9 +837,65 @@
         <v>7</v>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D25" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D29" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -837,7 +916,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -870,7 +949,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -902,8 +981,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -926,14 +1005,14 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>49</v>
+      <c r="A2" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -941,49 +1020,77 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>52</v>
+      <c r="A4" s="11" t="s">
+        <v>59</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>54</v>
+      <c r="A5" s="10" t="s">
+        <v>60</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D5" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D7" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1004,7 +1111,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1028,13 +1135,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1063,7 +1170,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1096,7 +1203,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1129,7 +1236,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
updated the TC Skeleton part
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -173,34 +173,34 @@
     <t xml:space="preserve">Functional/UI/SA/test_UPI_Payment</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_008</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_008</t>
   </si>
   <si>
     <t xml:space="preserve">test_com_100_101_004</t>
@@ -509,7 +509,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="16.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -853,12 +853,12 @@
         <v>6</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>47</v>
@@ -872,7 +872,7 @@
     </row>
     <row r="26" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B26" s="0" t="s">
         <v>47</v>
@@ -885,12 +885,8 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D23" type="list">
-      <formula1>"True,False"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D24:D26" type="list">
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D26" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -911,7 +907,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -979,7 +975,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1012,7 +1008,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1034,13 +1030,13 @@
     </row>
     <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1048,13 +1044,13 @@
     </row>
     <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -1062,13 +1058,13 @@
     </row>
     <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1076,13 +1072,13 @@
     </row>
     <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -1090,16 +1086,16 @@
     </row>
     <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1107,10 +1103,10 @@
         <v>58</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>7</v>
@@ -1124,7 +1120,7 @@
         <v>60</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>7</v>
@@ -1135,10 +1131,10 @@
         <v>61</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>7</v>
@@ -1149,10 +1145,10 @@
         <v>62</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>7</v>
@@ -1181,7 +1177,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1240,7 +1236,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1273,7 +1269,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1306,7 +1302,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
UPI Refund/Pending test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="71">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -179,43 +179,58 @@
     <t xml:space="preserve">test_sa_100_101_003</t>
   </si>
   <si>
+    <t xml:space="preserve">test_com_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_com_100_101_005</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_com_100_101_006</t>
   </si>
   <si>
     <t xml:space="preserve">test_com_100_101_007</t>
   </si>
   <si>
+    <t xml:space="preserve">test_com_100_101_008</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_com_100_101_009</t>
   </si>
   <si>
-    <t xml:space="preserve">test_com_100_101_008</t>
+    <t xml:space="preserve">test_com_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Refund_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">True</t>
   </si>
   <si>
-    <t xml:space="preserve">test_com_100_101_004</t>
+    <t xml:space="preserve">test_com_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Pending_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_SubFeatureCode_CNP_TXN</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_cnp_testCase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_011</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -236,7 +251,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -307,13 +322,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="13.5"/>
-      <color rgb="FFFFC66D"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -370,7 +378,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -424,10 +432,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -481,7 +485,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFC66D"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -509,7 +513,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -907,7 +911,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -975,7 +979,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1007,8 +1011,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1029,7 +1033,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>50</v>
       </c>
       <c r="B2" s="0" t="s">
@@ -1043,7 +1047,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="0" t="s">
@@ -1057,7 +1061,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>54</v>
       </c>
       <c r="B4" s="0" t="s">
@@ -1071,7 +1075,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>55</v>
       </c>
       <c r="B5" s="0" t="s">
@@ -1085,7 +1089,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>56</v>
       </c>
       <c r="B6" s="0" t="s">
@@ -1095,12 +1099,12 @@
         <v>52</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>58</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>51</v>
@@ -1113,25 +1117,25 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>59</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>60</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>7</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="11" t="s">
         <v>61</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>52</v>
@@ -1145,7 +1149,7 @@
         <v>62</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>52</v>
@@ -1154,9 +1158,51 @@
         <v>7</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D10" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D13" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1177,12 +1223,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="69.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1201,13 +1246,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1236,7 +1281,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1269,7 +1314,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1302,7 +1347,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
TC Skeleton updated with chageslip validation
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="70">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -207,9 +207,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_com_100_101_011</t>
@@ -513,7 +510,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="17.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.08203125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -911,7 +908,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -979,7 +976,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1012,7 +1009,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1127,12 +1124,12 @@
         <v>52</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>60</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>59</v>
@@ -1146,7 +1143,7 @@
     </row>
     <row r="10" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>59</v>
@@ -1160,7 +1157,7 @@
     </row>
     <row r="11" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>59</v>
@@ -1174,10 +1171,10 @@
     </row>
     <row r="12" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>64</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>65</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>52</v>
@@ -1188,10 +1185,10 @@
     </row>
     <row r="13" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>66</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>67</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>52</v>
@@ -1223,7 +1220,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1246,13 +1243,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>69</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>70</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1281,7 +1278,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1314,7 +1311,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1347,7 +1344,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Commit before Chargeslip validation
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="72">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -170,12 +170,45 @@
     <t xml:space="preserve">test_sa_100_102_010</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Generate_BQR_HDFC</t>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_sa_100_102_011</t>
   </si>
   <si>
+    <t xml:space="preserve">test_success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_006</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_102_019</t>
   </si>
   <si>
@@ -185,37 +218,22 @@
     <t xml:space="preserve">test_sa_100_102_020</t>
   </si>
   <si>
-    <t xml:space="preserve">test_success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_006</t>
+    <t xml:space="preserve">test_sa_100_102_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -475,8 +493,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
-  <sheetFormatPr defaultColWidth="16.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr defaultColWidth="16.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -865,37 +883,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B29" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D29" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D27" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -916,7 +906,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -949,7 +939,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -981,8 +971,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1006,13 +996,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1020,27 +1010,27 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>59</v>
+      <c r="A4" s="10" t="s">
+        <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1048,27 +1038,27 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>61</v>
+      <c r="A6" s="11" t="s">
+        <v>58</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>7</v>
@@ -1076,21 +1066,95 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>7</v>
+      <c r="B9" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D7" type="list">
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D11" type="list">
+      <formula1>"True,False"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D12" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1111,7 +1175,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1135,13 +1199,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1170,7 +1234,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1203,7 +1267,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1236,7 +1300,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
configurations added to config.ini
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -191,6 +191,9 @@
     <t xml:space="preserve">UI/Common</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_102_002</t>
   </si>
   <si>
@@ -231,9 +234,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -494,7 +494,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L27"/>
-  <sheetFormatPr defaultColWidth="16.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -906,7 +906,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -939,7 +939,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -972,7 +972,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1005,12 +1005,12 @@
         <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>52</v>
@@ -1024,7 +1024,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>52</v>
@@ -1038,10 +1038,10 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>53</v>
@@ -1052,10 +1052,10 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>53</v>
@@ -1066,10 +1066,10 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>53</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>53</v>
@@ -1094,10 +1094,10 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="0" t="s">
         <v>62</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>61</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>53</v>
@@ -1108,10 +1108,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>53</v>
@@ -1122,10 +1122,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="0" t="s">
         <v>65</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>64</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>53</v>
@@ -1136,16 +1136,16 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1175,7 +1175,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1234,7 +1234,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1267,7 +1267,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1300,7 +1300,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
added cnpware test cases and integrated chargeslip validation
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="74">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -273,6 +273,9 @@
       </rPr>
       <t xml:space="preserve">test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -551,7 +554,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="17.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -949,7 +952,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1017,7 +1020,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1050,7 +1053,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1252,7 +1255,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
         <v>68</v>
       </c>
@@ -1263,7 +1266,7 @@
         <v>52</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>7</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1289,7 +1292,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1312,13 +1315,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1347,7 +1350,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1380,7 +1383,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1413,7 +1416,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Integration of chargeslip validation
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="71">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -155,85 +155,82 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_Upfront_Mobile_Number</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_102_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_011</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_success</t>
   </si>
   <si>
+    <t xml:space="preserve">/home/ezetap/EzeAuto/TestCases/test_sample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_success_2</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sample</t>
   </si>
   <si>
-    <t xml:space="preserve">test_common_100_102_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+    <t xml:space="preserve">test_sa_100_101_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_Common_PM_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
   </si>
   <si>
     <t xml:space="preserve">UI/Common</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
+    <t xml:space="preserve">test_com_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_SubFeatureCode_CNP_TXN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_cnp_testCase</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -254,7 +251,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -305,10 +302,24 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF067D17"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
+      <sz val="13.5"/>
+      <color rgb="FF00627A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF9B703F"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -367,7 +378,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -413,6 +424,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -436,9 +455,9 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF067D17"/>
+      <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF9B703F"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF00627A"/>
       <rgbColor rgb="FFB4C7DC"/>
@@ -493,8 +512,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
-  <sheetFormatPr defaultColWidth="16.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L26"/>
+  <sheetFormatPr defaultColWidth="17.3359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -813,12 +832,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+    <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>6</v>
@@ -827,23 +846,23 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>45</v>
+    <row r="24" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>47</v>
@@ -852,12 +871,12 @@
         <v>6</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="s">
+        <v>50</v>
       </c>
       <c r="B26" s="0" t="s">
         <v>47</v>
@@ -869,23 +888,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D27" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D26" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -905,8 +910,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -922,7 +931,38 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D5:D7 D9:D10" type="list">
+      <formula1>"True,False"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -939,7 +979,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -971,13 +1011,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -994,25 +1032,25 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+    <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -1022,26 +1060,26 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="4" t="s">
+    <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>58</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>52</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>53</v>
@@ -1050,12 +1088,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>52</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>53</v>
@@ -1064,12 +1102,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="4" t="s">
+    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>58</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>52</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>53</v>
@@ -1078,12 +1116,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>61</v>
+    <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>59</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>53</v>
@@ -1092,12 +1130,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>63</v>
+    <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>61</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>53</v>
@@ -1106,12 +1144,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>64</v>
+    <row r="10" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>53</v>
@@ -1120,12 +1158,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>66</v>
+    <row r="11" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>63</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>53</v>
@@ -1134,27 +1172,37 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>67</v>
+    <row r="12" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>64</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>54</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D11" type="list">
-      <formula1>"True,False"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D12" type="list">
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D13" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1175,12 +1223,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="69.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1199,13 +1246,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>70</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>71</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1234,7 +1281,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1267,7 +1314,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1300,7 +1347,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Excel updated with cnp test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="73">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -273,9 +273,6 @@
       </rPr>
       <t xml:space="preserve">test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -554,7 +551,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="17.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -952,7 +949,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1020,7 +1017,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1053,7 +1050,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1255,7 +1252,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
         <v>68</v>
       </c>
@@ -1266,7 +1263,7 @@
         <v>52</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1292,7 +1289,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1315,13 +1312,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>73</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1350,7 +1347,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1383,7 +1380,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1416,7 +1413,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Added chargeslip marker and integrated with 13 test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="97">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">test_sa_100_101_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_Common_PM_UPI_HDFC_CheckStatus_01</t>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
   </si>
   <si>
     <t xml:space="preserve">True</t>
@@ -182,6 +182,27 @@
     <t xml:space="preserve">test_sa_100_101_003</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_011</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_com_100_101_004</t>
   </si>
   <si>
@@ -227,10 +248,67 @@
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Pending_HDFC</t>
   </si>
   <si>
-    <t xml:space="preserve">test_SubFeatureCode_CNP_TXN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_cnp_testCase</t>
+    <t xml:space="preserve">test_common_100_102_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -251,7 +329,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="16">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -274,6 +352,47 @@
       <family val="0"/>
     </font>
     <font>
+      <sz val="13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF00627A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF080808"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF00627A"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
@@ -281,7 +400,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="13.5"/>
       <color rgb="FF00627A"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -295,20 +414,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF00627A"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="13.5"/>
-      <color rgb="FF00627A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="13.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -316,10 +421,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="13.5"/>
-      <color rgb="FF9B703F"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <sz val="13"/>
+      <color rgb="FF067D17"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00627A"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -378,24 +490,72 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -403,35 +563,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -455,9 +603,9 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF067D17"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF9B703F"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF00627A"/>
       <rgbColor rgb="FFB4C7DC"/>
@@ -512,385 +660,456 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="17.3359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr defaultColWidth="17.40625" defaultRowHeight="16.15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="57.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="87.38"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="17.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.52"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="1" width="17.39"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="6"/>
+      <c r="C3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="H3" s="7"/>
       <c r="J3" s="7"/>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="C5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="C13" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="5" t="s">
+      <c r="C16" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>7</v>
       </c>
       <c r="L16" s="9"/>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
         <v>36</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C17" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
         <v>37</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
         <v>39</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C23" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="5" t="s">
+      <c r="C24" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="5" t="s">
+      <c r="C25" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="5" t="s">
+      <c r="C26" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D26" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D31" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -911,50 +1130,50 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
+      <c r="A5" s="15"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
+      <c r="A6" s="15"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
+      <c r="A7" s="18"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="17"/>
     </row>
     <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
+      <c r="A9" s="15"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="17"/>
     </row>
     <row r="10" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
+      <c r="A10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -979,19 +1198,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1011,198 +1230,381 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr defaultColWidth="14.76953125" defaultRowHeight="16.15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="91.15"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="3" style="1" width="14.75"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="5" t="s">
+    <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D13" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D26" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1223,7 +1625,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1231,30 +1633,30 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="A2" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1281,19 +1683,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1314,19 +1716,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1347,19 +1749,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
tcs updated to accomodate the parallel execution for 13 tcs
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -173,133 +173,133 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_com_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_com_100_101_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_002</t>
@@ -1006,12 +1006,12 @@
         <v>6</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>47</v>
@@ -1020,12 +1020,12 @@
         <v>6</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>47</v>
@@ -1039,24 +1039,24 @@
     </row>
     <row r="27" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="C27" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>6</v>
@@ -1067,24 +1067,24 @@
     </row>
     <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>6</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="31" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>6</v>
@@ -1130,7 +1130,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1198,7 +1198,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
@@ -1254,13 +1254,13 @@
     </row>
     <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C2" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>7</v>
@@ -1268,27 +1268,27 @@
     </row>
     <row r="3" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>7</v>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>7</v>
@@ -1310,13 +1310,13 @@
     </row>
     <row r="6" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>7</v>
@@ -1324,13 +1324,13 @@
     </row>
     <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>7</v>
@@ -1338,13 +1338,13 @@
     </row>
     <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>7</v>
@@ -1352,13 +1352,13 @@
     </row>
     <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>7</v>
@@ -1366,13 +1366,13 @@
     </row>
     <row r="10" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>7</v>
@@ -1380,41 +1380,41 @@
     </row>
     <row r="11" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="C13" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>7</v>
@@ -1422,13 +1422,13 @@
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>7</v>
@@ -1436,27 +1436,27 @@
     </row>
     <row r="15" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>78</v>
-      </c>
       <c r="C16" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>7</v>
@@ -1464,13 +1464,13 @@
     </row>
     <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>7</v>
@@ -1478,27 +1478,27 @@
     </row>
     <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="C19" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>7</v>
@@ -1506,13 +1506,13 @@
     </row>
     <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>7</v>
@@ -1520,13 +1520,13 @@
     </row>
     <row r="21" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="C21" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>7</v>
@@ -1534,13 +1534,13 @@
     </row>
     <row r="22" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>7</v>
@@ -1548,30 +1548,30 @@
     </row>
     <row r="23" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="C23" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="C24" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1579,13 +1579,13 @@
         <v>91</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1596,10 +1596,10 @@
         <v>93</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1625,7 +1625,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1683,7 +1683,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
@@ -1716,7 +1716,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
@@ -1749,7 +1749,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">

</xml_diff>

<commit_message>
made little changes in the test case side to over come app sync
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="96">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -297,9 +297,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_002</t>
@@ -1130,7 +1127,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1198,7 +1195,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
@@ -1571,12 +1568,12 @@
         <v>59</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>90</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B25" s="20" t="s">
         <v>89</v>
@@ -1585,21 +1582,21 @@
         <v>59</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>90</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B26" s="20" t="s">
-        <v>93</v>
-      </c>
       <c r="C26" s="5" t="s">
         <v>59</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>90</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1625,7 +1622,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1648,13 +1645,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="C2" s="22" t="s">
         <v>95</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>96</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>7</v>
@@ -1683,7 +1680,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
@@ -1716,7 +1713,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
@@ -1749,7 +1746,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">

</xml_diff>

<commit_message>
Add test cases for debit card cnp txn and fix for sycn issue.
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -299,43 +299,43 @@
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
   </si>
   <si>
+    <t xml:space="preserve">test_common_100_103_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_010</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_010</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_011</t>
@@ -359,7 +359,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -471,6 +471,17 @@
       <family val="3"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00627A"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -527,7 +538,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -625,6 +636,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1213,7 +1232,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1281,7 +1300,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1676,13 +1695,13 @@
         <v>59</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="E24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>89</v>
@@ -1697,10 +1716,10 @@
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="21" t="s">
         <v>92</v>
-      </c>
-      <c r="B26" s="21" t="s">
-        <v>93</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>59</v>
@@ -1712,10 +1731,10 @@
     </row>
     <row r="27" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>94</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>95</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>59</v>
@@ -1727,10 +1746,10 @@
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>59</v>
@@ -1742,10 +1761,10 @@
     </row>
     <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>59</v>
@@ -1756,10 +1775,10 @@
     </row>
     <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B30" s="21" t="s">
         <v>98</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>99</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>59</v>
@@ -1770,10 +1789,10 @@
     </row>
     <row r="31" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>59</v>
@@ -1784,7 +1803,7 @@
     </row>
     <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B32" s="21" t="s">
         <v>89</v>
@@ -1798,7 +1817,7 @@
     </row>
     <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="21" t="s">
         <v>89</v>
@@ -1807,15 +1826,15 @@
         <v>59</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23" t="s">
+      <c r="A34" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>99</v>
+      <c r="B34" s="26" t="s">
+        <v>98</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>59</v>
@@ -1847,7 +1866,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1869,13 +1888,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="28" t="s">
         <v>106</v>
       </c>
       <c r="D2" s="18" t="s">
@@ -1905,7 +1924,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1938,7 +1957,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1971,7 +1990,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">

</xml_diff>

<commit_message>
added some test cases to excel an added one api details to DB.
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -299,6 +299,9 @@
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_103_002</t>
   </si>
   <si>
@@ -333,9 +336,6 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_011</t>
@@ -359,7 +359,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -471,17 +471,6 @@
       <family val="3"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF00627A"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -538,7 +527,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -636,14 +625,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1232,7 +1213,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1300,7 +1281,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1695,13 +1676,13 @@
         <v>59</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="E24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>89</v>
@@ -1716,10 +1697,10 @@
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>59</v>
@@ -1731,10 +1712,10 @@
     </row>
     <row r="27" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>59</v>
@@ -1746,10 +1727,10 @@
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" s="21" t="s">
         <v>95</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>94</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>59</v>
@@ -1761,10 +1742,10 @@
     </row>
     <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>59</v>
@@ -1775,10 +1756,10 @@
     </row>
     <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>59</v>
@@ -1789,10 +1770,10 @@
     </row>
     <row r="31" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>99</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>98</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>59</v>
@@ -1803,7 +1784,7 @@
     </row>
     <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B32" s="21" t="s">
         <v>89</v>
@@ -1817,7 +1798,7 @@
     </row>
     <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B33" s="21" t="s">
         <v>89</v>
@@ -1826,15 +1807,15 @@
         <v>59</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="s">
+      <c r="A34" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="B34" s="26" t="s">
-        <v>98</v>
+      <c r="B34" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>59</v>
@@ -1866,7 +1847,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1888,13 +1869,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="26" t="s">
         <v>106</v>
       </c>
       <c r="D2" s="18" t="s">
@@ -1924,7 +1905,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1957,7 +1938,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1990,7 +1971,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">

</xml_diff>

<commit_message>
after hdfc push correction
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -182,6 +182,9 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_YES_ATOS</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_102_029</t>
   </si>
   <si>
@@ -210,9 +213,6 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_100_102_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_102_006</t>
@@ -534,7 +534,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L29"/>
-  <sheetFormatPr defaultColWidth="16.94921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -920,12 +920,12 @@
         <v>6</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="0" t="s">
         <v>50</v>
@@ -939,7 +939,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B29" s="0" t="s">
         <v>50</v>
@@ -974,7 +974,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1007,7 +1007,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1040,7 +1040,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1064,27 +1064,27 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -1092,13 +1092,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1106,13 +1106,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -1120,16 +1120,16 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>59</v>
-      </c>
       <c r="C6" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1137,13 +1137,13 @@
         <v>62</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1151,10 +1151,10 @@
         <v>63</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>7</v>
@@ -1165,10 +1165,10 @@
         <v>64</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>7</v>
@@ -1179,10 +1179,10 @@
         <v>65</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>7</v>
@@ -1196,7 +1196,7 @@
         <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>7</v>
@@ -1210,7 +1210,7 @@
         <v>67</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>7</v>
@@ -1224,7 +1224,7 @@
         <v>70</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>7</v>
@@ -1238,7 +1238,7 @@
         <v>70</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>7</v>
@@ -1252,7 +1252,7 @@
         <v>73</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>7</v>
@@ -1266,7 +1266,7 @@
         <v>75</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>7</v>
@@ -1280,7 +1280,7 @@
         <v>75</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>7</v>
@@ -1294,7 +1294,7 @@
         <v>75</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>7</v>
@@ -1308,10 +1308,10 @@
         <v>79</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1322,7 +1322,7 @@
         <v>79</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>7</v>
@@ -1336,10 +1336,10 @@
         <v>79</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1350,7 +1350,7 @@
         <v>83</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>7</v>
@@ -1364,7 +1364,7 @@
         <v>83</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>7</v>
@@ -1378,7 +1378,7 @@
         <v>83</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>7</v>
@@ -1407,7 +1407,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1465,7 +1465,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1498,7 +1498,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1531,7 +1531,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
api parametrization of curl data and manage orgsetting, updated api validation with the new api txnDetails, resource assigner integrated with all 14 upi test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="107">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -194,6 +194,9 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_101_002</t>
   </si>
   <si>
@@ -299,13 +302,13 @@
     <t xml:space="preserve">test_common_100_101_014</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Pending_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_010</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_UPI_Refund_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_011</t>
@@ -314,24 +317,18 @@
     <t xml:space="preserve">test_common_100_101_012</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_common_100_101_013</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_004</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UPI_Payment_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_005</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_common_100_101_006</t>
   </si>
   <si>
@@ -342,27 +339,6 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_020</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -383,7 +359,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -414,35 +390,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFFC66D"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFFC66D"/>
+      <color rgb="FF00627A"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -459,6 +407,13 @@
       <color rgb="FF00627A"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFFC66D"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -517,7 +472,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -534,7 +489,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -546,19 +505,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -567,22 +518,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -663,8 +598,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
-  <sheetFormatPr defaultColWidth="17.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L32"/>
+  <sheetFormatPr defaultColWidth="17.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -689,13 +624,13 @@
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -703,44 +638,44 @@
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="J3" s="6"/>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="H3" s="7"/>
+      <c r="J3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -748,111 +683,111 @@
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="C13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -860,224 +795,224 @@
       <c r="A14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="L16" s="8"/>
+      <c r="C16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="C19" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="C20" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="C21" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="C24" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="C28" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1085,57 +1020,47 @@
       <c r="A30" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>7</v>
+      <c r="C30" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B32" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="4"/>
+      <c r="C32" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>55</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D34" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D32" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1156,7 +1081,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1189,7 +1114,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1221,8 +1146,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D35"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="81.47"/>
@@ -1246,568 +1171,484 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B2" s="14" t="s">
+      <c r="A2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="B2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="14" t="s">
+      <c r="A3" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="C3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" s="14" t="s">
+      <c r="A4" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="C4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="14" t="s">
+      <c r="A5" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="B5" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="14" t="s">
+      <c r="C8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="C9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" s="15" t="s">
+      <c r="C10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>69</v>
+      <c r="A11" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B13" s="10" t="s">
+      <c r="A13" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="B13" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="A15" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="B16" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="A18" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="A19" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="B19" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="C20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="A21" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="A22" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="B22" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="B23" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="A24" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="B25" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>7</v>
+      <c r="B25" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B26" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>7</v>
+      <c r="B26" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>7</v>
+      <c r="C27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="B28" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>7</v>
+      <c r="B28" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>7</v>
+      <c r="B29" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>7</v>
+      <c r="C30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="B31" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>7</v>
+      <c r="B31" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="B32" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>7</v>
+      <c r="C32" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>7</v>
+        <v>101</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>7</v>
+        <v>102</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B35" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>7</v>
+      <c r="C35" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D41" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D35" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1828,7 +1669,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1850,16 +1691,16 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D2" s="15" t="s">
+      <c r="A2" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1886,7 +1727,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1919,7 +1760,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1952,7 +1793,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
renamed one method wait_for_navigation_to_load
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="112">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -302,13 +302,13 @@
     <t xml:space="preserve">test_common_100_101_014</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_PM_Common_UPI_Pending_HDFC</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_010</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_PM_Common_UPI_Refund_HDFC</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_011</t>
@@ -317,19 +317,22 @@
     <t xml:space="preserve">test_common_100_101_012</t>
   </si>
   <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_101_013</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_004</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_PM_Common_UPI_Callback_HDFC_01</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_005</t>
   </si>
   <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_PM_Common_UPI_Checkstatus_HDFC_01</t>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_006</t>
@@ -630,7 +633,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L32"/>
-  <sheetFormatPr defaultColWidth="17.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.5625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1112,7 +1115,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1145,7 +1148,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1178,7 +1181,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D38"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="81.47"/>
@@ -1570,7 +1573,7 @@
         <v>95</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>60</v>
@@ -1581,10 +1584,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>93</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>60</v>
@@ -1595,10 +1598,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>60</v>
@@ -1609,10 +1612,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>60</v>
@@ -1623,10 +1626,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>60</v>
@@ -1637,10 +1640,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>60</v>
@@ -1651,10 +1654,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>60</v>
@@ -1665,10 +1668,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>60</v>
@@ -1679,10 +1682,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>60</v>
@@ -1693,10 +1696,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>60</v>
@@ -1707,10 +1710,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>60</v>
@@ -1742,7 +1745,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1765,13 +1768,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>7</v>
@@ -1800,7 +1803,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1833,7 +1836,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1866,7 +1869,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
resource assiner implemented and yes bank cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="96">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -182,18 +182,6 @@
     <t xml:space="preserve">test_sa_100_102_027</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_003</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_common_100_102_001</t>
   </si>
   <si>
@@ -314,109 +302,10 @@
     <t xml:space="preserve">test_common_100_102_034</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_102_035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_011</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -437,7 +326,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -485,20 +374,6 @@
       <color rgb="FF00627A"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -557,7 +432,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -600,26 +475,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -699,8 +554,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="17.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr defaultColWidth="17.1015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1089,55 +944,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D29" type="list">
-      <formula1>"True,False"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D30" type="list">
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D27" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1158,7 +967,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1191,7 +1000,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1223,8 +1032,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z55"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1248,13 +1057,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1262,13 +1071,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -1276,13 +1085,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1290,13 +1099,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -1304,13 +1113,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>7</v>
@@ -1318,13 +1127,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>7</v>
@@ -1332,13 +1141,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>7</v>
@@ -1346,13 +1155,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>7</v>
@@ -1360,13 +1169,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>7</v>
@@ -1374,13 +1183,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>7</v>
@@ -1388,13 +1197,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>7</v>
@@ -1402,13 +1211,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>7</v>
@@ -1416,13 +1225,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>7</v>
@@ -1430,13 +1239,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>7</v>
@@ -1444,13 +1253,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>7</v>
@@ -1458,13 +1267,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>7</v>
@@ -1472,13 +1281,13 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>7</v>
@@ -1486,13 +1295,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>7</v>
@@ -1500,13 +1309,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>7</v>
@@ -1514,13 +1323,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>7</v>
@@ -1528,13 +1337,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>7</v>
@@ -1542,13 +1351,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>7</v>
@@ -1556,13 +1365,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>7</v>
@@ -1570,13 +1379,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>7</v>
@@ -1584,13 +1393,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>7</v>
@@ -1598,13 +1407,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>7</v>
@@ -1612,13 +1421,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>7</v>
@@ -1626,561 +1435,35 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C41" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="B45" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="C45" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="B46" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="C46" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="B47" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="6"/>
-      <c r="N48" s="6"/>
-      <c r="O48" s="6"/>
-      <c r="P48" s="6"/>
-      <c r="Q48" s="6"/>
-      <c r="R48" s="6"/>
-      <c r="S48" s="6"/>
-      <c r="T48" s="6"/>
-      <c r="U48" s="6"/>
-      <c r="V48" s="6"/>
-      <c r="W48" s="6"/>
-      <c r="X48" s="6"/>
-      <c r="Y48" s="6"/>
-      <c r="Z48" s="6"/>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
-      <c r="L49" s="6"/>
-      <c r="M49" s="6"/>
-      <c r="N49" s="6"/>
-      <c r="O49" s="6"/>
-      <c r="P49" s="6"/>
-      <c r="Q49" s="6"/>
-      <c r="R49" s="6"/>
-      <c r="S49" s="6"/>
-      <c r="T49" s="6"/>
-      <c r="U49" s="6"/>
-      <c r="V49" s="6"/>
-      <c r="W49" s="6"/>
-      <c r="X49" s="6"/>
-      <c r="Y49" s="6"/>
-      <c r="Z49" s="6"/>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="C50" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="6"/>
-      <c r="N50" s="6"/>
-      <c r="O50" s="6"/>
-      <c r="P50" s="6"/>
-      <c r="Q50" s="6"/>
-      <c r="R50" s="6"/>
-      <c r="S50" s="6"/>
-      <c r="T50" s="6"/>
-      <c r="U50" s="6"/>
-      <c r="V50" s="6"/>
-      <c r="W50" s="6"/>
-      <c r="X50" s="6"/>
-      <c r="Y50" s="6"/>
-      <c r="Z50" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
-      <c r="I51" s="6"/>
-      <c r="J51" s="6"/>
-      <c r="K51" s="6"/>
-      <c r="L51" s="6"/>
-      <c r="M51" s="6"/>
-      <c r="N51" s="6"/>
-      <c r="O51" s="6"/>
-      <c r="P51" s="6"/>
-      <c r="Q51" s="6"/>
-      <c r="R51" s="6"/>
-      <c r="S51" s="6"/>
-      <c r="T51" s="6"/>
-      <c r="U51" s="6"/>
-      <c r="V51" s="6"/>
-      <c r="W51" s="6"/>
-      <c r="X51" s="6"/>
-      <c r="Y51" s="6"/>
-      <c r="Z51" s="6"/>
-    </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="B52" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="C52" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="6"/>
-      <c r="N52" s="6"/>
-      <c r="O52" s="6"/>
-      <c r="P52" s="6"/>
-      <c r="Q52" s="6"/>
-      <c r="R52" s="6"/>
-      <c r="S52" s="6"/>
-      <c r="T52" s="6"/>
-      <c r="U52" s="6"/>
-      <c r="V52" s="6"/>
-      <c r="W52" s="6"/>
-      <c r="X52" s="6"/>
-      <c r="Y52" s="6"/>
-      <c r="Z52" s="6"/>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6"/>
-      <c r="I53" s="6"/>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="6"/>
-      <c r="N53" s="6"/>
-      <c r="O53" s="6"/>
-      <c r="P53" s="6"/>
-      <c r="Q53" s="6"/>
-      <c r="R53" s="6"/>
-      <c r="S53" s="6"/>
-      <c r="T53" s="6"/>
-      <c r="U53" s="6"/>
-      <c r="V53" s="6"/>
-      <c r="W53" s="6"/>
-      <c r="X53" s="6"/>
-      <c r="Y53" s="6"/>
-      <c r="Z53" s="6"/>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="B54" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="C54" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="6"/>
-      <c r="N54" s="6"/>
-      <c r="O54" s="6"/>
-      <c r="P54" s="6"/>
-      <c r="Q54" s="6"/>
-      <c r="R54" s="6"/>
-      <c r="S54" s="6"/>
-      <c r="T54" s="6"/>
-      <c r="U54" s="6"/>
-      <c r="V54" s="6"/>
-      <c r="W54" s="6"/>
-      <c r="X54" s="6"/>
-      <c r="Y54" s="6"/>
-      <c r="Z54" s="6"/>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="B55" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="C55" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="6"/>
-      <c r="K55" s="6"/>
-      <c r="L55" s="6"/>
-      <c r="M55" s="6"/>
-      <c r="N55" s="6"/>
-      <c r="O55" s="6"/>
-      <c r="P55" s="6"/>
-      <c r="Q55" s="6"/>
-      <c r="R55" s="6"/>
-      <c r="S55" s="6"/>
-      <c r="T55" s="6"/>
-      <c r="U55" s="6"/>
-      <c r="V55" s="6"/>
-      <c r="W55" s="6"/>
-      <c r="X55" s="6"/>
-      <c r="Y55" s="6"/>
-      <c r="Z55" s="6"/>
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D55" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D30" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2201,7 +1484,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2224,13 +1507,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>130</v>
+        <v>93</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>131</v>
+        <v>94</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>132</v>
+        <v>95</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -2259,7 +1542,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2292,7 +1575,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2325,7 +1608,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
changes before jenkins run
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="134">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -182,6 +182,18 @@
     <t xml:space="preserve">test_sa_100_102_027</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_101_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_102_001</t>
   </si>
   <si>
@@ -254,6 +266,9 @@
     <t xml:space="preserve">test_common_100_102_021</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_102_022</t>
   </si>
   <si>
@@ -302,10 +317,109 @@
     <t xml:space="preserve">test_common_100_102_034</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_common_100_102_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_011</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -326,7 +440,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -374,6 +488,20 @@
       <color rgb="FF00627A"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -432,7 +560,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -475,6 +603,22 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -554,8 +698,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
-  <sheetFormatPr defaultColWidth="17.1015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L30"/>
+  <sheetFormatPr defaultColWidth="17.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -944,9 +1088,51 @@
         <v>7</v>
       </c>
     </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D27" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D30" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -967,7 +1153,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1000,7 +1186,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1032,8 +1218,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Z55"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1057,13 +1243,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1071,13 +1257,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -1085,13 +1271,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1099,13 +1285,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -1113,13 +1299,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>7</v>
@@ -1127,13 +1313,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>7</v>
@@ -1141,13 +1327,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>7</v>
@@ -1155,13 +1341,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>7</v>
@@ -1169,13 +1355,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>7</v>
@@ -1183,13 +1369,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>7</v>
@@ -1197,13 +1383,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>7</v>
@@ -1211,13 +1397,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>7</v>
@@ -1225,13 +1411,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>7</v>
@@ -1239,13 +1425,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>7</v>
@@ -1253,13 +1439,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>7</v>
@@ -1267,13 +1453,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>7</v>
@@ -1281,27 +1467,27 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>7</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>7</v>
@@ -1309,13 +1495,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>7</v>
@@ -1323,13 +1509,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>7</v>
@@ -1337,13 +1523,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>7</v>
@@ -1351,13 +1537,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="B23" s="0" t="s">
-        <v>76</v>
-      </c>
       <c r="C23" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>7</v>
@@ -1365,13 +1551,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>7</v>
@@ -1379,13 +1565,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>7</v>
@@ -1393,13 +1579,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>7</v>
@@ -1407,13 +1593,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>7</v>
@@ -1421,13 +1607,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>7</v>
@@ -1435,35 +1621,561 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>91</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>91</v>
-      </c>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6"/>
+      <c r="K48" s="6"/>
+      <c r="L48" s="6"/>
+      <c r="M48" s="6"/>
+      <c r="N48" s="6"/>
+      <c r="O48" s="6"/>
+      <c r="P48" s="6"/>
+      <c r="Q48" s="6"/>
+      <c r="R48" s="6"/>
+      <c r="S48" s="6"/>
+      <c r="T48" s="6"/>
+      <c r="U48" s="6"/>
+      <c r="V48" s="6"/>
+      <c r="W48" s="6"/>
+      <c r="X48" s="6"/>
+      <c r="Y48" s="6"/>
+      <c r="Z48" s="6"/>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6"/>
+      <c r="K49" s="6"/>
+      <c r="L49" s="6"/>
+      <c r="M49" s="6"/>
+      <c r="N49" s="6"/>
+      <c r="O49" s="6"/>
+      <c r="P49" s="6"/>
+      <c r="Q49" s="6"/>
+      <c r="R49" s="6"/>
+      <c r="S49" s="6"/>
+      <c r="T49" s="6"/>
+      <c r="U49" s="6"/>
+      <c r="V49" s="6"/>
+      <c r="W49" s="6"/>
+      <c r="X49" s="6"/>
+      <c r="Y49" s="6"/>
+      <c r="Z49" s="6"/>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="6"/>
+      <c r="L50" s="6"/>
+      <c r="M50" s="6"/>
+      <c r="N50" s="6"/>
+      <c r="O50" s="6"/>
+      <c r="P50" s="6"/>
+      <c r="Q50" s="6"/>
+      <c r="R50" s="6"/>
+      <c r="S50" s="6"/>
+      <c r="T50" s="6"/>
+      <c r="U50" s="6"/>
+      <c r="V50" s="6"/>
+      <c r="W50" s="6"/>
+      <c r="X50" s="6"/>
+      <c r="Y50" s="6"/>
+      <c r="Z50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" s="6"/>
+      <c r="F51" s="6"/>
+      <c r="G51" s="6"/>
+      <c r="H51" s="6"/>
+      <c r="I51" s="6"/>
+      <c r="J51" s="6"/>
+      <c r="K51" s="6"/>
+      <c r="L51" s="6"/>
+      <c r="M51" s="6"/>
+      <c r="N51" s="6"/>
+      <c r="O51" s="6"/>
+      <c r="P51" s="6"/>
+      <c r="Q51" s="6"/>
+      <c r="R51" s="6"/>
+      <c r="S51" s="6"/>
+      <c r="T51" s="6"/>
+      <c r="U51" s="6"/>
+      <c r="V51" s="6"/>
+      <c r="W51" s="6"/>
+      <c r="X51" s="6"/>
+      <c r="Y51" s="6"/>
+      <c r="Z51" s="6"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B52" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E52" s="6"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="6"/>
+      <c r="I52" s="6"/>
+      <c r="J52" s="6"/>
+      <c r="K52" s="6"/>
+      <c r="L52" s="6"/>
+      <c r="M52" s="6"/>
+      <c r="N52" s="6"/>
+      <c r="O52" s="6"/>
+      <c r="P52" s="6"/>
+      <c r="Q52" s="6"/>
+      <c r="R52" s="6"/>
+      <c r="S52" s="6"/>
+      <c r="T52" s="6"/>
+      <c r="U52" s="6"/>
+      <c r="V52" s="6"/>
+      <c r="W52" s="6"/>
+      <c r="X52" s="6"/>
+      <c r="Y52" s="6"/>
+      <c r="Z52" s="6"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="6"/>
+      <c r="N53" s="6"/>
+      <c r="O53" s="6"/>
+      <c r="P53" s="6"/>
+      <c r="Q53" s="6"/>
+      <c r="R53" s="6"/>
+      <c r="S53" s="6"/>
+      <c r="T53" s="6"/>
+      <c r="U53" s="6"/>
+      <c r="V53" s="6"/>
+      <c r="W53" s="6"/>
+      <c r="X53" s="6"/>
+      <c r="Y53" s="6"/>
+      <c r="Z53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="B54" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="6"/>
+      <c r="N54" s="6"/>
+      <c r="O54" s="6"/>
+      <c r="P54" s="6"/>
+      <c r="Q54" s="6"/>
+      <c r="R54" s="6"/>
+      <c r="S54" s="6"/>
+      <c r="T54" s="6"/>
+      <c r="U54" s="6"/>
+      <c r="V54" s="6"/>
+      <c r="W54" s="6"/>
+      <c r="X54" s="6"/>
+      <c r="Y54" s="6"/>
+      <c r="Z54" s="6"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
+      <c r="L55" s="6"/>
+      <c r="M55" s="6"/>
+      <c r="N55" s="6"/>
+      <c r="O55" s="6"/>
+      <c r="P55" s="6"/>
+      <c r="Q55" s="6"/>
+      <c r="R55" s="6"/>
+      <c r="S55" s="6"/>
+      <c r="T55" s="6"/>
+      <c r="U55" s="6"/>
+      <c r="V55" s="6"/>
+      <c r="W55" s="6"/>
+      <c r="X55" s="6"/>
+      <c r="Y55" s="6"/>
+      <c r="Z55" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D30" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D55" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1484,7 +2196,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1507,13 +2219,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1542,7 +2254,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1575,7 +2287,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1608,7 +2320,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
input excel update and ini file
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -386,28 +386,28 @@
     <t xml:space="preserve">test_common_100_103_002</t>
   </si>
   <si>
+    <t xml:space="preserve">test_common_100_103_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_007</t>
+  </si>
+  <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_007</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_008</t>
@@ -703,7 +703,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="17.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1161,7 +1161,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1194,7 +1194,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1227,7 +1227,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z55"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1870,7 +1870,7 @@
         <v>118</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>58</v>
@@ -1881,10 +1881,10 @@
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" s="0" t="s">
         <v>120</v>
-      </c>
-      <c r="B47" s="0" t="s">
-        <v>121</v>
       </c>
       <c r="C47" s="13" t="s">
         <v>58</v>
@@ -1895,10 +1895,10 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>122</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>123</v>
       </c>
       <c r="C48" s="13" t="s">
         <v>58</v>
@@ -1931,10 +1931,10 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>58</v>
@@ -1967,10 +1967,10 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C50" s="13" t="s">
         <v>58</v>
@@ -2003,10 +2003,10 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B51" s="15" t="s">
         <v>126</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>119</v>
       </c>
       <c r="C51" s="13" t="s">
         <v>58</v>
@@ -2042,7 +2042,7 @@
         <v>127</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C52" s="13" t="s">
         <v>58</v>
@@ -2150,7 +2150,7 @@
         <v>130</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C55" s="13" t="s">
         <v>58</v>
@@ -2204,7 +2204,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2262,7 +2262,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2295,7 +2295,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2328,7 +2328,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
An emergency Fix to timecalculator logic in conftest file. In one process, if more than one testcases added in one pytest command it is considered as one process. In the end of each TC, the GlobalVariables.time_calc should be set to None
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="75">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -192,6 +192,21 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_dummy_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SubFeatureCodeDummy_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_dummy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_dummy_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SubFeatureCodeDummy_2</t>
   </si>
   <si>
     <t xml:space="preserve">test_com_100_101_005</t>
@@ -246,7 +261,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -276,6 +291,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -327,13 +348,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -353,12 +378,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="41.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.38"/>
@@ -884,7 +909,46 @@
         <v>7</v>
       </c>
       <c r="F29" s="0" t="n">
-        <f aca="false">TRUE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="F30" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="F31" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -905,7 +969,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:F1"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -941,7 +1005,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:F1"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -977,10 +1041,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="41.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.05"/>
@@ -1009,13 +1073,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F2" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1027,13 +1091,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F3" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1045,13 +1109,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1063,13 +1127,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F5" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1081,13 +1145,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>56</v>
-      </c>
       <c r="E6" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1099,13 +1163,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>62</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>57</v>
       </c>
       <c r="F7" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1117,13 +1181,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1135,13 +1199,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F9" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1153,13 +1217,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1183,7 +1247,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1207,13 +1271,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="F2" s="0" t="n">
         <f aca="false">FALSE()</f>
@@ -1237,7 +1301,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:F1"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1273,7 +1337,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:F1"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1309,7 +1373,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:F1"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.71"/>

</xml_diff>

<commit_message>
changes before avinash pull
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -161,19 +161,19 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_sa_100_102_026</t>
@@ -703,7 +703,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="17.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1019,12 +1019,12 @@
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>43</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="0" t="s">
         <v>43</v>
@@ -1052,16 +1052,16 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="C25" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1102,8 +1102,8 @@
       <c r="C28" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D28" s="14" t="s">
-        <v>44</v>
+      <c r="D28" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1116,8 +1116,8 @@
       <c r="C29" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="14" t="s">
-        <v>44</v>
+      <c r="D29" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1136,11 +1136,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D27" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D29" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D28:D30" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D30" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1161,7 +1161,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1194,7 +1194,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1227,7 +1227,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z55"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1302,7 +1302,7 @@
         <v>58</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1316,7 +1316,7 @@
         <v>58</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1330,7 +1330,7 @@
         <v>58</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1344,7 +1344,7 @@
         <v>58</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1358,7 +1358,7 @@
         <v>58</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1372,7 +1372,7 @@
         <v>58</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1386,7 +1386,7 @@
         <v>58</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1400,7 +1400,7 @@
         <v>58</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1484,7 +1484,7 @@
         <v>58</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1666,7 +1666,7 @@
         <v>58</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1694,7 +1694,7 @@
         <v>58</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1750,7 +1750,7 @@
         <v>58</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1862,7 +1862,7 @@
         <v>58</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1876,7 +1876,7 @@
         <v>58</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1904,7 +1904,7 @@
         <v>58</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
@@ -1940,7 +1940,7 @@
         <v>58</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
@@ -2204,7 +2204,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2262,7 +2262,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2295,7 +2295,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2328,7 +2328,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
integrated test cases with user assigner.
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -314,6 +314,9 @@
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_103_005</t>
   </si>
   <si>
@@ -333,9 +336,6 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_011</t>
@@ -359,7 +359,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -471,17 +471,6 @@
       <family val="3"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF00627A"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -538,7 +527,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -636,14 +625,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1232,7 +1213,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1300,7 +1281,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1740,13 +1721,13 @@
         <v>59</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>7</v>
+        <v>95</v>
       </c>
       <c r="E27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B28" s="21" t="s">
         <v>94</v>
@@ -1755,13 +1736,13 @@
         <v>59</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>7</v>
+        <v>95</v>
       </c>
       <c r="E28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B29" s="21" t="s">
         <v>92</v>
@@ -1775,10 +1756,10 @@
     </row>
     <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>59</v>
@@ -1789,10 +1770,10 @@
     </row>
     <row r="31" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>99</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>98</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>59</v>
@@ -1803,7 +1784,7 @@
     </row>
     <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B32" s="21" t="s">
         <v>89</v>
@@ -1817,7 +1798,7 @@
     </row>
     <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B33" s="21" t="s">
         <v>89</v>
@@ -1826,15 +1807,15 @@
         <v>59</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>102</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="s">
+      <c r="A34" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="B34" s="26" t="s">
-        <v>98</v>
+      <c r="B34" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>59</v>
@@ -1866,7 +1847,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1888,13 +1869,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="26" t="s">
         <v>106</v>
       </c>
       <c r="D2" s="18" t="s">
@@ -1924,7 +1905,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1957,7 +1938,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1990,7 +1971,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">

</xml_diff>

<commit_message>
changes before dev merge vineeth
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="133">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -171,9 +171,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_sa_100_102_026</t>
@@ -703,7 +700,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="17.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1061,15 +1058,15 @@
         <v>6</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="0" t="s">
         <v>49</v>
-      </c>
-      <c r="B26" s="0" t="s">
-        <v>50</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>6</v>
@@ -1080,10 +1077,10 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>6</v>
@@ -1094,10 +1091,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>52</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>53</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>6</v>
@@ -1108,10 +1105,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>6</v>
@@ -1122,10 +1119,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>6</v>
@@ -1161,7 +1158,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1194,7 +1191,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1227,7 +1224,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z55"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1251,13 +1248,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>57</v>
-      </c>
       <c r="C2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1265,13 +1262,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>7</v>
@@ -1279,13 +1276,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -1293,111 +1290,111 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>62</v>
-      </c>
       <c r="C5" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="0" t="s">
-        <v>69</v>
-      </c>
       <c r="C11" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>7</v>
@@ -1405,13 +1402,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>72</v>
-      </c>
       <c r="C13" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>7</v>
@@ -1419,13 +1416,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>7</v>
@@ -1433,13 +1430,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="0" t="s">
-        <v>75</v>
-      </c>
       <c r="C15" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>7</v>
@@ -1447,13 +1444,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="B16" s="0" t="s">
-        <v>77</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>7</v>
@@ -1461,13 +1458,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>7</v>
@@ -1475,13 +1472,13 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>7</v>
@@ -1489,13 +1486,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="0" t="s">
-        <v>81</v>
-      </c>
       <c r="C19" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>7</v>
@@ -1503,13 +1500,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>7</v>
@@ -1517,13 +1514,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="0" t="s">
-        <v>84</v>
-      </c>
       <c r="C21" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>7</v>
@@ -1531,13 +1528,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>7</v>
@@ -1545,13 +1542,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>7</v>
@@ -1559,13 +1556,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="0" t="s">
-        <v>88</v>
-      </c>
       <c r="C24" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>7</v>
@@ -1573,13 +1570,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>7</v>
@@ -1587,13 +1584,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="0" t="s">
-        <v>91</v>
-      </c>
       <c r="C26" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>7</v>
@@ -1601,13 +1598,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>7</v>
@@ -1615,13 +1612,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B28" s="0" t="s">
-        <v>94</v>
-      </c>
       <c r="C28" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>7</v>
@@ -1629,13 +1626,13 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>7</v>
@@ -1643,13 +1640,13 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>7</v>
@@ -1657,13 +1654,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B31" s="12" t="s">
-        <v>98</v>
-      </c>
       <c r="C31" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>7</v>
@@ -1671,13 +1668,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>100</v>
-      </c>
       <c r="C32" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>7</v>
@@ -1685,13 +1682,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>7</v>
@@ -1699,13 +1696,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B34" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="B34" s="12" t="s">
-        <v>103</v>
-      </c>
       <c r="C34" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>7</v>
@@ -1713,13 +1710,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>7</v>
@@ -1727,13 +1724,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B36" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B36" s="12" t="s">
-        <v>106</v>
-      </c>
       <c r="C36" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>7</v>
@@ -1741,13 +1738,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="B37" s="12" t="s">
-        <v>108</v>
-      </c>
       <c r="C37" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>7</v>
@@ -1755,13 +1752,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>7</v>
@@ -1769,13 +1766,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>7</v>
@@ -1783,13 +1780,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>7</v>
@@ -1797,13 +1794,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>7</v>
@@ -1811,13 +1808,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>7</v>
@@ -1825,13 +1822,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>7</v>
@@ -1839,13 +1836,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>7</v>
@@ -1853,13 +1850,13 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="B45" s="0" t="s">
-        <v>117</v>
-      </c>
       <c r="C45" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>7</v>
@@ -1867,13 +1864,13 @@
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>7</v>
@@ -1881,13 +1878,13 @@
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B47" s="0" t="s">
         <v>119</v>
       </c>
-      <c r="B47" s="0" t="s">
-        <v>120</v>
-      </c>
       <c r="C47" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>7</v>
@@ -1895,13 +1892,13 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="B48" s="15" t="s">
-        <v>122</v>
-      </c>
       <c r="C48" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>7</v>
@@ -1931,13 +1928,13 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>7</v>
@@ -1967,13 +1964,13 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>7</v>
@@ -2003,13 +2000,13 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="B51" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="B51" s="15" t="s">
-        <v>126</v>
-      </c>
       <c r="C51" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>7</v>
@@ -2039,13 +2036,13 @@
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>7</v>
@@ -2075,13 +2072,13 @@
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>7</v>
@@ -2111,13 +2108,13 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>7</v>
@@ -2147,13 +2144,13 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>7</v>
@@ -2204,7 +2201,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2227,13 +2224,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>132</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>133</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -2262,7 +2259,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2295,7 +2292,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2328,7 +2325,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Updated test cases with user assigner.
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -299,6 +299,9 @@
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_103_002</t>
   </si>
   <si>
@@ -312,9 +315,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_005</t>
@@ -1213,7 +1213,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1281,7 +1281,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1676,13 +1676,13 @@
         <v>59</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="E24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>89</v>
@@ -1691,16 +1691,16 @@
         <v>59</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="E25" s="7"/>
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>59</v>
@@ -1712,16 +1712,16 @@
     </row>
     <row r="27" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>59</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
       <c r="E27" s="7"/>
     </row>
@@ -1730,13 +1730,13 @@
         <v>96</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>59</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
       <c r="E28" s="7"/>
     </row>
@@ -1745,7 +1745,7 @@
         <v>97</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>59</v>
@@ -1793,7 +1793,7 @@
         <v>59</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1807,7 +1807,7 @@
         <v>59</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1847,7 +1847,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1905,7 +1905,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1938,7 +1938,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -1971,7 +1971,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">

</xml_diff>

<commit_message>
after taking pull from dev and config.ini modified
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="138">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -161,36 +161,36 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_102_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_sa_100_101_002</t>
   </si>
   <si>
@@ -375,6 +375,18 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_020</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_001</t>
@@ -560,7 +572,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -615,10 +627,6 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -703,7 +711,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="17.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1019,12 +1027,12 @@
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>43</v>
@@ -1038,7 +1046,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="0" t="s">
         <v>43</v>
@@ -1052,10 +1060,10 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" s="0" t="s">
         <v>47</v>
-      </c>
-      <c r="B25" s="0" t="s">
-        <v>48</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>6</v>
@@ -1066,10 +1074,10 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="0" t="s">
         <v>49</v>
-      </c>
-      <c r="B26" s="0" t="s">
-        <v>50</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>6</v>
@@ -1080,10 +1088,10 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>6</v>
@@ -1094,16 +1102,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="C28" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,13 +1119,13 @@
         <v>54</v>
       </c>
       <c r="B29" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1125,22 +1133,18 @@
         <v>55</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>7</v>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D27" type="list">
-      <formula1>"True,False"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D28:D30" type="list">
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D30" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1161,7 +1165,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1194,7 +1198,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1226,8 +1230,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z55"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Z58"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1302,7 +1306,7 @@
         <v>58</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1330,7 +1334,7 @@
         <v>58</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1400,7 +1404,7 @@
         <v>58</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1484,7 +1488,7 @@
         <v>58</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1666,7 +1670,7 @@
         <v>58</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1680,7 +1684,7 @@
         <v>58</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1694,7 +1698,7 @@
         <v>58</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1708,7 +1712,7 @@
         <v>58</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1722,7 +1726,7 @@
         <v>58</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,7 +1740,7 @@
         <v>58</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1750,7 +1754,7 @@
         <v>58</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1764,7 +1768,7 @@
         <v>58</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1778,7 +1782,7 @@
         <v>58</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1792,7 +1796,7 @@
         <v>58</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1806,7 +1810,7 @@
         <v>58</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1820,7 +1824,7 @@
         <v>58</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1834,7 +1838,7 @@
         <v>58</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1848,164 +1852,98 @@
         <v>58</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="B45" s="12" t="s">
         <v>117</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>58</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="B46" s="0" t="s">
+      <c r="B46" s="12" t="s">
         <v>117</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>58</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="B47" s="0" t="s">
+      <c r="B47" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="s">
         <v>120</v>
       </c>
-      <c r="C47" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
+      <c r="B48" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="C48" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="C48" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="6"/>
-      <c r="N48" s="6"/>
-      <c r="O48" s="6"/>
-      <c r="P48" s="6"/>
-      <c r="Q48" s="6"/>
-      <c r="R48" s="6"/>
-      <c r="S48" s="6"/>
-      <c r="T48" s="6"/>
-      <c r="U48" s="6"/>
-      <c r="V48" s="6"/>
-      <c r="W48" s="6"/>
-      <c r="X48" s="6"/>
-      <c r="Y48" s="6"/>
-      <c r="Z48" s="6"/>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
+      <c r="B49" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="B49" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
-      <c r="L49" s="6"/>
-      <c r="M49" s="6"/>
-      <c r="N49" s="6"/>
-      <c r="O49" s="6"/>
-      <c r="P49" s="6"/>
-      <c r="Q49" s="6"/>
-      <c r="R49" s="6"/>
-      <c r="S49" s="6"/>
-      <c r="T49" s="6"/>
-      <c r="U49" s="6"/>
-      <c r="V49" s="6"/>
-      <c r="W49" s="6"/>
-      <c r="X49" s="6"/>
-      <c r="Y49" s="6"/>
-      <c r="Z49" s="6"/>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
+      <c r="B50" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="B50" s="15" t="s">
-        <v>120</v>
-      </c>
       <c r="C50" s="13" t="s">
         <v>58</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="6"/>
-      <c r="N50" s="6"/>
-      <c r="O50" s="6"/>
-      <c r="P50" s="6"/>
-      <c r="Q50" s="6"/>
-      <c r="R50" s="6"/>
-      <c r="S50" s="6"/>
-      <c r="T50" s="6"/>
-      <c r="U50" s="6"/>
-      <c r="V50" s="6"/>
-      <c r="W50" s="6"/>
-      <c r="X50" s="6"/>
-      <c r="Y50" s="6"/>
-      <c r="Z50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
+      <c r="A51" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B51" s="15" t="s">
+      <c r="B51" s="14" t="s">
         <v>126</v>
       </c>
       <c r="C51" s="13" t="s">
@@ -2038,10 +1976,10 @@
       <c r="Z51" s="6"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
+      <c r="A52" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="B52" s="15" t="s">
+      <c r="B52" s="14" t="s">
         <v>126</v>
       </c>
       <c r="C52" s="13" t="s">
@@ -2074,11 +2012,11 @@
       <c r="Z52" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
+      <c r="A53" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="B53" s="15" t="s">
-        <v>117</v>
+      <c r="B53" s="14" t="s">
+        <v>124</v>
       </c>
       <c r="C53" s="13" t="s">
         <v>58</v>
@@ -2110,11 +2048,11 @@
       <c r="Z53" s="6"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
+      <c r="A54" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="B54" s="15" t="s">
-        <v>117</v>
+      <c r="B54" s="14" t="s">
+        <v>130</v>
       </c>
       <c r="C54" s="13" t="s">
         <v>58</v>
@@ -2146,11 +2084,11 @@
       <c r="Z54" s="6"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="15" t="s">
+      <c r="A55" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B55" s="14" t="s">
         <v>130</v>
-      </c>
-      <c r="B55" s="15" t="s">
-        <v>126</v>
       </c>
       <c r="C55" s="13" t="s">
         <v>58</v>
@@ -2181,9 +2119,117 @@
       <c r="Y55" s="6"/>
       <c r="Z55" s="6"/>
     </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B56" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6"/>
+      <c r="K56" s="6"/>
+      <c r="L56" s="6"/>
+      <c r="M56" s="6"/>
+      <c r="N56" s="6"/>
+      <c r="O56" s="6"/>
+      <c r="P56" s="6"/>
+      <c r="Q56" s="6"/>
+      <c r="R56" s="6"/>
+      <c r="S56" s="6"/>
+      <c r="T56" s="6"/>
+      <c r="U56" s="6"/>
+      <c r="V56" s="6"/>
+      <c r="W56" s="6"/>
+      <c r="X56" s="6"/>
+      <c r="Y56" s="6"/>
+      <c r="Z56" s="6"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B57" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6"/>
+      <c r="H57" s="6"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="6"/>
+      <c r="K57" s="6"/>
+      <c r="L57" s="6"/>
+      <c r="M57" s="6"/>
+      <c r="N57" s="6"/>
+      <c r="O57" s="6"/>
+      <c r="P57" s="6"/>
+      <c r="Q57" s="6"/>
+      <c r="R57" s="6"/>
+      <c r="S57" s="6"/>
+      <c r="T57" s="6"/>
+      <c r="U57" s="6"/>
+      <c r="V57" s="6"/>
+      <c r="W57" s="6"/>
+      <c r="X57" s="6"/>
+      <c r="Y57" s="6"/>
+      <c r="Z57" s="6"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B58" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
+      <c r="L58" s="6"/>
+      <c r="M58" s="6"/>
+      <c r="N58" s="6"/>
+      <c r="O58" s="6"/>
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="6"/>
+      <c r="T58" s="6"/>
+      <c r="U58" s="6"/>
+      <c r="V58" s="6"/>
+      <c r="W58" s="6"/>
+      <c r="X58" s="6"/>
+      <c r="Y58" s="6"/>
+      <c r="Z58" s="6"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D55" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D58" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2204,7 +2250,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2227,13 +2273,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -2262,7 +2308,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2295,7 +2341,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2328,7 +2374,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
updated db and excel
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -161,6 +161,9 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_102_008</t>
   </si>
   <si>
@@ -186,9 +189,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_sa_100_101_002</t>
@@ -711,7 +711,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="17.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1027,12 +1027,12 @@
         <v>6</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>43</v>
@@ -1041,12 +1041,12 @@
         <v>6</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B24" s="0" t="s">
         <v>43</v>
@@ -1055,29 +1055,29 @@
         <v>6</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>6</v>
@@ -1088,10 +1088,10 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="0" t="s">
         <v>50</v>
-      </c>
-      <c r="B27" s="0" t="s">
-        <v>49</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>6</v>
@@ -1102,16 +1102,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1119,13 +1119,13 @@
         <v>54</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,13 +1133,13 @@
         <v>55</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1165,7 +1165,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1198,7 +1198,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1231,7 +1231,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z58"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.95"/>
@@ -1264,7 +1264,7 @@
         <v>58</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1278,7 +1278,7 @@
         <v>58</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1292,7 +1292,7 @@
         <v>58</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1306,7 +1306,7 @@
         <v>58</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1320,7 +1320,7 @@
         <v>58</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1334,7 +1334,7 @@
         <v>58</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1348,7 +1348,7 @@
         <v>58</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1362,7 +1362,7 @@
         <v>58</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1376,7 +1376,7 @@
         <v>58</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1390,7 +1390,7 @@
         <v>58</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1404,7 +1404,7 @@
         <v>58</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1418,7 +1418,7 @@
         <v>58</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1432,7 +1432,7 @@
         <v>58</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1446,7 +1446,7 @@
         <v>58</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1460,7 +1460,7 @@
         <v>58</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1474,7 +1474,7 @@
         <v>58</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1488,7 +1488,7 @@
         <v>58</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1670,7 +1670,7 @@
         <v>58</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1684,7 +1684,7 @@
         <v>58</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1698,7 +1698,7 @@
         <v>58</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1712,7 +1712,7 @@
         <v>58</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1726,7 +1726,7 @@
         <v>58</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1740,7 +1740,7 @@
         <v>58</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1754,7 +1754,7 @@
         <v>58</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1768,7 +1768,7 @@
         <v>58</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1782,7 +1782,7 @@
         <v>58</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1796,7 +1796,7 @@
         <v>58</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1810,7 +1810,7 @@
         <v>58</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1824,7 +1824,7 @@
         <v>58</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1838,7 +1838,7 @@
         <v>58</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1852,7 +1852,7 @@
         <v>58</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1866,7 +1866,7 @@
         <v>58</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1880,7 +1880,7 @@
         <v>58</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1894,7 +1894,7 @@
         <v>58</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1908,7 +1908,7 @@
         <v>58</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1922,7 +1922,7 @@
         <v>58</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1936,7 +1936,7 @@
         <v>58</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1950,7 +1950,7 @@
         <v>58</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
@@ -1986,7 +1986,7 @@
         <v>58</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -2022,7 +2022,7 @@
         <v>58</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
@@ -2058,7 +2058,7 @@
         <v>58</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
@@ -2094,7 +2094,7 @@
         <v>58</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
@@ -2130,7 +2130,7 @@
         <v>58</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E56" s="6"/>
       <c r="F56" s="6"/>
@@ -2166,7 +2166,7 @@
         <v>58</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
@@ -2202,7 +2202,7 @@
         <v>58</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
@@ -2250,7 +2250,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2308,7 +2308,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2341,7 +2341,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2374,7 +2374,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
JIRA tickets: EzeAuto 95, 94, 75 are fixed - Rerun related
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="176">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -213,6 +213,18 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_dummy_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_dummy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_dummy_02</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_102_001</t>
@@ -934,7 +946,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.73"/>
@@ -1398,17 +1410,36 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="6"/>
+      <c r="A32" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E31" type="list">
-      <formula1>"True,False"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E32" type="list">
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E33" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1428,20 +1459,30 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.06"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1461,20 +1502,30 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.06"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1499,9 +1550,9 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="15" width="35.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="15" width="94.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="15" width="68.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="15" width="68.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="15" width="10.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="15" width="10.12"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="15" width="14.82"/>
   </cols>
   <sheetData>
@@ -1524,13 +1575,13 @@
     </row>
     <row r="2" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E2" s="21" t="s">
         <v>8</v>
@@ -1538,13 +1589,13 @@
     </row>
     <row r="3" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>8</v>
@@ -1552,13 +1603,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E4" s="21" t="s">
         <v>8</v>
@@ -1566,13 +1617,13 @@
     </row>
     <row r="5" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E5" s="21" t="s">
         <v>8</v>
@@ -1580,13 +1631,13 @@
     </row>
     <row r="6" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E6" s="21" t="s">
         <v>8</v>
@@ -1594,13 +1645,13 @@
     </row>
     <row r="7" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E7" s="21" t="s">
         <v>8</v>
@@ -1608,13 +1659,13 @@
     </row>
     <row r="8" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E8" s="21" t="s">
         <v>8</v>
@@ -1622,13 +1673,13 @@
     </row>
     <row r="9" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E9" s="21" t="s">
         <v>8</v>
@@ -1636,13 +1687,13 @@
     </row>
     <row r="10" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E10" s="21" t="s">
         <v>8</v>
@@ -1650,13 +1701,13 @@
     </row>
     <row r="11" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E11" s="21" t="s">
         <v>8</v>
@@ -1664,13 +1715,13 @@
     </row>
     <row r="12" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E12" s="21" t="s">
         <v>8</v>
@@ -1678,13 +1729,13 @@
     </row>
     <row r="13" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E13" s="21" t="s">
         <v>8</v>
@@ -1692,13 +1743,13 @@
     </row>
     <row r="14" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E14" s="21" t="s">
         <v>8</v>
@@ -1706,13 +1757,13 @@
     </row>
     <row r="15" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E15" s="21" t="s">
         <v>8</v>
@@ -1720,13 +1771,13 @@
     </row>
     <row r="16" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E16" s="21" t="s">
         <v>8</v>
@@ -1734,13 +1785,13 @@
     </row>
     <row r="17" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E17" s="21" t="s">
         <v>8</v>
@@ -1748,13 +1799,13 @@
     </row>
     <row r="18" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E18" s="21" t="s">
         <v>8</v>
@@ -1762,13 +1813,13 @@
     </row>
     <row r="19" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E19" s="21" t="s">
         <v>8</v>
@@ -1776,13 +1827,13 @@
     </row>
     <row r="20" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E20" s="21" t="s">
         <v>8</v>
@@ -1790,13 +1841,13 @@
     </row>
     <row r="21" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E21" s="21" t="s">
         <v>8</v>
@@ -1804,13 +1855,13 @@
     </row>
     <row r="22" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E22" s="21" t="s">
         <v>8</v>
@@ -1818,13 +1869,13 @@
     </row>
     <row r="23" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E23" s="21" t="s">
         <v>8</v>
@@ -1832,13 +1883,13 @@
     </row>
     <row r="24" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E24" s="21" t="s">
         <v>8</v>
@@ -1846,13 +1897,13 @@
     </row>
     <row r="25" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E25" s="21" t="s">
         <v>8</v>
@@ -1860,13 +1911,13 @@
     </row>
     <row r="26" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E26" s="21" t="s">
         <v>8</v>
@@ -1874,13 +1925,13 @@
     </row>
     <row r="27" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E27" s="21" t="s">
         <v>8</v>
@@ -1888,13 +1939,13 @@
     </row>
     <row r="28" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E28" s="21" t="s">
         <v>8</v>
@@ -1902,13 +1953,13 @@
     </row>
     <row r="29" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E29" s="21" t="s">
         <v>8</v>
@@ -1916,13 +1967,13 @@
     </row>
     <row r="30" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E30" s="21" t="s">
         <v>8</v>
@@ -1930,16 +1981,16 @@
     </row>
     <row r="31" customFormat="false" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="22" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E31" s="21" t="s">
         <v>8</v>
@@ -1947,16 +1998,16 @@
     </row>
     <row r="32" customFormat="false" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="22" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E32" s="21" t="s">
         <v>8</v>
@@ -1964,16 +2015,16 @@
     </row>
     <row r="33" customFormat="false" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E33" s="21" t="s">
         <v>8</v>
@@ -1981,16 +2032,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="22" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E34" s="21" t="s">
         <v>8</v>
@@ -1998,16 +2049,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E35" s="21" t="s">
         <v>8</v>
@@ -2015,16 +2066,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E36" s="21" t="s">
         <v>8</v>
@@ -2032,16 +2083,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E37" s="21" t="s">
         <v>8</v>
@@ -2049,16 +2100,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C38" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>118</v>
-      </c>
       <c r="D38" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E38" s="21" t="s">
         <v>8</v>
@@ -2066,16 +2117,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B39" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C39" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C39" s="15" t="s">
-        <v>121</v>
-      </c>
       <c r="D39" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E39" s="21" t="s">
         <v>8</v>
@@ -2083,16 +2134,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E40" s="21" t="s">
         <v>8</v>
@@ -2100,16 +2151,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E41" s="21" t="s">
         <v>8</v>
@@ -2117,16 +2168,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D42" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E42" s="21" t="s">
         <v>8</v>
@@ -2134,16 +2185,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E43" s="21" t="s">
         <v>8</v>
@@ -2151,16 +2202,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E44" s="21" t="s">
         <v>8</v>
@@ -2168,16 +2219,16 @@
     </row>
     <row r="45" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D45" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E45" s="21" t="s">
         <v>8</v>
@@ -2185,16 +2236,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="22" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E46" s="21" t="s">
         <v>8</v>
@@ -2202,16 +2253,16 @@
     </row>
     <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="22" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B47" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="C47" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="C47" s="15" t="s">
-        <v>138</v>
-      </c>
       <c r="D47" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E47" s="21" t="s">
         <v>8</v>
@@ -2219,13 +2270,13 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="15" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D48" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E48" s="21" t="s">
         <v>8</v>
@@ -2233,13 +2284,13 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="15" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E49" s="21" t="s">
         <v>8</v>
@@ -2247,13 +2298,13 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="15" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D50" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E50" s="21" t="s">
         <v>8</v>
@@ -2261,13 +2312,13 @@
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="15" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D51" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E51" s="21" t="s">
         <v>8</v>
@@ -2275,13 +2326,13 @@
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="15" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E52" s="21" t="s">
         <v>8</v>
@@ -2289,13 +2340,13 @@
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="C53" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C53" s="15" t="s">
-        <v>147</v>
-      </c>
       <c r="D53" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E53" s="21" t="s">
         <v>8</v>
@@ -2303,13 +2354,13 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="15" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D54" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E54" s="21" t="s">
         <v>8</v>
@@ -2317,13 +2368,13 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="15" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D55" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E55" s="21" t="s">
         <v>8</v>
@@ -2331,13 +2382,13 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="15" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D56" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E56" s="21" t="s">
         <v>8</v>
@@ -2345,13 +2396,13 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="15" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D57" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E57" s="21" t="s">
         <v>8</v>
@@ -2359,13 +2410,13 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="C58" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C58" s="15" t="s">
-        <v>153</v>
-      </c>
       <c r="D58" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E58" s="21" t="s">
         <v>8</v>
@@ -2373,16 +2424,16 @@
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="15" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B59" s="24" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E59" s="21" t="s">
         <v>8</v>
@@ -2390,16 +2441,16 @@
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="25" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E60" s="21" t="s">
         <v>8</v>
@@ -2407,16 +2458,16 @@
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="25" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B61" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="C61" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="C61" s="15" t="s">
-        <v>160</v>
-      </c>
       <c r="D61" s="15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E61" s="21" t="s">
         <v>8</v>
@@ -2424,16 +2475,16 @@
     </row>
     <row r="62" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="25" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B62" s="23" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E62" s="21" t="s">
         <v>8</v>
@@ -2441,16 +2492,16 @@
     </row>
     <row r="63" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="26" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B63" s="27" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D63" s="20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E63" s="21" t="s">
         <v>8</v>
@@ -3504,45 +3555,49 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="15.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="28" width="26.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="28" width="25.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="28" width="69.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="28" width="25.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="28" width="69.15"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="B2" s="30" t="s">
-        <v>170</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="B2" s="29"/>
       <c r="C2" s="30" t="s">
-        <v>171</v>
-      </c>
-      <c r="D2" s="31" t="s">
+        <v>174</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>175</v>
+      </c>
+      <c r="E2" s="31" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3562,20 +3617,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="15.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3595,20 +3653,30 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.06"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3628,20 +3696,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="15.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="15.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Config related Test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="105">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -330,6 +330,18 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_300_304_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_02</t>
   </si>
 </sst>
 </file>
@@ -622,7 +634,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultColWidth="17.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.5234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="87.38"/>
@@ -1048,7 +1060,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.82"/>
@@ -1116,7 +1128,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1149,7 +1161,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="81.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70.48"/>
@@ -1318,7 +1330,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -1376,7 +1388,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1409,7 +1421,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1441,8 +1453,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultColWidth="14.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64.42"/>
@@ -1813,9 +1825,51 @@
         <v>70</v>
       </c>
     </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D26" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D29" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
adapted CNP test scripts and removed space from rerun command.
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="193">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -167,424 +167,436 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_HDFC</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQR_Checkstatus_Failed_HDFC _08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQR_Checkstatus_AfterExpiry_HDFC _09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQR_HDFC_QR_Generation_Success_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_CheckStatus_After_qr_expiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Success_HDFC _01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Failed_HDFC _02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_AfterExpiry_HDFC _03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Success_HDFC _04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Failed_HDFC _05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_AfterExpiry_HDFC _06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_two_Callback_Success_HDFC_11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_disabled_HDFC_12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_enabled_HDFC_13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_HDFC_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_HDFC_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_HDFC_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_HDFC_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Pending_HDFC _018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_Failed_AUTOREFUND_ENABLED_HDFC_21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_full_Refund_via-Portal_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_partial_Refund_via-Portal_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_HDFC _08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Expired_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHREFUNDED_UPGRefund_UPGAutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_Success_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_Failed_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_RP_UPI_Success_Via_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_RP_upi collect_Success_Via_Pure_upi collect_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_RP_upi collect_failed_Via_Pure_upicollect_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_RP_UPI_Failed_Via_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Debit_Card_Success_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Debit_Card_Failed_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_After_Expiry_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_After_Timeout_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Debit_Card_After_Timeout_Cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_103_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_CNP_Cyber_Refund_Card_txn</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQR_Checkstatus_Failed_HDFC _08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQR_Checkstatus_AfterExpiry_HDFC _09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQR_HDFC_QR_Generation_Success_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_CheckStatus_After_qr_expiry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Success_HDFC _01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Failed_HDFC _02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_AfterExpiry_HDFC _03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Success_HDFC _04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Failed_HDFC _05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_AfterExpiry_HDFC _06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_two_Callback_Success_HDFC_11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_disabled_HDFC_12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_enabled_HDFC_13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_HDFC_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_HDFC_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_HDFC_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_HDFC_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Pending_HDFC _018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_Failed_AUTOREFUND_ENABLED_HDFC_21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_full_Refund_via-Portal_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_partial_Refund_via-Portal_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_HDFC _08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Expired_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHREFUNDED_UPGRefund_UPGAutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_Success_Cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_Failed_Cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_UPI_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_RP_upi collect_Success_Via_Pure_upi collect_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_RP_upiCollect_HDFC_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_RP_upi collect_failed_Via_Pure_upicollect_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Debit_Card_Success_Cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Debit_Card_Failed_Cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_After_Expiry_Cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Credit_Card_After_Timeout_Cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_103_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_CNP_Debit_Card_After_Timeout_Cyber</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -605,7 +617,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -677,6 +689,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -740,7 +759,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -806,6 +825,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -887,7 +914,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="17.21875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -1210,15 +1237,15 @@
         <v>7</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>48</v>
       </c>
       <c r="C23" s="0" t="s">
         <v>45</v>
@@ -1227,15 +1254,15 @@
         <v>7</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>49</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>50</v>
       </c>
       <c r="C24" s="0" t="s">
         <v>45</v>
@@ -1244,32 +1271,32 @@
         <v>7</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="C25" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="0" t="s">
-        <v>53</v>
-      </c>
       <c r="D25" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>54</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>55</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>7</v>
@@ -1280,67 +1307,67 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+      <c r="B28" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="C28" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>59</v>
-      </c>
       <c r="D28" s="16" t="s">
         <v>7</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="14" t="s">
-        <v>61</v>
-      </c>
       <c r="C29" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D29" s="16" t="s">
         <v>7</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="14" t="s">
-        <v>63</v>
-      </c>
       <c r="C30" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D30" s="16" t="s">
         <v>7</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1366,7 +1393,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1399,7 +1426,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1431,10 +1458,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA58"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AA59"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="81.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24.95"/>
@@ -1460,302 +1487,302 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>66</v>
-      </c>
       <c r="D2" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>69</v>
-      </c>
       <c r="C3" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>71</v>
-      </c>
       <c r="C4" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="C5" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="D5" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>76</v>
-      </c>
       <c r="C6" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="0" t="s">
-        <v>78</v>
-      </c>
       <c r="C7" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="0" t="s">
-        <v>80</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="0" t="s">
-        <v>82</v>
-      </c>
       <c r="C9" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="0" t="s">
-        <v>84</v>
-      </c>
       <c r="C10" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="C11" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>87</v>
-      </c>
       <c r="D11" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="0" t="s">
-        <v>89</v>
-      </c>
       <c r="C12" s="0" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="C13" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D13" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B14" s="0" t="s">
-        <v>94</v>
-      </c>
       <c r="C14" s="0" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="C15" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>97</v>
-      </c>
       <c r="D15" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="C16" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="0" t="s">
-        <v>100</v>
-      </c>
       <c r="D16" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="B17" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="C17" s="0" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="B18" s="0" t="s">
-        <v>104</v>
-      </c>
       <c r="C18" s="0" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="C19" s="0" t="s">
-        <v>106</v>
-      </c>
       <c r="D19" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>8</v>
@@ -1763,13 +1790,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>8</v>
@@ -1777,13 +1804,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="0" t="s">
-        <v>109</v>
-      </c>
       <c r="D21" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>8</v>
@@ -1791,13 +1818,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>8</v>
@@ -1805,13 +1832,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>8</v>
@@ -1819,13 +1846,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" s="0" t="s">
         <v>112</v>
       </c>
-      <c r="C24" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="D24" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>8</v>
@@ -1833,13 +1860,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>8</v>
@@ -1847,13 +1874,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>115</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>116</v>
-      </c>
       <c r="D26" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>8</v>
@@ -1861,13 +1888,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>8</v>
@@ -1875,13 +1902,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" s="0" t="s">
         <v>118</v>
       </c>
-      <c r="C28" s="0" t="s">
-        <v>119</v>
-      </c>
       <c r="D28" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>8</v>
@@ -1889,13 +1916,13 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>8</v>
@@ -1903,13 +1930,13 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>8</v>
@@ -1917,342 +1944,345 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="C31" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="C31" s="15" t="s">
-        <v>124</v>
-      </c>
       <c r="D31" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="B32" s="0" t="s">
         <v>125</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="C32" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C32" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D32" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="B33" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="B33" s="0" t="s">
-        <v>129</v>
-      </c>
       <c r="C33" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="B34" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="C34" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="C34" s="15" t="s">
-        <v>132</v>
-      </c>
       <c r="D34" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="B35" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="B35" s="0" t="s">
-        <v>134</v>
-      </c>
       <c r="C35" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="B36" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="C36" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="C36" s="15" t="s">
-        <v>137</v>
-      </c>
       <c r="D36" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B37" s="0" t="s">
         <v>138</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="C37" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="C37" s="15" t="s">
-        <v>140</v>
-      </c>
       <c r="D37" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="B38" s="0" t="s">
         <v>141</v>
       </c>
-      <c r="B38" s="0" t="s">
-        <v>142</v>
-      </c>
       <c r="C38" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="B39" s="0" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="0" t="s">
-        <v>144</v>
-      </c>
       <c r="C39" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="B40" s="0" t="s">
         <v>145</v>
       </c>
-      <c r="B40" s="0" t="s">
-        <v>146</v>
-      </c>
       <c r="C40" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="B41" s="0" t="s">
         <v>147</v>
       </c>
-      <c r="B41" s="0" t="s">
-        <v>148</v>
-      </c>
       <c r="C41" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="B42" s="0" t="s">
         <v>149</v>
       </c>
-      <c r="B42" s="0" t="s">
-        <v>150</v>
-      </c>
       <c r="C42" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="B43" s="0" t="s">
         <v>151</v>
       </c>
-      <c r="B43" s="0" t="s">
-        <v>152</v>
-      </c>
       <c r="C43" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="B44" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="B44" s="0" t="s">
-        <v>154</v>
-      </c>
       <c r="C44" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="B45" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="C45" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="C45" s="15" t="s">
-        <v>157</v>
-      </c>
       <c r="D45" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="B46" s="0" t="s">
         <v>158</v>
       </c>
-      <c r="B46" s="0" t="s">
-        <v>159</v>
-      </c>
       <c r="C46" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B47" s="0" t="s">
         <v>160</v>
       </c>
-      <c r="B47" s="0" t="s">
-        <v>161</v>
-      </c>
       <c r="C47" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="B48" s="0" t="s">
         <v>162</v>
       </c>
-      <c r="B48" s="0" t="s">
+      <c r="C48" s="0" t="s">
         <v>163</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>164</v>
-      </c>
       <c r="D48" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="B49" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="B49" s="14" t="s">
+      <c r="C49" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="D49" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="s">
         <v>166</v>
       </c>
-      <c r="C49" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="D49" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
+      <c r="B50" s="14" t="s">
         <v>167</v>
       </c>
       <c r="C50" s="0" t="s">
         <v>168</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
         <v>169</v>
       </c>
@@ -2263,10 +2293,10 @@
         <v>171</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F51" s="7"/>
       <c r="G51" s="7"/>
@@ -2291,7 +2321,7 @@
       <c r="Z51" s="7"/>
       <c r="AA51" s="7"/>
     </row>
-    <row r="52" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
         <v>172</v>
       </c>
@@ -2302,10 +2332,10 @@
         <v>171</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F52" s="7"/>
       <c r="G52" s="7"/>
@@ -2330,15 +2360,18 @@
       <c r="Z52" s="7"/>
       <c r="AA52" s="7"/>
     </row>
-    <row r="53" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
         <v>174</v>
       </c>
+      <c r="B53" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="C53" s="14" t="s">
         <v>168</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>8</v>
@@ -2366,21 +2399,21 @@
       <c r="Z53" s="7"/>
       <c r="AA53" s="7"/>
     </row>
-    <row r="54" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
@@ -2405,21 +2438,21 @@
       <c r="Z54" s="7"/>
       <c r="AA54" s="7"/>
     </row>
-    <row r="55" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C55" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B55" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="C55" s="14" t="s">
-        <v>177</v>
-      </c>
       <c r="D55" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
@@ -2444,21 +2477,21 @@
       <c r="Z55" s="7"/>
       <c r="AA55" s="7"/>
     </row>
-    <row r="56" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
@@ -2483,21 +2516,21 @@
       <c r="Z56" s="7"/>
       <c r="AA56" s="7"/>
     </row>
-    <row r="57" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
@@ -2522,21 +2555,21 @@
       <c r="Z57" s="7"/>
       <c r="AA57" s="7"/>
     </row>
-    <row r="58" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="F58" s="7"/>
       <c r="G58" s="7"/>
@@ -2561,9 +2594,26 @@
       <c r="Z58" s="7"/>
       <c r="AA58" s="7"/>
     </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="B59" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="C59" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D59" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E58" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E59" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2584,7 +2634,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2607,13 +2657,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
@@ -2642,7 +2692,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2675,7 +2725,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2708,7 +2758,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
excel and db update
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="239">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -197,6 +197,45 @@
     <t xml:space="preserve">test_sa_100_102_027</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_QR_Generation_Success_YES_ATOS _28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_Generation_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_QR_Generation_Failed_YES_ATOS _29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_Success_Via_CheckStatus_HDFC_49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_QR_Generation_Success_HDFC_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_QR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_CheckStatus_YES_ATOS</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_sa_100_101_001</t>
   </si>
   <si>
@@ -390,6 +429,105 @@
   </si>
   <si>
     <t xml:space="preserve">test_common_100_102_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_YES_ATOS_36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_YES_ATOS_37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_YES_ATOS_38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Pending_YES_ATOS_39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPGAutoRefund_Enabled_YES_ATOS _40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPGAutoRefund_Disabled_YES_ATOS _41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_YES_ATOS_42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_API_YES_ATOS_43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_Posted_YES_ATOS_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_Failed_YES_ATOS_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Success_UPI_Callback_HDFC _046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Success_UPI_Callback_HDFC _047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Expired_UPI_ExpiredCallback_HDFC _048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Success_Checkstatus_HDFC _048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Refund_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_014</t>
@@ -617,7 +755,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -676,14 +814,21 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -695,6 +840,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -759,7 +905,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -816,7 +962,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -828,11 +974,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -913,11 +1091,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="17.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M35"/>
+  <sheetFormatPr defaultColWidth="17.28125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="87.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.52"/>
   </cols>
@@ -1319,7 +1497,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" s="15" customFormat="true" ht="11.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
         <v>56</v>
       </c>
@@ -1332,11 +1510,11 @@
       <c r="D28" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E28" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E28" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" s="15" customFormat="true" ht="11.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
         <v>59</v>
       </c>
@@ -1349,11 +1527,11 @@
       <c r="D29" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E29" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E29" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" s="15" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
         <v>61</v>
       </c>
@@ -1361,18 +1539,103 @@
         <v>62</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D30" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" s="15" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" s="15" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E30" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E35" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1393,7 +1656,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1426,7 +1689,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1458,8 +1721,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA59"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AA74"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
@@ -1487,16 +1750,16 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>8</v>
@@ -1504,16 +1767,16 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>8</v>
@@ -1521,16 +1784,16 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>8</v>
@@ -1538,16 +1801,16 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>8</v>
@@ -1555,16 +1818,16 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>8</v>
@@ -1572,16 +1835,16 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>8</v>
@@ -1589,16 +1852,16 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="D8" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>8</v>
@@ -1606,16 +1869,16 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>8</v>
@@ -1623,16 +1886,16 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>8</v>
@@ -1640,16 +1903,16 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>8</v>
@@ -1657,16 +1920,16 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>8</v>
@@ -1674,16 +1937,16 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>8</v>
@@ -1691,16 +1954,16 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>8</v>
@@ -1708,16 +1971,16 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>8</v>
@@ -1725,16 +1988,16 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>8</v>
@@ -1742,16 +2005,16 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>8</v>
@@ -1759,16 +2022,16 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>8</v>
@@ -1776,13 +2039,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>8</v>
@@ -1790,13 +2053,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>8</v>
@@ -1804,13 +2067,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>8</v>
@@ -1818,13 +2081,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>8</v>
@@ -1832,13 +2095,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>8</v>
@@ -1846,13 +2109,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>8</v>
@@ -1860,13 +2123,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>8</v>
@@ -1874,13 +2137,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>8</v>
@@ -1888,13 +2151,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>8</v>
@@ -1902,13 +2165,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>8</v>
@@ -1916,13 +2179,13 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>8</v>
@@ -1930,285 +2193,285 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="B31" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="B32" s="0" t="s">
+    <row r="31" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C31" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="B33" s="0" t="s">
+      <c r="D31" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C32" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C33" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="B34" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="C34" s="15" t="s">
+      <c r="D32" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="D33" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C34" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="D34" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="B35" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="D35" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>134</v>
-      </c>
-      <c r="B36" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D36" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="B37" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="D37" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="B38" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D38" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="D34" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B35" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="C39" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="D39" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="C35" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="0" t="s">
+      <c r="D35" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="C40" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="B36" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="B41" s="0" t="s">
+      <c r="C36" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E36" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D41" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="B37" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="B42" s="0" t="s">
+      <c r="C37" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E37" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="C42" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="D42" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+      <c r="B38" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="B43" s="0" t="s">
+      <c r="C38" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="C43" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D43" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="B39" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="B44" s="0" t="s">
+      <c r="C39" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="D39" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E39" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" s="21" customFormat="true" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C44" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D44" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+      <c r="B40" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="C40" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="D40" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" s="21" customFormat="true" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="C45" s="15" t="s">
+      <c r="B41" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="D45" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E45" s="6" t="s">
+      <c r="C41" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D41" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" s="21" customFormat="true" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="B42" s="24" t="s">
+        <v>159</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D42" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E42" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" s="21" customFormat="true" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E43" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" s="21" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="B44" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="D44" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E44" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" s="21" customFormat="true" ht="15.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="B45" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="D45" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E45" s="23" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>8</v>
@@ -2216,16 +2479,16 @@
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>8</v>
@@ -2233,50 +2496,50 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="C48" s="0" t="s">
-        <v>163</v>
+        <v>174</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>172</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="C49" s="0" t="s">
-        <v>163</v>
+        <v>175</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>177</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B50" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="C50" s="0" t="s">
-        <v>168</v>
+        <v>178</v>
+      </c>
+      <c r="B50" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>177</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>8</v>
@@ -2284,336 +2547,591 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="B51" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>171</v>
+        <v>180</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>182</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="7"/>
-      <c r="I51" s="7"/>
-      <c r="J51" s="7"/>
-      <c r="K51" s="7"/>
-      <c r="L51" s="7"/>
-      <c r="M51" s="7"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="7"/>
-      <c r="P51" s="7"/>
-      <c r="Q51" s="7"/>
-      <c r="R51" s="7"/>
-      <c r="S51" s="7"/>
-      <c r="T51" s="7"/>
-      <c r="U51" s="7"/>
-      <c r="V51" s="7"/>
-      <c r="W51" s="7"/>
-      <c r="X51" s="7"/>
-      <c r="Y51" s="7"/>
-      <c r="Z51" s="7"/>
-      <c r="AA51" s="7"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="B52" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="C52" s="14" t="s">
-        <v>171</v>
+        <v>183</v>
+      </c>
+      <c r="B52" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>185</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F52" s="7"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
-      <c r="J52" s="7"/>
-      <c r="K52" s="7"/>
-      <c r="L52" s="7"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="7"/>
-      <c r="P52" s="7"/>
-      <c r="Q52" s="7"/>
-      <c r="R52" s="7"/>
-      <c r="S52" s="7"/>
-      <c r="T52" s="7"/>
-      <c r="U52" s="7"/>
-      <c r="V52" s="7"/>
-      <c r="W52" s="7"/>
-      <c r="X52" s="7"/>
-      <c r="Y52" s="7"/>
-      <c r="Z52" s="7"/>
-      <c r="AA52" s="7"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="B53" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="C53" s="14" t="s">
-        <v>168</v>
+        <v>186</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="C53" s="15" t="s">
+        <v>182</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F53" s="7"/>
-      <c r="G53" s="7"/>
-      <c r="H53" s="7"/>
-      <c r="I53" s="7"/>
-      <c r="J53" s="7"/>
-      <c r="K53" s="7"/>
-      <c r="L53" s="7"/>
-      <c r="M53" s="7"/>
-      <c r="N53" s="7"/>
-      <c r="O53" s="7"/>
-      <c r="P53" s="7"/>
-      <c r="Q53" s="7"/>
-      <c r="R53" s="7"/>
-      <c r="S53" s="7"/>
-      <c r="T53" s="7"/>
-      <c r="U53" s="7"/>
-      <c r="V53" s="7"/>
-      <c r="W53" s="7"/>
-      <c r="X53" s="7"/>
-      <c r="Y53" s="7"/>
-      <c r="Z53" s="7"/>
-      <c r="AA53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="B54" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>178</v>
+        <v>188</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="C54" s="15" t="s">
+        <v>185</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F54" s="7"/>
-      <c r="G54" s="7"/>
-      <c r="H54" s="7"/>
-      <c r="I54" s="7"/>
-      <c r="J54" s="7"/>
-      <c r="K54" s="7"/>
-      <c r="L54" s="7"/>
-      <c r="M54" s="7"/>
-      <c r="N54" s="7"/>
-      <c r="O54" s="7"/>
-      <c r="P54" s="7"/>
-      <c r="Q54" s="7"/>
-      <c r="R54" s="7"/>
-      <c r="S54" s="7"/>
-      <c r="T54" s="7"/>
-      <c r="U54" s="7"/>
-      <c r="V54" s="7"/>
-      <c r="W54" s="7"/>
-      <c r="X54" s="7"/>
-      <c r="Y54" s="7"/>
-      <c r="Z54" s="7"/>
-      <c r="AA54" s="7"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="B55" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="C55" s="14" t="s">
-        <v>178</v>
+        <v>190</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="C55" s="15" t="s">
+        <v>185</v>
       </c>
       <c r="D55" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F55" s="7"/>
-      <c r="G55" s="7"/>
-      <c r="H55" s="7"/>
-      <c r="I55" s="7"/>
-      <c r="J55" s="7"/>
-      <c r="K55" s="7"/>
-      <c r="L55" s="7"/>
-      <c r="M55" s="7"/>
-      <c r="N55" s="7"/>
-      <c r="O55" s="7"/>
-      <c r="P55" s="7"/>
-      <c r="Q55" s="7"/>
-      <c r="R55" s="7"/>
-      <c r="S55" s="7"/>
-      <c r="T55" s="7"/>
-      <c r="U55" s="7"/>
-      <c r="V55" s="7"/>
-      <c r="W55" s="7"/>
-      <c r="X55" s="7"/>
-      <c r="Y55" s="7"/>
-      <c r="Z55" s="7"/>
-      <c r="AA55" s="7"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="B56" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="C56" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="C56" s="14" t="s">
-        <v>163</v>
-      </c>
       <c r="D56" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
-      <c r="H56" s="7"/>
-      <c r="I56" s="7"/>
-      <c r="J56" s="7"/>
-      <c r="K56" s="7"/>
-      <c r="L56" s="7"/>
-      <c r="M56" s="7"/>
-      <c r="N56" s="7"/>
-      <c r="O56" s="7"/>
-      <c r="P56" s="7"/>
-      <c r="Q56" s="7"/>
-      <c r="R56" s="7"/>
-      <c r="S56" s="7"/>
-      <c r="T56" s="7"/>
-      <c r="U56" s="7"/>
-      <c r="V56" s="7"/>
-      <c r="W56" s="7"/>
-      <c r="X56" s="7"/>
-      <c r="Y56" s="7"/>
-      <c r="Z56" s="7"/>
-      <c r="AA56" s="7"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>184</v>
-      </c>
-      <c r="C57" s="14" t="s">
-        <v>163</v>
+        <v>195</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>185</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
-      <c r="H57" s="7"/>
-      <c r="I57" s="7"/>
-      <c r="J57" s="7"/>
-      <c r="K57" s="7"/>
-      <c r="L57" s="7"/>
-      <c r="M57" s="7"/>
-      <c r="N57" s="7"/>
-      <c r="O57" s="7"/>
-      <c r="P57" s="7"/>
-      <c r="Q57" s="7"/>
-      <c r="R57" s="7"/>
-      <c r="S57" s="7"/>
-      <c r="T57" s="7"/>
-      <c r="U57" s="7"/>
-      <c r="V57" s="7"/>
-      <c r="W57" s="7"/>
-      <c r="X57" s="7"/>
-      <c r="Y57" s="7"/>
-      <c r="Z57" s="7"/>
-      <c r="AA57" s="7"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="C58" s="14" t="s">
-        <v>178</v>
+        <v>197</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>182</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F58" s="7"/>
-      <c r="G58" s="7"/>
-      <c r="H58" s="7"/>
-      <c r="I58" s="7"/>
-      <c r="J58" s="7"/>
-      <c r="K58" s="7"/>
-      <c r="L58" s="7"/>
-      <c r="M58" s="7"/>
-      <c r="N58" s="7"/>
-      <c r="O58" s="7"/>
-      <c r="P58" s="7"/>
-      <c r="Q58" s="7"/>
-      <c r="R58" s="7"/>
-      <c r="S58" s="7"/>
-      <c r="T58" s="7"/>
-      <c r="U58" s="7"/>
-      <c r="V58" s="7"/>
-      <c r="W58" s="7"/>
-      <c r="X58" s="7"/>
-      <c r="Y58" s="7"/>
-      <c r="Z58" s="7"/>
-      <c r="AA58" s="7"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="B59" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="C59" s="14" t="s">
-        <v>163</v>
+      <c r="A59" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="B59" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>182</v>
       </c>
       <c r="D59" s="16" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>189</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="B60" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="C60" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="B61" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D61" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D62" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="B63" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="C63" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="D63" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>210</v>
+      </c>
+      <c r="B64" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="C64" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="D64" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="13.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="B65" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="C65" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="D65" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="B66" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="C66" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D66" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F66" s="7"/>
+      <c r="G66" s="7"/>
+      <c r="H66" s="7"/>
+      <c r="I66" s="7"/>
+      <c r="J66" s="7"/>
+      <c r="K66" s="7"/>
+      <c r="L66" s="7"/>
+      <c r="M66" s="7"/>
+      <c r="N66" s="7"/>
+      <c r="O66" s="7"/>
+      <c r="P66" s="7"/>
+      <c r="Q66" s="7"/>
+      <c r="R66" s="7"/>
+      <c r="S66" s="7"/>
+      <c r="T66" s="7"/>
+      <c r="U66" s="7"/>
+      <c r="V66" s="7"/>
+      <c r="W66" s="7"/>
+      <c r="X66" s="7"/>
+      <c r="Y66" s="7"/>
+      <c r="Z66" s="7"/>
+      <c r="AA66" s="7"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="B67" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="C67" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="7"/>
+      <c r="M67" s="7"/>
+      <c r="N67" s="7"/>
+      <c r="O67" s="7"/>
+      <c r="P67" s="7"/>
+      <c r="Q67" s="7"/>
+      <c r="R67" s="7"/>
+      <c r="S67" s="7"/>
+      <c r="T67" s="7"/>
+      <c r="U67" s="7"/>
+      <c r="V67" s="7"/>
+      <c r="W67" s="7"/>
+      <c r="X67" s="7"/>
+      <c r="Y67" s="7"/>
+      <c r="Z67" s="7"/>
+      <c r="AA67" s="7"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="B68" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="C68" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="D68" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="7"/>
+      <c r="I68" s="7"/>
+      <c r="J68" s="7"/>
+      <c r="K68" s="7"/>
+      <c r="L68" s="7"/>
+      <c r="M68" s="7"/>
+      <c r="N68" s="7"/>
+      <c r="O68" s="7"/>
+      <c r="P68" s="7"/>
+      <c r="Q68" s="7"/>
+      <c r="R68" s="7"/>
+      <c r="S68" s="7"/>
+      <c r="T68" s="7"/>
+      <c r="U68" s="7"/>
+      <c r="V68" s="7"/>
+      <c r="W68" s="7"/>
+      <c r="X68" s="7"/>
+      <c r="Y68" s="7"/>
+      <c r="Z68" s="7"/>
+      <c r="AA68" s="7"/>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="B69" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="C69" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D69" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="7"/>
+      <c r="I69" s="7"/>
+      <c r="J69" s="7"/>
+      <c r="K69" s="7"/>
+      <c r="L69" s="7"/>
+      <c r="M69" s="7"/>
+      <c r="N69" s="7"/>
+      <c r="O69" s="7"/>
+      <c r="P69" s="7"/>
+      <c r="Q69" s="7"/>
+      <c r="R69" s="7"/>
+      <c r="S69" s="7"/>
+      <c r="T69" s="7"/>
+      <c r="U69" s="7"/>
+      <c r="V69" s="7"/>
+      <c r="W69" s="7"/>
+      <c r="X69" s="7"/>
+      <c r="Y69" s="7"/>
+      <c r="Z69" s="7"/>
+      <c r="AA69" s="7"/>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="C70" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D70" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F70" s="7"/>
+      <c r="G70" s="7"/>
+      <c r="H70" s="7"/>
+      <c r="I70" s="7"/>
+      <c r="J70" s="7"/>
+      <c r="K70" s="7"/>
+      <c r="L70" s="7"/>
+      <c r="M70" s="7"/>
+      <c r="N70" s="7"/>
+      <c r="O70" s="7"/>
+      <c r="P70" s="7"/>
+      <c r="Q70" s="7"/>
+      <c r="R70" s="7"/>
+      <c r="S70" s="7"/>
+      <c r="T70" s="7"/>
+      <c r="U70" s="7"/>
+      <c r="V70" s="7"/>
+      <c r="W70" s="7"/>
+      <c r="X70" s="7"/>
+      <c r="Y70" s="7"/>
+      <c r="Z70" s="7"/>
+      <c r="AA70" s="7"/>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="B71" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="D71" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="7"/>
+      <c r="I71" s="7"/>
+      <c r="J71" s="7"/>
+      <c r="K71" s="7"/>
+      <c r="L71" s="7"/>
+      <c r="M71" s="7"/>
+      <c r="N71" s="7"/>
+      <c r="O71" s="7"/>
+      <c r="P71" s="7"/>
+      <c r="Q71" s="7"/>
+      <c r="R71" s="7"/>
+      <c r="S71" s="7"/>
+      <c r="T71" s="7"/>
+      <c r="U71" s="7"/>
+      <c r="V71" s="7"/>
+      <c r="W71" s="7"/>
+      <c r="X71" s="7"/>
+      <c r="Y71" s="7"/>
+      <c r="Z71" s="7"/>
+      <c r="AA71" s="7"/>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="B72" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="D72" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F72" s="7"/>
+      <c r="G72" s="7"/>
+      <c r="H72" s="7"/>
+      <c r="I72" s="7"/>
+      <c r="J72" s="7"/>
+      <c r="K72" s="7"/>
+      <c r="L72" s="7"/>
+      <c r="M72" s="7"/>
+      <c r="N72" s="7"/>
+      <c r="O72" s="7"/>
+      <c r="P72" s="7"/>
+      <c r="Q72" s="7"/>
+      <c r="R72" s="7"/>
+      <c r="S72" s="7"/>
+      <c r="T72" s="7"/>
+      <c r="U72" s="7"/>
+      <c r="V72" s="7"/>
+      <c r="W72" s="7"/>
+      <c r="X72" s="7"/>
+      <c r="Y72" s="7"/>
+      <c r="Z72" s="7"/>
+      <c r="AA72" s="7"/>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="B73" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C73" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D73" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="7"/>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="7"/>
+      <c r="N73" s="7"/>
+      <c r="O73" s="7"/>
+      <c r="P73" s="7"/>
+      <c r="Q73" s="7"/>
+      <c r="R73" s="7"/>
+      <c r="S73" s="7"/>
+      <c r="T73" s="7"/>
+      <c r="U73" s="7"/>
+      <c r="V73" s="7"/>
+      <c r="W73" s="7"/>
+      <c r="X73" s="7"/>
+      <c r="Y73" s="7"/>
+      <c r="Z73" s="7"/>
+      <c r="AA73" s="7"/>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="B74" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="C74" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="D74" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E59" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E74" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2634,7 +3152,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -2657,13 +3175,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>191</v>
+        <v>237</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>192</v>
+        <v>238</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
@@ -2692,7 +3210,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2725,7 +3243,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2758,7 +3276,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="14.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
date and time validation incorported for one upi test case and added date_and_time utility
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -1439,7 +1439,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -1472,7 +1472,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -2144,7 +2144,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
         <v>139</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
         <v>149</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>56</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2413,10 +2413,10 @@
         <v>56</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
         <v>177</v>
       </c>
@@ -2427,7 +2427,7 @@
         <v>56</v>
       </c>
       <c r="E54" s="16" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2500,7 +2500,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
         <v>186</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>56</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,7 +2965,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="21" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="21" width="25.4"/>
@@ -3023,7 +3023,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -3056,7 +3056,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -3089,7 +3089,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">

</xml_diff>

<commit_message>
updated the date validation with valid names.
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -1439,7 +1439,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -1472,7 +1472,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -2144,7 +2144,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
         <v>139</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
         <v>149</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>56</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2413,10 +2413,10 @@
         <v>56</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
         <v>177</v>
       </c>
@@ -2427,7 +2427,7 @@
         <v>56</v>
       </c>
       <c r="E54" s="16" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2500,7 +2500,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
         <v>186</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>56</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,7 +2965,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="21" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="21" width="25.4"/>
@@ -3023,7 +3023,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -3056,7 +3056,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
@@ -3089,7 +3089,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">

</xml_diff>

<commit_message>
Added Ezewallet related TCS
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="342">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -608,7 +608,7 @@
     <t xml:space="preserve">test_common_300_301_001</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_tax_outstandingV3</t>
+    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_tax_outstandingV3_01</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Goa</t>
@@ -620,19 +620,19 @@
     <t xml:space="preserve">test_common_300_301_002</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_trade_outstanding</t>
+    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_trade_outstanding_02</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_301_003</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_rental_outstanding</t>
+    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_rental_outstanding_03</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_001</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_pos_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_pos_details_01</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_01</t>
@@ -641,31 +641,31 @@
     <t xml:space="preserve">test_common_300_302_002</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_dth_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_dth_details_02</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_003</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_rtn_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_rtn_details_03</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_004</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_rtn_dth_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_rtn_dth_details_04</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_005</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Mobile</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Mobile_05</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_006</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Account</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Account_06</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_02</t>
@@ -674,31 +674,31 @@
     <t xml:space="preserve">test_common_300_302_007</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Mobile</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Mobile_07</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_008</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Account</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Account_08</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_009</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_prepaid_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_prepaid_details_09</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_010</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_butterfly</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_butterfly_11</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_011</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_Order_Details</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_Order_Details_12</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_03</t>
@@ -707,19 +707,19 @@
     <t xml:space="preserve">test_common_300_302_012</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_mobile</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_mobile_13</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_302_013</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_landline</t>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_landline_15</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_303_001</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_User_Charges_Tax_PullV2</t>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_User_Charges_Tax_PullV2_01</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_GWMC_01</t>
@@ -728,31 +728,31 @@
     <t xml:space="preserve">test_common_300_303_002</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Meter_Charges_Tax_PullV2</t>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Meter_Charges_Tax_PullV2_02</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_303_003</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Trade_Tax_PullV2</t>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Trade_Tax_PullV2_03</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_303_004</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_wcdemand</t>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_wcdemand_04</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_303_005</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_head</t>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_head_05</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_303_006</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax</t>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_06</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_GWMC_02</t>
@@ -761,7 +761,7 @@
     <t xml:space="preserve">test_common_300_304_001</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_details_01</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_01</t>
@@ -770,31 +770,31 @@
     <t xml:space="preserve">test_common_300_304_002</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_water</t>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_water_05</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_304_003</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_prop</t>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_prop_05</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_304_004</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_update_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_update_details_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_304_005</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_details_04</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_300_304_006</t>
   </si>
   <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_update_details</t>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_update_details_04</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_02</t>
@@ -807,6 +807,9 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agency_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_200_201_002</t>
@@ -1158,7 +1161,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1175,12 +1178,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF87CEEB"/>
         <bgColor rgb="FFB4C7DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1232,7 +1229,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1314,14 +1311,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1407,7 +1396,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="18.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -1886,7 +1875,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1919,7 +1908,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1952,7 +1941,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA59"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
@@ -3127,7 +3116,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -3185,7 +3174,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3218,7 +3207,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3251,7 +3240,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="16.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="75.14"/>
@@ -3757,7 +3746,7 @@
       <c r="A30" s="17" t="s">
         <v>257</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="20" t="s">
         <v>258</v>
       </c>
       <c r="C30" s="10" t="s">
@@ -3767,15 +3756,15 @@
         <v>195</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>260</v>
-      </c>
-      <c r="B31" s="21" t="s">
         <v>261</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>262</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>259</v>
@@ -3784,15 +3773,15 @@
         <v>195</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>262</v>
-      </c>
-      <c r="B32" s="22" t="s">
         <v>263</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>264</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>259</v>
@@ -3801,15 +3790,15 @@
         <v>195</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C33" s="10" t="s">
         <v>259</v>
@@ -3818,15 +3807,15 @@
         <v>195</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>259</v>
@@ -3835,586 +3824,586 @@
         <v>195</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>268</v>
-      </c>
-      <c r="B35" s="22" t="s">
         <v>269</v>
       </c>
+      <c r="B35" s="20" t="s">
+        <v>270</v>
+      </c>
       <c r="C35" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="C36" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="B36" s="20" t="s">
-        <v>272</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>270</v>
-      </c>
       <c r="D36" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>275</v>
-      </c>
-      <c r="B38" s="22" t="s">
         <v>276</v>
       </c>
+      <c r="B38" s="20" t="s">
+        <v>277</v>
+      </c>
       <c r="C38" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D38" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
+        <v>279</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="B39" s="22" t="s">
-        <v>279</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>277</v>
-      </c>
       <c r="D39" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17" t="s">
-        <v>280</v>
-      </c>
-      <c r="B40" s="22" t="s">
         <v>281</v>
       </c>
+      <c r="B40" s="20" t="s">
+        <v>282</v>
+      </c>
       <c r="C40" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="17" t="s">
-        <v>282</v>
-      </c>
-      <c r="B41" s="22" t="s">
         <v>283</v>
       </c>
+      <c r="B41" s="20" t="s">
+        <v>284</v>
+      </c>
       <c r="C41" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D41" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D42" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
-        <v>286</v>
-      </c>
-      <c r="B43" s="21" t="s">
         <v>287</v>
       </c>
+      <c r="B43" s="20" t="s">
+        <v>288</v>
+      </c>
       <c r="C43" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D43" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
+        <v>290</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="B44" s="21" t="s">
-        <v>290</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>288</v>
-      </c>
       <c r="D44" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="B46" s="21" t="s">
         <v>294</v>
       </c>
+      <c r="B46" s="20" t="s">
+        <v>295</v>
+      </c>
       <c r="C46" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="17" t="s">
-        <v>295</v>
-      </c>
-      <c r="B47" s="21" t="s">
         <v>296</v>
       </c>
+      <c r="B47" s="20" t="s">
+        <v>297</v>
+      </c>
       <c r="C47" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D48" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="B49" s="20" t="s">
-        <v>301</v>
-      </c>
-      <c r="C49" s="10" t="s">
-        <v>299</v>
-      </c>
       <c r="D49" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="17" t="s">
-        <v>306</v>
-      </c>
-      <c r="B52" s="21" t="s">
         <v>307</v>
       </c>
+      <c r="B52" s="20" t="s">
+        <v>308</v>
+      </c>
       <c r="C52" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D52" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D53" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="C54" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="B54" s="22" t="s">
-        <v>312</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>310</v>
-      </c>
       <c r="D54" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D56" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="17" t="s">
-        <v>315</v>
-      </c>
-      <c r="B57" s="22" t="s">
         <v>316</v>
       </c>
+      <c r="B57" s="20" t="s">
+        <v>317</v>
+      </c>
       <c r="C57" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D57" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="B58" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="C58" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="B58" s="22" t="s">
-        <v>319</v>
-      </c>
-      <c r="C58" s="10" t="s">
-        <v>317</v>
-      </c>
       <c r="D58" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="17" t="s">
-        <v>320</v>
-      </c>
-      <c r="B59" s="22" t="s">
         <v>321</v>
       </c>
+      <c r="B59" s="20" t="s">
+        <v>322</v>
+      </c>
       <c r="C59" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D59" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="17" t="s">
-        <v>322</v>
-      </c>
-      <c r="B60" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="B60" s="20" t="s">
+        <v>324</v>
+      </c>
       <c r="C60" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D60" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F60" s="23"/>
+        <v>260</v>
+      </c>
+      <c r="F60" s="21"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="17" t="s">
-        <v>324</v>
-      </c>
-      <c r="B61" s="22" t="s">
         <v>325</v>
       </c>
+      <c r="B61" s="20" t="s">
+        <v>326</v>
+      </c>
       <c r="C61" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D61" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="17" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="B63" s="20" t="s">
+        <v>331</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="B63" s="22" t="s">
-        <v>330</v>
-      </c>
-      <c r="C63" s="10" t="s">
-        <v>328</v>
-      </c>
       <c r="D63" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="17" t="s">
-        <v>331</v>
-      </c>
-      <c r="B64" s="22" t="s">
         <v>332</v>
       </c>
+      <c r="B64" s="20" t="s">
+        <v>333</v>
+      </c>
       <c r="C64" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D64" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="17" t="s">
-        <v>333</v>
-      </c>
-      <c r="B65" s="22" t="s">
         <v>334</v>
       </c>
+      <c r="B65" s="20" t="s">
+        <v>335</v>
+      </c>
       <c r="C65" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D65" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="17" t="s">
-        <v>335</v>
-      </c>
-      <c r="B66" s="22" t="s">
         <v>336</v>
       </c>
+      <c r="B66" s="20" t="s">
+        <v>337</v>
+      </c>
       <c r="C66" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D66" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="17" t="s">
-        <v>337</v>
-      </c>
-      <c r="B67" s="22" t="s">
         <v>338</v>
       </c>
+      <c r="B67" s="20" t="s">
+        <v>339</v>
+      </c>
       <c r="C67" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D67" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B68" s="20" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D68" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes to ezewallet TCS
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -617,286 +617,286 @@
     <t xml:space="preserve">API_DB/Common</t>
   </si>
   <si>
+    <t xml:space="preserve">test_common_300_301_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_trade_outstanding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_301_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_rental_outstanding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_pos_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_dth_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_rtn_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_rtn_dth_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_prepaid_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_butterfly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_Order_Details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_302_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_landline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_303_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_User_Charges_Tax_PullV2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_GWMC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_303_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Meter_Charges_Tax_PullV2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_303_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Trade_Tax_PullV2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_303_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_wcdemand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_303_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_303_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_GWMC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_water</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_prop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_update_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_300_304_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_update_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agency_Card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agency_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agency_UPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Transfer_FromAgency_ToAgent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Transfer_FromAgency_ToAgent_MoreThan_Balance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Transfer_FromAgency_ToAgent_Zero_Amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Withdraw_FromAgent_ToAgency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agency_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Withdraw_FromAgent_More_than_Balance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_201_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Withdraw_FromAgent_Zero_amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_203_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agency_Fetch_Passbook_statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Fetch_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_203_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_TransferAmount_ToAgent_Fetch_passbook_statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_203_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_WithdrawAmount_FromAgent_Fetch_passbook_statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_203_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_Multiple_transactions_Fetch_passbook_statement_Agency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_203_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_fetch_Invalid_Merchant_Passbook_statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_200_202_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agent_01</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_301_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_trade_outstanding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_301_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Goa_fetch_get_rental_outstanding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_pos_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_dth_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_airtel_rtn_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_rtn_dth_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_postpaid_Account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_fixedLine_Account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_prepaid_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_butterfly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_Order_Details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_Airtel_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_302_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_Airtel_fetch_get_active_landline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_303_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_User_Charges_Tax_PullV2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_GWMC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_303_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Meter_Charges_Tax_PullV2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_303_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_Trade_Tax_PullV2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_303_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_wcdemand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_303_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax_head</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_303_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_GWMC_fetch_get_gwmc_tax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_GWMC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_304_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_304_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_water</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_304_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_BMC_prop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_304_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_property_update_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_304_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_300_304_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Config_BMP_fetch_get_mp_water_update_details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Config_BMC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agency_Card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agency_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agency_UPI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Transfer_FromAgency_ToAgent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Transfer_FromAgency_ToAgent_MoreThan_Balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Transfer_FromAgency_ToAgent_Zero_Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Withdraw_FromAgent_ToAgency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agency_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Withdraw_FromAgent_More_than_Balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_201_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Withdraw_FromAgent_Zero_amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_203_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agency_Fetch_Passbook_statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Fetch_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_203_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_TransferAmount_ToAgent_Fetch_passbook_statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_203_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_WithdrawAmount_FromAgent_Fetch_passbook_statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_203_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_Multiple_transactions_Fetch_passbook_statement_Agency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_203_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_fetch_Invalid_Merchant_Passbook_statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_200_202_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_Ezewallet_DigitalTopUp_Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agent_01</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_200_202_002</t>
@@ -1410,7 +1410,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="18.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -1889,7 +1889,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1922,7 +1922,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1955,7 +1955,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA59"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
@@ -3130,7 +3130,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -3188,7 +3188,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3221,7 +3221,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3254,7 +3254,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="75.14"/>
@@ -3294,15 +3294,15 @@
         <v>195</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>197</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>198</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>194</v>
@@ -3311,15 +3311,15 @@
         <v>195</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>199</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>200</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>194</v>
@@ -3328,443 +3328,443 @@
         <v>195</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>203</v>
-      </c>
       <c r="D5" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="B6" s="20" t="s">
-        <v>205</v>
-      </c>
       <c r="C6" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="20" t="s">
-        <v>207</v>
-      </c>
       <c r="C7" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>209</v>
-      </c>
       <c r="C8" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>211</v>
-      </c>
       <c r="C9" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="C10" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>214</v>
-      </c>
       <c r="D10" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="B11" s="20" t="s">
-        <v>216</v>
-      </c>
       <c r="C11" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="B12" s="20" t="s">
-        <v>218</v>
-      </c>
       <c r="C12" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="B13" s="20" t="s">
-        <v>220</v>
-      </c>
       <c r="C13" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="B14" s="20" t="s">
-        <v>222</v>
-      </c>
       <c r="C14" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="C15" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>225</v>
-      </c>
       <c r="D15" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="B16" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="B16" s="20" t="s">
-        <v>227</v>
-      </c>
       <c r="C16" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" s="20" t="s">
         <v>228</v>
       </c>
-      <c r="B17" s="20" t="s">
-        <v>229</v>
-      </c>
       <c r="C17" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="C18" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>232</v>
-      </c>
       <c r="D18" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="B19" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="B19" s="20" t="s">
-        <v>234</v>
-      </c>
       <c r="C19" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="B20" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="B20" s="20" t="s">
-        <v>236</v>
-      </c>
       <c r="C20" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="B21" s="20" t="s">
-        <v>238</v>
-      </c>
       <c r="C21" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="B22" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="C22" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="C23" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="C23" s="10" t="s">
-        <v>243</v>
-      </c>
       <c r="D23" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="C24" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>246</v>
-      </c>
       <c r="D24" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>247</v>
       </c>
-      <c r="B25" s="20" t="s">
-        <v>248</v>
-      </c>
       <c r="C25" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
+        <v>248</v>
+      </c>
+      <c r="B26" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="B26" s="20" t="s">
-        <v>250</v>
-      </c>
       <c r="C26" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="B27" s="20" t="s">
         <v>251</v>
       </c>
-      <c r="B27" s="20" t="s">
-        <v>252</v>
-      </c>
       <c r="C27" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="B28" s="20" t="s">
-        <v>254</v>
-      </c>
       <c r="C28" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="B29" s="20" t="s">
         <v>255</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="C29" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="C29" s="10" t="s">
-        <v>257</v>
-      </c>
       <c r="D29" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>196</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="B30" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="C30" s="10" t="s">
         <v>259</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>260</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>195</v>
@@ -3775,13 +3775,13 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="B31" s="21" t="s">
-        <v>262</v>
-      </c>
       <c r="C31" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>195</v>
@@ -3792,13 +3792,13 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="B32" s="22" t="s">
         <v>263</v>
       </c>
-      <c r="B32" s="22" t="s">
-        <v>264</v>
-      </c>
       <c r="C32" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>195</v>
@@ -3809,13 +3809,13 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
+        <v>264</v>
+      </c>
+      <c r="B33" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="B33" s="20" t="s">
-        <v>266</v>
-      </c>
       <c r="C33" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>195</v>
@@ -3826,13 +3826,13 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="B34" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="B34" s="20" t="s">
-        <v>268</v>
-      </c>
       <c r="C34" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>195</v>
@@ -3843,13 +3843,13 @@
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="B35" s="22" t="s">
         <v>269</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="C35" s="10" t="s">
         <v>270</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>271</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>195</v>
@@ -3860,13 +3860,13 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="B36" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="B36" s="20" t="s">
-        <v>273</v>
-      </c>
       <c r="C36" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>195</v>
@@ -3877,13 +3877,13 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="B37" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="B37" s="20" t="s">
-        <v>275</v>
-      </c>
       <c r="C37" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>195</v>
@@ -3894,13 +3894,13 @@
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="B38" s="22" t="s">
         <v>276</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="C38" s="10" t="s">
         <v>277</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>278</v>
       </c>
       <c r="D38" s="10" t="s">
         <v>195</v>
@@ -3911,13 +3911,13 @@
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="B39" s="22" t="s">
         <v>279</v>
       </c>
-      <c r="B39" s="22" t="s">
-        <v>280</v>
-      </c>
       <c r="C39" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>195</v>
@@ -3928,13 +3928,13 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="B40" s="22" t="s">
         <v>281</v>
       </c>
-      <c r="B40" s="22" t="s">
-        <v>282</v>
-      </c>
       <c r="C40" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>195</v>
@@ -3945,13 +3945,13 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="B41" s="22" t="s">
         <v>283</v>
       </c>
-      <c r="B41" s="22" t="s">
-        <v>284</v>
-      </c>
       <c r="C41" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D41" s="10" t="s">
         <v>195</v>
@@ -3962,13 +3962,13 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="B42" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="B42" s="20" t="s">
-        <v>286</v>
-      </c>
       <c r="C42" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D42" s="10" t="s">
         <v>195</v>
@@ -3979,19 +3979,19 @@
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="B43" s="21" t="s">
         <v>287</v>
       </c>
-      <c r="B43" s="21" t="s">
+      <c r="C43" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="D43" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>289</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4002,13 +4002,13 @@
         <v>291</v>
       </c>
       <c r="C44" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>289</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4019,13 +4019,13 @@
         <v>293</v>
       </c>
       <c r="C45" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>289</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,13 +4036,13 @@
         <v>295</v>
       </c>
       <c r="C46" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>289</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4053,13 +4053,13 @@
         <v>297</v>
       </c>
       <c r="C47" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>289</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4076,7 +4076,7 @@
         <v>195</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4093,7 +4093,7 @@
         <v>195</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4110,7 +4110,7 @@
         <v>195</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4127,7 +4127,7 @@
         <v>195</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4144,7 +4144,7 @@
         <v>195</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4161,7 +4161,7 @@
         <v>195</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4178,7 +4178,7 @@
         <v>195</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4186,7 +4186,7 @@
         <v>314</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C55" s="10" t="s">
         <v>311</v>
@@ -4195,7 +4195,7 @@
         <v>195</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4203,7 +4203,7 @@
         <v>315</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C56" s="10" t="s">
         <v>311</v>
@@ -4212,7 +4212,7 @@
         <v>195</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>8</v>
+        <v>289</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
run db val tcs
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -1410,7 +1410,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="19.40625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.43359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -1889,7 +1889,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1922,7 +1922,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1955,7 +1955,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA59"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
@@ -3130,7 +3130,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -3188,7 +3188,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3221,7 +3221,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3254,7 +3254,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="75.14"/>

</xml_diff>

<commit_message>
Added card HDFC cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="483">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -1094,193 +1094,388 @@
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Sale_01</t>
   </si>
   <si>
+    <t xml:space="preserve">test_common_100_104_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Sale_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Void_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Void_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Reversal_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_HDFC_Sale_01</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
   </si>
   <si>
-    <t xml:space="preserve">test_common_100_104_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_DEBIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_DEBIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_CREDIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_CREDIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMV_CREDIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_DEBIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Sale_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_DEBIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_DEBIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_CREDIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_CREDIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Sale_EMVCTLS_CREDIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_DEBIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Void_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_DEBIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_DEBIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_CREDIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_CREDIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMV_CREDIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_DEBIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Void_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_DEBIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_DEBIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_CREDIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_CREDIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Void_EMVCTLS_CREDIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_DEBIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Reversal_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_DEBIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_DEBIT_RUPAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_CREDIT_VISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_CREDIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_104_030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonUI_Common_ATOS_TLE_Card_Reversal_EMV_CREDIT_RUPAY</t>
+    <t xml:space="preserve">test_common_100_104_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_HDFC_Sale_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Sale_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_HDFC_Void_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_HDFC_Void_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Void_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Reversal_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_HDFC_Reversal_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Reversal_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Reversal_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Reversal_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Reversal_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_HDFC_Card_Reversal_EMV_CREDIT_RUPAY</t>
   </si>
 </sst>
 </file>
@@ -1624,7 +1819,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="20.65234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="21.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -2103,7 +2298,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2136,7 +2331,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2169,7 +2364,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA59"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
@@ -3344,7 +3539,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -3402,7 +3597,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3435,7 +3630,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3467,8 +3662,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
-  <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F133"/>
+  <sheetFormatPr defaultColWidth="17.8671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="75.14"/>
@@ -4732,15 +4927,15 @@
         <v>195</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="17" t="s">
+        <v>355</v>
+      </c>
+      <c r="B75" s="20" t="s">
         <v>356</v>
-      </c>
-      <c r="B75" s="20" t="s">
-        <v>357</v>
       </c>
       <c r="C75" s="10" t="s">
         <v>354</v>
@@ -4749,15 +4944,15 @@
         <v>195</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="17" t="s">
+        <v>357</v>
+      </c>
+      <c r="B76" s="20" t="s">
         <v>358</v>
-      </c>
-      <c r="B76" s="20" t="s">
-        <v>359</v>
       </c>
       <c r="C76" s="10" t="s">
         <v>354</v>
@@ -4766,15 +4961,15 @@
         <v>195</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="B77" s="20" t="s">
         <v>360</v>
-      </c>
-      <c r="B77" s="20" t="s">
-        <v>361</v>
       </c>
       <c r="C77" s="10" t="s">
         <v>354</v>
@@ -4783,15 +4978,15 @@
         <v>195</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="B78" s="20" t="s">
         <v>362</v>
-      </c>
-      <c r="B78" s="20" t="s">
-        <v>363</v>
       </c>
       <c r="C78" s="10" t="s">
         <v>354</v>
@@ -4800,15 +4995,15 @@
         <v>195</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="B79" s="20" t="s">
         <v>364</v>
-      </c>
-      <c r="B79" s="20" t="s">
-        <v>365</v>
       </c>
       <c r="C79" s="10" t="s">
         <v>354</v>
@@ -4817,420 +5012,930 @@
         <v>195</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="17" t="s">
+        <v>365</v>
+      </c>
+      <c r="B80" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="B80" s="20" t="s">
+      <c r="C80" s="10" t="s">
         <v>367</v>
       </c>
-      <c r="C80" s="10" t="s">
-        <v>368</v>
-      </c>
       <c r="D80" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="B81" s="20" t="s">
         <v>369</v>
       </c>
-      <c r="B81" s="20" t="s">
-        <v>370</v>
-      </c>
       <c r="C81" s="10" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D81" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="B82" s="20" t="s">
         <v>371</v>
       </c>
-      <c r="B82" s="20" t="s">
-        <v>372</v>
-      </c>
       <c r="C82" s="10" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D82" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="B83" s="20" t="s">
         <v>373</v>
       </c>
-      <c r="B83" s="20" t="s">
-        <v>374</v>
-      </c>
       <c r="C83" s="10" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="B84" s="20" t="s">
         <v>375</v>
       </c>
-      <c r="B84" s="20" t="s">
-        <v>376</v>
-      </c>
       <c r="C84" s="10" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D84" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="17" t="s">
+        <v>376</v>
+      </c>
+      <c r="B85" s="20" t="s">
         <v>377</v>
       </c>
-      <c r="B85" s="20" t="s">
-        <v>378</v>
-      </c>
       <c r="C85" s="10" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D85" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="17" t="s">
+        <v>378</v>
+      </c>
+      <c r="B86" s="20" t="s">
         <v>379</v>
       </c>
-      <c r="B86" s="20" t="s">
+      <c r="C86" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="C86" s="10" t="s">
-        <v>381</v>
-      </c>
       <c r="D86" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="17" t="s">
+        <v>381</v>
+      </c>
+      <c r="B87" s="20" t="s">
         <v>382</v>
       </c>
-      <c r="B87" s="20" t="s">
-        <v>383</v>
-      </c>
       <c r="C87" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="17" t="s">
+        <v>383</v>
+      </c>
+      <c r="B88" s="20" t="s">
         <v>384</v>
       </c>
-      <c r="B88" s="20" t="s">
-        <v>385</v>
-      </c>
       <c r="C88" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D88" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="B89" s="20" t="s">
         <v>386</v>
       </c>
-      <c r="B89" s="20" t="s">
-        <v>387</v>
-      </c>
       <c r="C89" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D89" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="B90" s="20" t="s">
         <v>388</v>
       </c>
-      <c r="B90" s="20" t="s">
-        <v>389</v>
-      </c>
       <c r="C90" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D90" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="17" t="s">
+        <v>389</v>
+      </c>
+      <c r="B91" s="20" t="s">
         <v>390</v>
       </c>
-      <c r="B91" s="20" t="s">
-        <v>391</v>
-      </c>
       <c r="C91" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="17" t="s">
+        <v>391</v>
+      </c>
+      <c r="B92" s="20" t="s">
         <v>392</v>
       </c>
-      <c r="B92" s="20" t="s">
+      <c r="C92" s="10" t="s">
         <v>393</v>
       </c>
-      <c r="C92" s="10" t="s">
-        <v>394</v>
-      </c>
       <c r="D92" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="17" t="s">
+        <v>394</v>
+      </c>
+      <c r="B93" s="20" t="s">
         <v>395</v>
       </c>
-      <c r="B93" s="20" t="s">
-        <v>396</v>
-      </c>
       <c r="C93" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="17" t="s">
+        <v>396</v>
+      </c>
+      <c r="B94" s="20" t="s">
         <v>397</v>
       </c>
-      <c r="B94" s="20" t="s">
-        <v>398</v>
-      </c>
       <c r="C94" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="17" t="s">
+        <v>398</v>
+      </c>
+      <c r="B95" s="20" t="s">
         <v>399</v>
       </c>
-      <c r="B95" s="20" t="s">
-        <v>400</v>
-      </c>
       <c r="C95" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D95" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="17" t="s">
+        <v>400</v>
+      </c>
+      <c r="B96" s="20" t="s">
         <v>401</v>
       </c>
-      <c r="B96" s="20" t="s">
-        <v>402</v>
-      </c>
       <c r="C96" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D96" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="17" t="s">
+        <v>402</v>
+      </c>
+      <c r="B97" s="20" t="s">
         <v>403</v>
       </c>
-      <c r="B97" s="20" t="s">
-        <v>404</v>
-      </c>
       <c r="C97" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D97" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="17" t="s">
+        <v>404</v>
+      </c>
+      <c r="B98" s="20" t="s">
         <v>405</v>
       </c>
-      <c r="B98" s="20" t="s">
+      <c r="C98" s="10" t="s">
         <v>406</v>
       </c>
-      <c r="C98" s="10" t="s">
-        <v>407</v>
-      </c>
       <c r="D98" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="B99" s="20" t="s">
         <v>408</v>
       </c>
-      <c r="B99" s="20" t="s">
-        <v>409</v>
-      </c>
       <c r="C99" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D99" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="17" t="s">
+        <v>409</v>
+      </c>
+      <c r="B100" s="20" t="s">
         <v>410</v>
       </c>
-      <c r="B100" s="20" t="s">
-        <v>411</v>
-      </c>
       <c r="C100" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D100" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="B101" s="20" t="s">
         <v>412</v>
       </c>
-      <c r="B101" s="20" t="s">
-        <v>413</v>
-      </c>
       <c r="C101" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D101" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="17" t="s">
+        <v>413</v>
+      </c>
+      <c r="B102" s="20" t="s">
         <v>414</v>
       </c>
-      <c r="B102" s="20" t="s">
-        <v>415</v>
-      </c>
       <c r="C102" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D102" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>355</v>
+        <v>8</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="17" t="s">
+        <v>415</v>
+      </c>
+      <c r="B103" s="20" t="s">
         <v>416</v>
       </c>
-      <c r="B103" s="20" t="s">
+      <c r="C103" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="D103" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="17" t="s">
         <v>417</v>
       </c>
-      <c r="C103" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="D103" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E103" s="6" t="s">
-        <v>355</v>
+      <c r="B104" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="C104" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D104" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="17" t="s">
+        <v>421</v>
+      </c>
+      <c r="B105" s="20" t="s">
+        <v>422</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D105" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="17" t="s">
+        <v>423</v>
+      </c>
+      <c r="B106" s="20" t="s">
+        <v>424</v>
+      </c>
+      <c r="C106" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D106" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="17" t="s">
+        <v>425</v>
+      </c>
+      <c r="B107" s="20" t="s">
+        <v>426</v>
+      </c>
+      <c r="C107" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D107" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="B108" s="20" t="s">
+        <v>428</v>
+      </c>
+      <c r="C108" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D108" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E108" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="B109" s="20" t="s">
+        <v>430</v>
+      </c>
+      <c r="C109" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D109" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E109" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="B110" s="20" t="s">
+        <v>432</v>
+      </c>
+      <c r="C110" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="D110" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E110" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="17" t="s">
+        <v>434</v>
+      </c>
+      <c r="B111" s="20" t="s">
+        <v>435</v>
+      </c>
+      <c r="C111" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="D111" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E111" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="17" t="s">
+        <v>436</v>
+      </c>
+      <c r="B112" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="C112" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="D112" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E112" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="17" t="s">
+        <v>438</v>
+      </c>
+      <c r="B113" s="20" t="s">
+        <v>439</v>
+      </c>
+      <c r="C113" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="D113" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E113" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="B114" s="20" t="s">
+        <v>441</v>
+      </c>
+      <c r="C114" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="D114" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E114" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="17" t="s">
+        <v>442</v>
+      </c>
+      <c r="B115" s="20" t="s">
+        <v>443</v>
+      </c>
+      <c r="C115" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="D115" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="B116" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="C116" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D116" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="B117" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="C117" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D117" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E117" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="B118" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="C118" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D118" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E118" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="17" t="s">
+        <v>451</v>
+      </c>
+      <c r="B119" s="20" t="s">
+        <v>452</v>
+      </c>
+      <c r="C119" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D119" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E119" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="17" t="s">
+        <v>453</v>
+      </c>
+      <c r="B120" s="20" t="s">
+        <v>454</v>
+      </c>
+      <c r="C120" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D120" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="17" t="s">
+        <v>455</v>
+      </c>
+      <c r="B121" s="20" t="s">
+        <v>456</v>
+      </c>
+      <c r="C121" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D121" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="B122" s="20" t="s">
+        <v>458</v>
+      </c>
+      <c r="C122" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="D122" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E122" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="17" t="s">
+        <v>460</v>
+      </c>
+      <c r="B123" s="20" t="s">
+        <v>461</v>
+      </c>
+      <c r="C123" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="D123" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E123" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="B124" s="20" t="s">
+        <v>463</v>
+      </c>
+      <c r="C124" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="D124" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E124" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="B125" s="20" t="s">
+        <v>465</v>
+      </c>
+      <c r="C125" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="D125" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E125" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="17" t="s">
+        <v>466</v>
+      </c>
+      <c r="B126" s="20" t="s">
+        <v>467</v>
+      </c>
+      <c r="C126" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="D126" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E126" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B127" s="20" t="s">
+        <v>469</v>
+      </c>
+      <c r="C127" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="D127" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E127" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="B128" s="20" t="s">
+        <v>471</v>
+      </c>
+      <c r="C128" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D128" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E128" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="B129" s="20" t="s">
+        <v>474</v>
+      </c>
+      <c r="C129" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D129" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E129" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="B130" s="20" t="s">
+        <v>476</v>
+      </c>
+      <c r="C130" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D130" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E130" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="17" t="s">
+        <v>477</v>
+      </c>
+      <c r="B131" s="20" t="s">
+        <v>478</v>
+      </c>
+      <c r="C131" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D131" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E131" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="17" t="s">
+        <v>479</v>
+      </c>
+      <c r="B132" s="20" t="s">
+        <v>480</v>
+      </c>
+      <c r="C132" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D132" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E132" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="B133" s="20" t="s">
+        <v>482</v>
+      </c>
+      <c r="C133" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D133" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E133" s="6" t="s">
+        <v>420</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E103" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E133" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Card API scripts changes
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="610">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -617,6 +617,9 @@
     <t xml:space="preserve">API_DB/Common</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_300_301_002</t>
   </si>
   <si>
@@ -1094,9 +1097,6 @@
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_ATOS_TLE_Sale_01</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_common_100_104_002</t>
   </si>
   <si>
@@ -1662,6 +1662,201 @@
   </si>
   <si>
     <t xml:space="preserve">NonUI_Common_PRIZMV2_Card_Reversal_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_091</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_FDC_Sale_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_093</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_097</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_FDC_Sale_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_098</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Sale_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_FDC_Void_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_109</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_FDC_Void_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_113</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_114</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Void_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_115</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Reversal_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Card_FDC_Reversal_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_116</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Reversal_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_117</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Reversal_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Reversal_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_119</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Reversal_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_104_120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonUI_Common_FDC_Card_Reversal_EMV_CREDIT_RUPAY</t>
   </si>
 </sst>
 </file>
@@ -2005,7 +2200,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="21.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="21.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -2484,7 +2679,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2517,7 +2712,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2550,7 +2745,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA59"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78"/>
@@ -3725,7 +3920,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -3783,7 +3978,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3816,7 +4011,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3848,8 +4043,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F163"/>
-  <sheetFormatPr defaultColWidth="18.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F193"/>
+  <sheetFormatPr defaultColWidth="18.3828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="75.14"/>
@@ -3888,15 +4083,15 @@
         <v>195</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>194</v>
@@ -3905,15 +4100,15 @@
         <v>195</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>194</v>
@@ -3922,1198 +4117,1198 @@
         <v>195</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="B6" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>202</v>
-      </c>
       <c r="D6" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="B11" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>213</v>
-      </c>
       <c r="D11" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="B16" s="20" t="s">
-        <v>226</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>224</v>
-      </c>
       <c r="D16" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B19" s="20" t="s">
-        <v>233</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>231</v>
-      </c>
       <c r="D19" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="B25" s="20" t="s">
-        <v>247</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>245</v>
-      </c>
       <c r="D25" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="B31" s="20" t="s">
-        <v>261</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>259</v>
-      </c>
       <c r="D31" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="C36" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="B36" s="20" t="s">
-        <v>272</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>270</v>
-      </c>
       <c r="D36" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D38" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
+        <v>279</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="B39" s="20" t="s">
-        <v>279</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>277</v>
-      </c>
       <c r="D39" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D41" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D42" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D43" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
+        <v>290</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="B44" s="20" t="s">
-        <v>290</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>288</v>
-      </c>
       <c r="D44" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D48" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="B49" s="20" t="s">
-        <v>301</v>
-      </c>
-      <c r="C49" s="10" t="s">
-        <v>299</v>
-      </c>
       <c r="D49" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D52" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D53" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="C54" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="B54" s="20" t="s">
-        <v>312</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>310</v>
-      </c>
       <c r="D54" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D56" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="17" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D57" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D58" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="17" t="s">
+        <v>323</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="C59" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="B59" s="20" t="s">
-        <v>323</v>
-      </c>
-      <c r="C59" s="10" t="s">
-        <v>321</v>
-      </c>
       <c r="D59" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="17" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D60" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D61" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="17" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="B63" s="20" t="s">
+        <v>331</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="B63" s="20" t="s">
-        <v>330</v>
-      </c>
-      <c r="C63" s="10" t="s">
-        <v>328</v>
-      </c>
       <c r="D63" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D64" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="17" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B65" s="20" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D65" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
       <c r="F65" s="21"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D66" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B67" s="20" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D67" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="B68" s="20" t="s">
+        <v>342</v>
+      </c>
+      <c r="C68" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="B68" s="20" t="s">
-        <v>341</v>
-      </c>
-      <c r="C68" s="10" t="s">
-        <v>339</v>
-      </c>
       <c r="D68" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B69" s="20" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D69" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B70" s="20" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B73" s="20" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="17" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5124,13 +5319,13 @@
         <v>357</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5141,13 +5336,13 @@
         <v>359</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D76" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5158,13 +5353,13 @@
         <v>361</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D77" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,13 +5370,13 @@
         <v>363</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D78" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5192,13 +5387,13 @@
         <v>365</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D79" s="10" t="s">
         <v>195</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5215,7 +5410,7 @@
         <v>195</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5232,7 +5427,7 @@
         <v>195</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5249,7 +5444,7 @@
         <v>195</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5266,7 +5461,7 @@
         <v>195</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5283,7 +5478,7 @@
         <v>195</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5300,7 +5495,7 @@
         <v>195</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5317,7 +5512,7 @@
         <v>195</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5334,7 +5529,7 @@
         <v>195</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5351,7 +5546,7 @@
         <v>195</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5368,7 +5563,7 @@
         <v>195</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5385,7 +5580,7 @@
         <v>195</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5402,7 +5597,7 @@
         <v>195</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5419,7 +5614,7 @@
         <v>195</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5436,7 +5631,7 @@
         <v>195</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5453,7 +5648,7 @@
         <v>195</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5470,7 +5665,7 @@
         <v>195</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5487,7 +5682,7 @@
         <v>195</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5504,7 +5699,7 @@
         <v>195</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5521,7 +5716,7 @@
         <v>195</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5538,7 +5733,7 @@
         <v>195</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5555,7 +5750,7 @@
         <v>195</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5572,7 +5767,7 @@
         <v>195</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5589,7 +5784,7 @@
         <v>195</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5606,7 +5801,7 @@
         <v>195</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5623,7 +5818,7 @@
         <v>195</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5640,7 +5835,7 @@
         <v>195</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5657,7 +5852,7 @@
         <v>195</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5674,7 +5869,7 @@
         <v>195</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5691,7 +5886,7 @@
         <v>195</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5708,7 +5903,7 @@
         <v>195</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5725,7 +5920,7 @@
         <v>195</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5742,7 +5937,7 @@
         <v>195</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5759,7 +5954,7 @@
         <v>195</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5776,7 +5971,7 @@
         <v>195</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5793,7 +5988,7 @@
         <v>195</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5810,7 +6005,7 @@
         <v>195</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5827,7 +6022,7 @@
         <v>195</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5844,7 +6039,7 @@
         <v>195</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5861,7 +6056,7 @@
         <v>195</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5878,7 +6073,7 @@
         <v>195</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5895,7 +6090,7 @@
         <v>195</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5912,7 +6107,7 @@
         <v>195</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5929,7 +6124,7 @@
         <v>195</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5946,7 +6141,7 @@
         <v>195</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5963,7 +6158,7 @@
         <v>195</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5980,7 +6175,7 @@
         <v>195</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5997,7 +6192,7 @@
         <v>195</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6014,7 +6209,7 @@
         <v>195</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6031,7 +6226,7 @@
         <v>195</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6048,7 +6243,7 @@
         <v>195</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6065,7 +6260,7 @@
         <v>195</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6082,7 +6277,7 @@
         <v>195</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6099,7 +6294,7 @@
         <v>195</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6116,7 +6311,7 @@
         <v>195</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6133,7 +6328,7 @@
         <v>195</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6150,7 +6345,7 @@
         <v>195</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6167,7 +6362,7 @@
         <v>195</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6184,7 +6379,7 @@
         <v>195</v>
       </c>
       <c r="E137" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6201,7 +6396,7 @@
         <v>195</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6218,7 +6413,7 @@
         <v>195</v>
       </c>
       <c r="E139" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6235,7 +6430,7 @@
         <v>195</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6252,7 +6447,7 @@
         <v>195</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6269,7 +6464,7 @@
         <v>195</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6286,7 +6481,7 @@
         <v>195</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6303,7 +6498,7 @@
         <v>195</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6320,7 +6515,7 @@
         <v>195</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6337,7 +6532,7 @@
         <v>195</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6354,7 +6549,7 @@
         <v>195</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6371,7 +6566,7 @@
         <v>195</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6388,7 +6583,7 @@
         <v>195</v>
       </c>
       <c r="E149" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6405,7 +6600,7 @@
         <v>195</v>
       </c>
       <c r="E150" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6422,7 +6617,7 @@
         <v>195</v>
       </c>
       <c r="E151" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6439,7 +6634,7 @@
         <v>195</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6456,7 +6651,7 @@
         <v>195</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6473,7 +6668,7 @@
         <v>195</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6490,7 +6685,7 @@
         <v>195</v>
       </c>
       <c r="E155" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6507,7 +6702,7 @@
         <v>195</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6524,7 +6719,7 @@
         <v>195</v>
       </c>
       <c r="E157" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6541,7 +6736,7 @@
         <v>195</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6558,7 +6753,7 @@
         <v>195</v>
       </c>
       <c r="E159" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6575,7 +6770,7 @@
         <v>195</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6592,7 +6787,7 @@
         <v>195</v>
       </c>
       <c r="E161" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6609,7 +6804,7 @@
         <v>195</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6626,12 +6821,522 @@
         <v>195</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>355</v>
+        <v>196</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="17" t="s">
+        <v>545</v>
+      </c>
+      <c r="B164" s="20" t="s">
+        <v>546</v>
+      </c>
+      <c r="C164" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D164" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E164" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="17" t="s">
+        <v>548</v>
+      </c>
+      <c r="B165" s="20" t="s">
+        <v>549</v>
+      </c>
+      <c r="C165" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D165" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E165" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="B166" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="C166" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D166" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E166" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="17" t="s">
+        <v>552</v>
+      </c>
+      <c r="B167" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="C167" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D167" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E167" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="17" t="s">
+        <v>554</v>
+      </c>
+      <c r="B168" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="C168" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D168" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E168" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="17" t="s">
+        <v>556</v>
+      </c>
+      <c r="B169" s="20" t="s">
+        <v>557</v>
+      </c>
+      <c r="C169" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D169" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E169" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="B170" s="20" t="s">
+        <v>559</v>
+      </c>
+      <c r="C170" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D170" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E170" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="17" t="s">
+        <v>561</v>
+      </c>
+      <c r="B171" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="C171" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D171" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E171" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="17" t="s">
+        <v>563</v>
+      </c>
+      <c r="B172" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="C172" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D172" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E172" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="17" t="s">
+        <v>565</v>
+      </c>
+      <c r="B173" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="C173" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D173" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E173" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="17" t="s">
+        <v>567</v>
+      </c>
+      <c r="B174" s="20" t="s">
+        <v>568</v>
+      </c>
+      <c r="C174" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D174" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E174" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="17" t="s">
+        <v>569</v>
+      </c>
+      <c r="B175" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="C175" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D175" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E175" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="B176" s="20" t="s">
+        <v>572</v>
+      </c>
+      <c r="C176" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="D176" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E176" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="B177" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="C177" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="D177" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E177" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="17" t="s">
+        <v>576</v>
+      </c>
+      <c r="B178" s="20" t="s">
+        <v>577</v>
+      </c>
+      <c r="C178" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="D178" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E178" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="17" t="s">
+        <v>578</v>
+      </c>
+      <c r="B179" s="20" t="s">
+        <v>579</v>
+      </c>
+      <c r="C179" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="D179" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E179" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="17" t="s">
+        <v>580</v>
+      </c>
+      <c r="B180" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="C180" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="D180" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E180" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="17" t="s">
+        <v>582</v>
+      </c>
+      <c r="B181" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="C181" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="D181" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E181" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="17" t="s">
+        <v>584</v>
+      </c>
+      <c r="B182" s="20" t="s">
+        <v>585</v>
+      </c>
+      <c r="C182" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="D182" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E182" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="17" t="s">
+        <v>587</v>
+      </c>
+      <c r="B183" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="C183" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="D183" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E183" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="17" t="s">
+        <v>589</v>
+      </c>
+      <c r="B184" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="C184" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="D184" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E184" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="17" t="s">
+        <v>591</v>
+      </c>
+      <c r="B185" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="C185" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="D185" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E185" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="B186" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="C186" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="D186" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E186" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="17" t="s">
+        <v>595</v>
+      </c>
+      <c r="B187" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="C187" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="D187" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E187" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="17" t="s">
+        <v>597</v>
+      </c>
+      <c r="B188" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="C188" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="D188" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E188" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="17" t="s">
+        <v>600</v>
+      </c>
+      <c r="B189" s="20" t="s">
+        <v>601</v>
+      </c>
+      <c r="C189" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="D189" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E189" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="17" t="s">
+        <v>602</v>
+      </c>
+      <c r="B190" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="C190" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="D190" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E190" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="17" t="s">
+        <v>604</v>
+      </c>
+      <c r="B191" s="20" t="s">
+        <v>605</v>
+      </c>
+      <c r="C191" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="D191" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E191" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="17" t="s">
+        <v>606</v>
+      </c>
+      <c r="B192" s="20" t="s">
+        <v>607</v>
+      </c>
+      <c r="C192" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="D192" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E192" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="17" t="s">
+        <v>608</v>
+      </c>
+      <c r="B193" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="C193" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="D193" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E193" s="6" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E163" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E193" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
changed few test cases ID
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="482">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -146,22 +146,22 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_APB</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_KOTAK</t>
+    <t xml:space="preserve">test_sa_100_102_225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_124</t>
+    <t xml:space="preserve">test_sa_100_102_226</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_227</t>
   </si>
   <si>
     <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_KOTAK_ATOS</t>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_QR_Generation</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_152</t>
+    <t xml:space="preserve">test_sa_100_102_228</t>
   </si>
   <si>
     <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
@@ -179,13 +179,13 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_153</t>
+    <t xml:space="preserve">test_sa_100_102_229</t>
   </si>
   <si>
     <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_SA_CheckStatus_KOTAK</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_155</t>
+    <t xml:space="preserve">test_sa_100_102_230</t>
   </si>
   <si>
     <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_SA_CheckStatus_After_Expiry_KOTAK_ATOS</t>
@@ -950,514 +950,520 @@
     <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTH_REFUNDED_via_API_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Disabled_APB</t>
   </si>
   <si>
+    <t xml:space="preserve">test_common_100_102_231</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_API_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_232</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_API_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_233</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Callback_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_Kotak_Atos_Callback_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_234</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_2_Success_Callback_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_235</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_AUTHORIZED_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_Kotak_Atos_UPG_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_236</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_amount_mismatch_Via_BQRV4_UPI_Success_Callback_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_HDFC_TID_Dep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_two_times_successful_partial_refund_via_api_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_132</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_APB_Amount_Mismatch_Upon_Check_Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_134</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_HDFC_Amount_Mismatch_Upon_Check_Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_135</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_AXIS_DIRECT_Amount_Mismatch_Upon_Check_Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_136</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_HDFC_Amount_Mismatch_Upon_Check_Status_Tid_Dep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_137</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_two_times_successful_partial_refund_via_api_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_HDFC</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_100_101_122</t>
   </si>
   <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_API_CheckStatus_KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
+    <t xml:space="preserve">UI_Common_PM_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_APB_Partial_Refund</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_123</t>
   </si>
   <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_API_CheckStatus_KOTAK</t>
+    <t xml:space="preserve">UI_Common_PM_UPI_two_times_successful_partial_refund_via_api_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_APB</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_125</t>
   </si>
   <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Callback_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_Kotak_Atos_Callback_01</t>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_APB</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_126</t>
   </si>
   <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_2_Success_Callback_KOTAK_ATOS</t>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_Auto_Refund_Enabled_TID_Dep_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_Callback_TidDep_04</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_127</t>
   </si>
   <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_AUTHORIZED_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_Kotak_Atos_UPG_01</t>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_Auto_Refund_Enabled_TID_Dep_HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_128</t>
   </si>
   <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_amount_mismatch_Via_BQRV4_UPI_Success_Callback_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_HDFC_TID_Dep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_130</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_two_times_successful_partial_refund_via_api_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_132</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_133</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_APB_Amount_Mismatch_Upon_Check_Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_134</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_HDFC_Amount_Mismatch_Upon_Check_Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_135</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_AXIS_DIRECT_Amount_Mismatch_Upon_Check_Status</t>
+    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Pure_UPI_Callback_Auto_Refund_Enabled_TID_Dep_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_237</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Callback_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_Callback_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_2_Success_Callback_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_UPG_AUTHORIZED_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_UPG_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_amount_mismatch_Via_BQRV4_BQR_Success_Callback_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_241</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_API_CheckStatus_KOTAK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_242</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_API_CheckStatus_KOTAK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_243</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Check_Status_via_API_After_Expiry_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_244</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Callback_After_QR_Expiry_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_245</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Pending_Via_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_Pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_246</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_ICICI_FDC_CheckStatus_TID_Dep_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_151</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Via_BQRV4_UPI_Callback_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_ICICI_FDC_Callback_Tid_Dep_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_152</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_ICICI_FDC_CheckStatus_TID_Dep_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_153</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Via_BQRV4_BQR_Callback_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_ICICI_FDC_Callback_Tid_Dep_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_154</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Failed_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_ICICI_FDC_QR_Generation_Success_TID_Dep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_ICICI_FDC_QR_Generation_TID_Dep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_156</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_ICICI_FDC_QR_Generation_Failed_TID_Dep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_157</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Pending_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_158</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_CheckStatus_Via_API_After_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_159</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_1_BQR_1_UPI_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_1_UPI_1_BQR_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_163</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_2_BQR_Success_Callback_Before_QR_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_164</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_2_UPI_Success_Callback_Before_QR_Expiry_TID_Dep_ICICI_FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_165</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_167</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Ref_ID_Val_Via_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AxisDirect_Ref_ID_Val_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_168</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_using_UPI_Success_Callback_Via_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Callback_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_169</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Failed_using_UPI_Failed_Callback_Via_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_170</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_success_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_failed_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_172</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_173</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Partial_Refund_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_175</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_two_times_successful_partial_refund_via_api_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_176</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_PartialRefund_In_Decimal_via_api_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_2_success_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Callback_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_full_Refund_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Refund_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Refund_Failed_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Refund_Posted_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_1_UPI_AXIS_DIRECT_and_1_UPI_HDFC_success_callback_after_qr_expiry_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_1_UPI_AXIS_DIRECT_and_1_BQR_HDFC_success_callback_after_qr_expiry_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_213</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_AUTHORIZED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_UPG_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_214</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_FAILED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_REFUND_PENDING_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_216</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Refund_UPG_AUTHORIZED_via_API_when_UPGRefund_&amp;_UPGAutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_amount_mismatch_Via_UPI_Success_Callback_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_218</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Failed_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Check_Status_via_API_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Amount_Mismatch_Upon_Check_Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_223</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Pending_Via_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_2_failed_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
   </si>
   <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_136</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_HDFC_Amount_Mismatch_Upon_Check_Status_Tid_Dep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_137</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_138</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_two_times_successful_partial_refund_via_api_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_140</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_APB_Partial_Refund</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_141</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_two_times_successful_partial_refund_via_api_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_142</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_In_Decimal_via_api_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_143</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_144</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_Auto_Refund_Enabled_TID_Dep_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_Callback_TidDep_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_145</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_Auto_Refund_Enabled_TID_Dep_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_146</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Pure_UPI_Callback_Auto_Refund_Enabled_TID_Dep_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Callback_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_Callback_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_148</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_2_Success_Callback_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_149</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_UPG_AUTHORIZED_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_UPG_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_amount_mismatch_Via_BQRV4_BQR_Success_Callback_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_151</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_API_CheckStatus_KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_154</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_API_CheckStatus_KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_156</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Check_Status_via_API_After_Expiry_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_157</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Callback_After_QR_Expiry_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Pending_Via_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_Kotak_Atos_Pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_ICICI_FDC_CheckStatus_TID_Dep_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_151</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Via_BQRV4_UPI_Callback_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_ICICI_FDC_Callback_Tid_Dep_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_152</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_ICICI_FDC_CheckStatus_TID_Dep_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_153</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Via_BQRV4_BQR_Callback_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_BQR_ICICI_FDC_Callback_Tid_Dep_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_154</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Failed_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_155</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_ICICI_FDC_QR_Generation_Success_TID_Dep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_ICICI_FDC_QR_Generation_TID_Dep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_156</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_ICICI_FDC_QR_Generation_Failed_TID_Dep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_157</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Pending_Via_CheckStatus_API_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_CheckStatus_Via_API_After_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_BQR_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_160</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_1_BQR_1_UPI_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_161</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_162</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_1_UPI_1_BQR_Success_Callback_After_QR_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_163</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_2_BQR_Success_Callback_Before_QR_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_164</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_2_UPI_Success_Callback_Before_QR_Expiry_TID_Dep_ICICI_FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_165</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_167</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Ref_ID_Val_Via_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AxisDirect_Ref_ID_Val_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_168</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Success_using_UPI_Success_Callback_Via_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Callback_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_169</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Failed_using_UPI_Failed_Callback_Via_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_170</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_success_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_failed_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_172</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_173</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Partial_Refund_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_174</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_two_times_partial_refund_via_api_amount_greater_than_original_amount_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_175</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_two_times_successful_partial_refund_via_api_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_176</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_PartialRefund_In_Decimal_via_api_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_177</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_2_success_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Callback_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_178</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_full_Refund_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Refund_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_179</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Refund_Failed_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_180</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Refund_Posted_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_211</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_1_UPI_AXIS_DIRECT_and_1_UPI_HDFC_success_callback_after_qr_expiry_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_212</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_1_UPI_AXIS_DIRECT_and_1_BQR_HDFC_success_callback_after_qr_expiry_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_213</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_AUTHORIZED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_UPG_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_214</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_FAILED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_215</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_UPG_REFUND_PENDING_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_216</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Refund_UPG_AUTHORIZED_via_API_when_UPGRefund_&amp;_UPGAutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_217</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_amount_mismatch_Via_UPI_Success_Callback_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_218</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Failed_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_220</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Check_Status_via_API_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_222</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Amount_Mismatch_Upon_Check_Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_223</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_UPI_Pending_Via_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_BQRV4_UPI_AXIS_DIRECT_Pending</t>
   </si>
   <si>
     <t xml:space="preserve">test_API_SA_PreFetch_01</t>
@@ -2028,7 +2034,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>39</v>
       </c>
@@ -2233,7 +2239,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="23.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2266,7 +2272,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="23.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2298,7 +2304,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr defaultColWidth="14.83984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="41.68"/>
@@ -4343,15 +4349,15 @@
         <v>67</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>336</v>
+        <v>9</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B121" s="7" t="s">
         <v>337</v>
-      </c>
-      <c r="B121" s="7" t="s">
-        <v>338</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>262</v>
@@ -4365,10 +4371,10 @@
     </row>
     <row r="122" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B122" s="7" t="s">
         <v>339</v>
-      </c>
-      <c r="B122" s="7" t="s">
-        <v>340</v>
       </c>
       <c r="C122" s="7" t="s">
         <v>75</v>
@@ -4382,10 +4388,10 @@
     </row>
     <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="B123" s="7" t="s">
         <v>341</v>
-      </c>
-      <c r="B123" s="7" t="s">
-        <v>342</v>
       </c>
       <c r="C123" s="7" t="s">
         <v>75</v>
@@ -4399,10 +4405,10 @@
     </row>
     <row r="124" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B124" s="7" t="s">
         <v>343</v>
-      </c>
-      <c r="B124" s="7" t="s">
-        <v>344</v>
       </c>
       <c r="C124" s="7" t="s">
         <v>75</v>
@@ -4416,13 +4422,13 @@
     </row>
     <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="B125" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="B125" s="7" t="s">
+      <c r="C125" s="7" t="s">
         <v>346</v>
-      </c>
-      <c r="C125" s="7" t="s">
-        <v>347</v>
       </c>
       <c r="D125" s="13" t="s">
         <v>67</v>
@@ -4433,13 +4439,13 @@
     </row>
     <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B126" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="B126" s="7" t="s">
-        <v>349</v>
-      </c>
       <c r="C126" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D126" s="13" t="s">
         <v>67</v>
@@ -4450,13 +4456,13 @@
     </row>
     <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B127" s="7" t="s">
         <v>350</v>
       </c>
-      <c r="B127" s="7" t="s">
-        <v>351</v>
-      </c>
       <c r="C127" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D127" s="13" t="s">
         <v>67</v>
@@ -4467,13 +4473,13 @@
     </row>
     <row r="128" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B128" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="B128" s="7" t="s">
-        <v>353</v>
-      </c>
       <c r="C128" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D128" s="13" t="s">
         <v>67</v>
@@ -4484,13 +4490,13 @@
     </row>
     <row r="129" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="B129" s="7" t="s">
         <v>354</v>
       </c>
-      <c r="B129" s="7" t="s">
+      <c r="C129" s="7" t="s">
         <v>355</v>
-      </c>
-      <c r="C129" s="7" t="s">
-        <v>356</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>67</v>
@@ -4501,13 +4507,13 @@
     </row>
     <row r="130" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="B130" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="B130" s="7" t="s">
-        <v>358</v>
-      </c>
       <c r="C130" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D130" s="13" t="s">
         <v>67</v>
@@ -4518,13 +4524,13 @@
     </row>
     <row r="131" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B131" s="7" t="s">
         <v>359</v>
       </c>
-      <c r="B131" s="7" t="s">
-        <v>360</v>
-      </c>
       <c r="C131" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D131" s="13" t="s">
         <v>67</v>
@@ -4535,13 +4541,13 @@
     </row>
     <row r="132" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B132" s="7" t="s">
         <v>361</v>
       </c>
-      <c r="B132" s="7" t="s">
+      <c r="C132" s="7" t="s">
         <v>362</v>
-      </c>
-      <c r="C132" s="7" t="s">
-        <v>363</v>
       </c>
       <c r="D132" s="13" t="s">
         <v>67</v>
@@ -4552,13 +4558,13 @@
     </row>
     <row r="133" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="B133" s="7" t="s">
         <v>364</v>
       </c>
-      <c r="B133" s="7" t="s">
-        <v>365</v>
-      </c>
       <c r="C133" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D133" s="13" t="s">
         <v>67</v>
@@ -4569,13 +4575,13 @@
     </row>
     <row r="134" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="B134" s="7" t="s">
         <v>366</v>
       </c>
-      <c r="B134" s="7" t="s">
+      <c r="C134" s="7" t="s">
         <v>367</v>
-      </c>
-      <c r="C134" s="7" t="s">
-        <v>368</v>
       </c>
       <c r="D134" s="13" t="s">
         <v>67</v>
@@ -4586,13 +4592,13 @@
     </row>
     <row r="135" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="B135" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="B135" s="7" t="s">
-        <v>370</v>
-      </c>
       <c r="C135" s="7" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D135" s="13" t="s">
         <v>67</v>
@@ -4603,13 +4609,13 @@
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="B136" s="7" t="s">
         <v>371</v>
       </c>
-      <c r="B136" s="7" t="s">
+      <c r="C136" s="7" t="s">
         <v>372</v>
-      </c>
-      <c r="C136" s="7" t="s">
-        <v>373</v>
       </c>
       <c r="D136" s="13" t="s">
         <v>67</v>
@@ -4620,13 +4626,13 @@
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="B137" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="B137" s="7" t="s">
-        <v>375</v>
-      </c>
       <c r="C137" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D137" s="13" t="s">
         <v>67</v>
@@ -4637,13 +4643,13 @@
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="B138" s="7" t="s">
         <v>376</v>
       </c>
-      <c r="B138" s="7" t="s">
-        <v>377</v>
-      </c>
       <c r="C138" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D138" s="13" t="s">
         <v>67</v>
@@ -4654,13 +4660,13 @@
     </row>
     <row r="139" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="B139" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="B139" s="7" t="s">
-        <v>379</v>
-      </c>
       <c r="C139" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D139" s="13" t="s">
         <v>67</v>
@@ -4671,13 +4677,13 @@
     </row>
     <row r="140" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="B140" s="7" t="s">
         <v>380</v>
       </c>
-      <c r="B140" s="7" t="s">
+      <c r="C140" s="7" t="s">
         <v>381</v>
-      </c>
-      <c r="C140" s="7" t="s">
-        <v>382</v>
       </c>
       <c r="D140" s="13" t="s">
         <v>67</v>
@@ -4688,13 +4694,13 @@
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="B141" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="B141" s="7" t="s">
+      <c r="C141" s="7" t="s">
         <v>384</v>
-      </c>
-      <c r="C141" s="7" t="s">
-        <v>385</v>
       </c>
       <c r="D141" s="13" t="s">
         <v>67</v>
@@ -4705,13 +4711,13 @@
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="B142" s="7" t="s">
         <v>386</v>
       </c>
-      <c r="B142" s="7" t="s">
+      <c r="C142" s="7" t="s">
         <v>387</v>
-      </c>
-      <c r="C142" s="7" t="s">
-        <v>388</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>67</v>
@@ -4722,13 +4728,13 @@
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B143" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="B143" s="7" t="s">
+      <c r="C143" s="7" t="s">
         <v>390</v>
-      </c>
-      <c r="C143" s="7" t="s">
-        <v>391</v>
       </c>
       <c r="D143" s="13" t="s">
         <v>67</v>
@@ -4739,13 +4745,13 @@
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B144" s="7" t="s">
         <v>392</v>
       </c>
-      <c r="B144" s="7" t="s">
+      <c r="C144" s="7" t="s">
         <v>393</v>
-      </c>
-      <c r="C144" s="7" t="s">
-        <v>394</v>
       </c>
       <c r="D144" s="13" t="s">
         <v>67</v>
@@ -4756,13 +4762,13 @@
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="B145" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B145" s="7" t="s">
-        <v>396</v>
-      </c>
       <c r="C145" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D145" s="13" t="s">
         <v>67</v>
@@ -4773,13 +4779,13 @@
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="B146" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="B146" s="7" t="s">
+      <c r="C146" s="7" t="s">
         <v>398</v>
-      </c>
-      <c r="C146" s="7" t="s">
-        <v>399</v>
       </c>
       <c r="D146" s="13" t="s">
         <v>67</v>
@@ -4790,13 +4796,13 @@
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="B147" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="B147" s="7" t="s">
-        <v>401</v>
-      </c>
       <c r="C147" s="7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D147" s="13" t="s">
         <v>67</v>
@@ -4807,13 +4813,13 @@
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="B148" s="7" t="s">
         <v>402</v>
       </c>
-      <c r="B148" s="7" t="s">
-        <v>403</v>
-      </c>
       <c r="C148" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D148" s="13" t="s">
         <v>67</v>
@@ -4824,13 +4830,13 @@
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="B149" s="7" t="s">
         <v>404</v>
       </c>
-      <c r="B149" s="7" t="s">
-        <v>405</v>
-      </c>
       <c r="C149" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D149" s="13" t="s">
         <v>67</v>
@@ -4841,13 +4847,13 @@
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="B150" s="7" t="s">
         <v>406</v>
       </c>
-      <c r="B150" s="7" t="s">
-        <v>407</v>
-      </c>
       <c r="C150" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D150" s="13" t="s">
         <v>67</v>
@@ -4858,13 +4864,13 @@
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="B151" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="B151" s="7" t="s">
-        <v>409</v>
-      </c>
       <c r="C151" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D151" s="13" t="s">
         <v>67</v>
@@ -4875,13 +4881,13 @@
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="B152" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="B152" s="7" t="s">
-        <v>411</v>
-      </c>
       <c r="C152" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D152" s="13" t="s">
         <v>67</v>
@@ -4892,13 +4898,13 @@
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="B153" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="B153" s="7" t="s">
-        <v>413</v>
-      </c>
       <c r="C153" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D153" s="13" t="s">
         <v>67</v>
@@ -4909,13 +4915,13 @@
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="B154" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="B154" s="7" t="s">
-        <v>415</v>
-      </c>
       <c r="C154" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D154" s="13" t="s">
         <v>67</v>
@@ -4926,13 +4932,13 @@
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="B155" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="B155" s="7" t="s">
-        <v>417</v>
-      </c>
       <c r="C155" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D155" s="13" t="s">
         <v>67</v>
@@ -4943,13 +4949,13 @@
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="B156" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="B156" s="7" t="s">
+      <c r="C156" s="7" t="s">
         <v>419</v>
-      </c>
-      <c r="C156" s="7" t="s">
-        <v>420</v>
       </c>
       <c r="D156" s="13" t="s">
         <v>67</v>
@@ -4960,13 +4966,13 @@
     </row>
     <row r="157" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="B157" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="B157" s="7" t="s">
+      <c r="C157" s="7" t="s">
         <v>422</v>
-      </c>
-      <c r="C157" s="7" t="s">
-        <v>423</v>
       </c>
       <c r="D157" s="13" t="s">
         <v>67</v>
@@ -4977,13 +4983,13 @@
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="B158" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="B158" s="7" t="s">
+      <c r="C158" s="7" t="s">
         <v>425</v>
-      </c>
-      <c r="C158" s="7" t="s">
-        <v>426</v>
       </c>
       <c r="D158" s="13" t="s">
         <v>67</v>
@@ -4994,13 +5000,13 @@
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="B159" s="7" t="s">
         <v>427</v>
       </c>
-      <c r="B159" s="7" t="s">
-        <v>428</v>
-      </c>
       <c r="C159" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D159" s="13" t="s">
         <v>67</v>
@@ -5011,13 +5017,13 @@
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="B160" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="B160" s="7" t="s">
-        <v>430</v>
-      </c>
       <c r="C160" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D160" s="13" t="s">
         <v>67</v>
@@ -5028,13 +5034,13 @@
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B161" s="7" t="s">
         <v>431</v>
       </c>
-      <c r="B161" s="7" t="s">
-        <v>432</v>
-      </c>
       <c r="C161" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D161" s="13" t="s">
         <v>67</v>
@@ -5045,13 +5051,13 @@
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="B162" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="B162" s="7" t="s">
-        <v>434</v>
-      </c>
       <c r="C162" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D162" s="13" t="s">
         <v>67</v>
@@ -5062,13 +5068,13 @@
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B163" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="C163" s="7" t="s">
         <v>435</v>
-      </c>
-      <c r="B163" s="7" t="s">
-        <v>434</v>
-      </c>
-      <c r="C163" s="7" t="s">
-        <v>436</v>
       </c>
       <c r="D163" s="13" t="s">
         <v>67</v>
@@ -5079,13 +5085,13 @@
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="B164" s="7" t="s">
         <v>437</v>
       </c>
-      <c r="B164" s="7" t="s">
-        <v>438</v>
-      </c>
       <c r="C164" s="7" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D164" s="13" t="s">
         <v>67</v>
@@ -5096,13 +5102,13 @@
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="B165" s="7" t="s">
         <v>439</v>
       </c>
-      <c r="B165" s="7" t="s">
-        <v>440</v>
-      </c>
       <c r="C165" s="7" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D165" s="13" t="s">
         <v>67</v>
@@ -5113,13 +5119,13 @@
     </row>
     <row r="166" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="B166" s="7" t="s">
         <v>441</v>
       </c>
-      <c r="B166" s="7" t="s">
-        <v>442</v>
-      </c>
       <c r="C166" s="7" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D166" s="13" t="s">
         <v>67</v>
@@ -5130,47 +5136,47 @@
     </row>
     <row r="167" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="B167" s="7" t="s">
         <v>443</v>
       </c>
-      <c r="B167" s="7" t="s">
+      <c r="C167" s="7" t="s">
         <v>444</v>
       </c>
-      <c r="C167" s="7" t="s">
+      <c r="D167" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E167" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="7" t="s">
         <v>445</v>
       </c>
-      <c r="D167" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E167" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="168" customFormat="false" ht="28.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="7" t="s">
+      <c r="B168" s="7" t="s">
         <v>446</v>
       </c>
-      <c r="B168" s="7" t="s">
+      <c r="C168" s="7" t="s">
         <v>447</v>
       </c>
-      <c r="C168" s="7" t="s">
+      <c r="D168" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E168" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="7" t="s">
         <v>448</v>
       </c>
-      <c r="D168" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E168" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="169" customFormat="false" ht="28.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="7" t="s">
+      <c r="B169" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="B169" s="7" t="s">
-        <v>450</v>
-      </c>
       <c r="C169" s="7" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D169" s="13" t="s">
         <v>67</v>
@@ -5181,13 +5187,13 @@
     </row>
     <row r="170" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="B170" s="7" t="s">
         <v>451</v>
       </c>
-      <c r="B170" s="7" t="s">
-        <v>452</v>
-      </c>
       <c r="C170" s="7" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D170" s="13" t="s">
         <v>67</v>
@@ -5198,13 +5204,13 @@
     </row>
     <row r="171" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="B171" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="B171" s="7" t="s">
-        <v>454</v>
-      </c>
       <c r="C171" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D171" s="13" t="s">
         <v>67</v>
@@ -5215,13 +5221,13 @@
     </row>
     <row r="172" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="B172" s="7" t="s">
         <v>455</v>
       </c>
-      <c r="B172" s="7" t="s">
-        <v>456</v>
-      </c>
       <c r="C172" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D172" s="13" t="s">
         <v>67</v>
@@ -5232,13 +5238,13 @@
     </row>
     <row r="173" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="B173" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="B173" s="7" t="s">
+      <c r="C173" s="7" t="s">
         <v>458</v>
-      </c>
-      <c r="C173" s="7" t="s">
-        <v>459</v>
       </c>
       <c r="D173" s="13" t="s">
         <v>67</v>
@@ -5249,13 +5255,13 @@
     </row>
     <row r="174" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="B174" s="7" t="s">
         <v>460</v>
       </c>
-      <c r="B174" s="7" t="s">
-        <v>461</v>
-      </c>
       <c r="C174" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D174" s="13" t="s">
         <v>67</v>
@@ -5266,13 +5272,13 @@
     </row>
     <row r="175" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="B175" s="7" t="s">
         <v>462</v>
       </c>
-      <c r="B175" s="7" t="s">
-        <v>463</v>
-      </c>
       <c r="C175" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D175" s="13" t="s">
         <v>67</v>
@@ -5283,13 +5289,13 @@
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="B176" s="7" t="s">
         <v>464</v>
       </c>
-      <c r="B176" s="7" t="s">
-        <v>465</v>
-      </c>
       <c r="C176" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D176" s="13" t="s">
         <v>67</v>
@@ -5300,13 +5306,13 @@
     </row>
     <row r="177" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="B177" s="7" t="s">
         <v>466</v>
       </c>
-      <c r="B177" s="7" t="s">
-        <v>467</v>
-      </c>
       <c r="C177" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D177" s="13" t="s">
         <v>67</v>
@@ -5317,13 +5323,13 @@
     </row>
     <row r="178" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="B178" s="7" t="s">
         <v>468</v>
       </c>
-      <c r="B178" s="7" t="s">
-        <v>469</v>
-      </c>
       <c r="C178" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D178" s="13" t="s">
         <v>67</v>
@@ -5334,13 +5340,13 @@
     </row>
     <row r="179" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="B179" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="B179" s="7" t="s">
-        <v>471</v>
-      </c>
       <c r="C179" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D179" s="13" t="s">
         <v>67</v>
@@ -5351,13 +5357,13 @@
     </row>
     <row r="180" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="B180" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="B180" s="7" t="s">
-        <v>473</v>
-      </c>
       <c r="C180" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D180" s="13" t="s">
         <v>67</v>
@@ -5368,24 +5374,41 @@
     </row>
     <row r="181" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="B181" s="7" t="s">
         <v>474</v>
       </c>
-      <c r="B181" s="7" t="s">
+      <c r="C181" s="7" t="s">
         <v>475</v>
       </c>
-      <c r="C181" s="7" t="s">
+      <c r="D181" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E181" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="D181" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E181" s="6" t="s">
-        <v>9</v>
+      <c r="B182" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="C182" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="D182" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E182" s="6" t="s">
+        <v>478</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E181" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E182" type="list">
       <formula1>"True,False"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5406,7 +5429,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="23.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="23.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="16" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="16" width="25.4"/>
@@ -5429,13 +5452,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="D2" s="19" t="s">
         <v>9</v>
@@ -5464,7 +5487,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="23.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5497,7 +5520,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="23.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5530,7 +5553,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="23.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">

</xml_diff>

<commit_message>
added detailed validation in few of the HDFC and AXIS_DIRECT test cases
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -60,463 +60,463 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
+    <t xml:space="preserve">False</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_SA_CheckStatus_After_Expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_HDFC_QR_Generation_Success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Expired_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_AXIS_DIRECT_QR_Generation_Success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_APB_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_075</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_084</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_226</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_227</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_QR_Generation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_SA_CheckStatus_KOTAK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_SA_CheckStatus_After_Expiry_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_166</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_221</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_224</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_QR_Generation_Success_via_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_AXIS_DIRECT_QR_Generation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_full_Refund_via-Portal_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_partial_Refund_via-Portal_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_HDFC _08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Expired_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_UPG_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_FAILED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUND_PENDING_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_before_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_partial_Refund_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Partial_Refund_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_CheckStatus_via_API_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Success_Callback_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_failed_Callback_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">False</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_SA_CheckStatus_After_Expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_HDFC_QR_Generation_Success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Expired_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_AXIS_DIRECT_QR_Generation_Success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_068</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_APB_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_069</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_075</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_084</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_225</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_226</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_227</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_QR_Generation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_228</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_229</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_SA_CheckStatus_KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_230</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_SA_CheckStatus_After_Expiry_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_166</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_224</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_QR_Generation_Success_via_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_AXIS_DIRECT_QR_Generation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_full_Refund_via-Portal_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_partial_Refund_via-Portal_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_HDFC _08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Expired_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_UPG_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_FAILED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUND_PENDING_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_before_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_partial_Refund_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Partial_Refund_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_CheckStatus_via_API_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Success_Callback_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_failed_Callback_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_AXIS_DIRECT</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_052</t>
@@ -1516,11 +1516,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1596,6 +1597,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF00627A"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
@@ -1664,7 +1672,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1729,11 +1737,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1825,8 +1841,8 @@
   <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="17.48046875" defaultRowHeight="13.2" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="82.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="69.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="87.38"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="17.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.52"/>
@@ -1881,15 +1897,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -1898,347 +1914,347 @@
         <v>8</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="C19" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="C20" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>57</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C22" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="C23" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>64</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2264,7 +2280,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.24609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.41796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2297,7 +2313,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.24609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.41796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2329,7 +2345,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E187"/>
+  <dimension ref="A1:E188"/>
   <sheetFormatPr defaultColWidth="14.83984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="31.43"/>
@@ -2359,716 +2375,716 @@
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>67</v>
-      </c>
       <c r="D2" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>71</v>
-      </c>
       <c r="D3" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="C4" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>76</v>
-      </c>
       <c r="D5" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="C6" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>81</v>
-      </c>
       <c r="D7" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>84</v>
-      </c>
       <c r="D8" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>86</v>
-      </c>
       <c r="C9" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>88</v>
-      </c>
       <c r="C10" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>90</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="C12" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>94</v>
-      </c>
       <c r="C13" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>96</v>
-      </c>
       <c r="C14" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>98</v>
-      </c>
       <c r="C15" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="C16" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>101</v>
-      </c>
       <c r="D16" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>103</v>
-      </c>
       <c r="C17" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="D18" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>108</v>
-      </c>
       <c r="C19" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>110</v>
-      </c>
       <c r="C20" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>112</v>
-      </c>
       <c r="C21" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="14" t="s">
-        <v>114</v>
-      </c>
       <c r="C22" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="B23" s="14" t="s">
-        <v>116</v>
-      </c>
       <c r="C23" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>118</v>
-      </c>
       <c r="C24" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>120</v>
-      </c>
       <c r="C25" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="C26" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>123</v>
-      </c>
       <c r="D26" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>125</v>
-      </c>
       <c r="C27" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="B28" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="C28" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="B29" s="15" t="s">
-        <v>129</v>
-      </c>
       <c r="C29" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B30" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>131</v>
-      </c>
       <c r="C30" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B31" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>133</v>
-      </c>
       <c r="C31" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="C32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>136</v>
-      </c>
       <c r="D32" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B33" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>138</v>
-      </c>
       <c r="C33" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>140</v>
-      </c>
       <c r="C34" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="C35" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>143</v>
-      </c>
       <c r="D35" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="C36" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C36" s="7" t="s">
-        <v>146</v>
-      </c>
       <c r="D36" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B37" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B37" s="15" t="s">
-        <v>148</v>
-      </c>
       <c r="C37" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="B38" s="15" t="s">
-        <v>150</v>
-      </c>
       <c r="C38" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="15" t="s">
-        <v>152</v>
-      </c>
       <c r="C39" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="B40" s="15" t="s">
+      <c r="C40" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="C40" s="7" t="s">
-        <v>155</v>
-      </c>
       <c r="D40" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B41" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="15" t="s">
-        <v>157</v>
-      </c>
       <c r="C41" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B42" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>159</v>
-      </c>
       <c r="C42" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="C43" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3082,10 +3098,10 @@
         <v>164</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3096,13 +3112,13 @@
         <v>166</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3113,13 +3129,13 @@
         <v>168</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3130,13 +3146,13 @@
         <v>170</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3150,10 +3166,10 @@
         <v>173</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3167,10 +3183,10 @@
         <v>173</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3184,10 +3200,10 @@
         <v>173</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3201,10 +3217,10 @@
         <v>173</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3218,10 +3234,10 @@
         <v>173</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3235,10 +3251,10 @@
         <v>183</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3252,10 +3268,10 @@
         <v>186</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3269,10 +3285,10 @@
         <v>189</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3286,10 +3302,10 @@
         <v>189</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3303,10 +3319,10 @@
         <v>189</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3320,10 +3336,10 @@
         <v>189</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3337,10 +3353,10 @@
         <v>189</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3354,10 +3370,10 @@
         <v>200</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3371,10 +3387,10 @@
         <v>203</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3388,10 +3404,10 @@
         <v>203</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,10 +3421,10 @@
         <v>208</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3422,10 +3438,10 @@
         <v>208</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3439,10 +3455,10 @@
         <v>208</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3456,10 +3472,10 @@
         <v>214</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,10 +3489,10 @@
         <v>214</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3490,10 +3506,10 @@
         <v>214</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3507,10 +3523,10 @@
         <v>214</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3524,10 +3540,10 @@
         <v>214</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3541,10 +3557,10 @@
         <v>225</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3558,10 +3574,10 @@
         <v>225</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,10 +3591,10 @@
         <v>225</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3592,10 +3608,10 @@
         <v>225</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3609,10 +3625,10 @@
         <v>225</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,10 +3642,10 @@
         <v>236</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3643,10 +3659,10 @@
         <v>236</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3660,10 +3676,10 @@
         <v>236</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3677,10 +3693,10 @@
         <v>243</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3694,10 +3710,10 @@
         <v>243</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3711,10 +3727,10 @@
         <v>243</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3728,10 +3744,10 @@
         <v>243</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3745,10 +3761,10 @@
         <v>243</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3762,10 +3778,10 @@
         <v>254</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3779,10 +3795,10 @@
         <v>254</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3796,10 +3812,10 @@
         <v>254</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3813,10 +3829,10 @@
         <v>261</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3830,10 +3846,10 @@
         <v>264</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3847,10 +3863,10 @@
         <v>267</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3864,10 +3880,10 @@
         <v>270</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3881,10 +3897,10 @@
         <v>273</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3898,10 +3914,10 @@
         <v>270</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3915,10 +3931,10 @@
         <v>270</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3932,10 +3948,10 @@
         <v>270</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3949,10 +3965,10 @@
         <v>270</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3966,10 +3982,10 @@
         <v>284</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3983,10 +3999,10 @@
         <v>287</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4000,10 +4016,10 @@
         <v>287</v>
       </c>
       <c r="D98" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4017,10 +4033,10 @@
         <v>261</v>
       </c>
       <c r="D99" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4034,10 +4050,10 @@
         <v>261</v>
       </c>
       <c r="D100" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4051,10 +4067,10 @@
         <v>296</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4068,10 +4084,10 @@
         <v>296</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4085,10 +4101,10 @@
         <v>296</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4102,10 +4118,10 @@
         <v>296</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4119,10 +4135,10 @@
         <v>296</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4136,10 +4152,10 @@
         <v>203</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4153,10 +4169,10 @@
         <v>296</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4170,10 +4186,10 @@
         <v>311</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4187,10 +4203,10 @@
         <v>311</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4204,10 +4220,10 @@
         <v>316</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4221,10 +4237,10 @@
         <v>316</v>
       </c>
       <c r="D111" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4238,10 +4254,10 @@
         <v>321</v>
       </c>
       <c r="D112" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4255,10 +4271,10 @@
         <v>321</v>
       </c>
       <c r="D113" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4272,10 +4288,10 @@
         <v>261</v>
       </c>
       <c r="D114" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4286,13 +4302,13 @@
         <v>327</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4303,13 +4319,13 @@
         <v>329</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4320,13 +4336,13 @@
         <v>331</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4340,10 +4356,10 @@
         <v>208</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4354,13 +4370,13 @@
         <v>335</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4371,13 +4387,13 @@
         <v>337</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D120" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4391,10 +4407,10 @@
         <v>264</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4405,13 +4421,13 @@
         <v>341</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D122" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4422,13 +4438,13 @@
         <v>343</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D123" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4439,13 +4455,13 @@
         <v>345</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4459,10 +4475,10 @@
         <v>348</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4476,10 +4492,10 @@
         <v>348</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4493,10 +4509,10 @@
         <v>348</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4510,10 +4526,10 @@
         <v>348</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4527,10 +4543,10 @@
         <v>357</v>
       </c>
       <c r="D129" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4544,10 +4560,10 @@
         <v>357</v>
       </c>
       <c r="D130" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4561,10 +4577,10 @@
         <v>357</v>
       </c>
       <c r="D131" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4578,10 +4594,10 @@
         <v>364</v>
       </c>
       <c r="D132" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4595,10 +4611,10 @@
         <v>364</v>
       </c>
       <c r="D133" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4612,10 +4628,10 @@
         <v>369</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4629,10 +4645,10 @@
         <v>369</v>
       </c>
       <c r="D135" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4646,10 +4662,10 @@
         <v>374</v>
       </c>
       <c r="D136" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4663,10 +4679,10 @@
         <v>374</v>
       </c>
       <c r="D137" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E137" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4680,10 +4696,10 @@
         <v>374</v>
       </c>
       <c r="D138" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4697,10 +4713,10 @@
         <v>364</v>
       </c>
       <c r="D139" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E139" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4714,10 +4730,10 @@
         <v>383</v>
       </c>
       <c r="D140" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4731,10 +4747,10 @@
         <v>386</v>
       </c>
       <c r="D141" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4748,10 +4764,10 @@
         <v>389</v>
       </c>
       <c r="D142" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4765,10 +4781,10 @@
         <v>392</v>
       </c>
       <c r="D143" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4782,10 +4798,10 @@
         <v>395</v>
       </c>
       <c r="D144" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4799,10 +4815,10 @@
         <v>392</v>
       </c>
       <c r="D145" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4816,10 +4832,10 @@
         <v>400</v>
       </c>
       <c r="D146" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4833,10 +4849,10 @@
         <v>400</v>
       </c>
       <c r="D147" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4850,10 +4866,10 @@
         <v>392</v>
       </c>
       <c r="D148" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4867,10 +4883,10 @@
         <v>392</v>
       </c>
       <c r="D149" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E149" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4884,10 +4900,10 @@
         <v>395</v>
       </c>
       <c r="D150" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E150" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4901,10 +4917,10 @@
         <v>395</v>
       </c>
       <c r="D151" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E151" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4918,10 +4934,10 @@
         <v>389</v>
       </c>
       <c r="D152" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4935,10 +4951,10 @@
         <v>389</v>
       </c>
       <c r="D153" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4952,10 +4968,10 @@
         <v>395</v>
       </c>
       <c r="D154" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4969,10 +4985,10 @@
         <v>389</v>
       </c>
       <c r="D155" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E155" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4986,10 +5002,10 @@
         <v>421</v>
       </c>
       <c r="D156" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5003,10 +5019,10 @@
         <v>424</v>
       </c>
       <c r="D157" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E157" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5020,10 +5036,10 @@
         <v>427</v>
       </c>
       <c r="D158" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5037,10 +5053,10 @@
         <v>427</v>
       </c>
       <c r="D159" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E159" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5054,10 +5070,10 @@
         <v>427</v>
       </c>
       <c r="D160" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5071,10 +5087,10 @@
         <v>427</v>
       </c>
       <c r="D161" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E161" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5088,10 +5104,10 @@
         <v>427</v>
       </c>
       <c r="D162" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5105,10 +5121,10 @@
         <v>437</v>
       </c>
       <c r="D163" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5122,10 +5138,10 @@
         <v>437</v>
       </c>
       <c r="D164" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E164" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5139,10 +5155,10 @@
         <v>437</v>
       </c>
       <c r="D165" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E165" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5156,10 +5172,10 @@
         <v>437</v>
       </c>
       <c r="D166" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E166" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5173,10 +5189,10 @@
         <v>446</v>
       </c>
       <c r="D167" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E167" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5190,10 +5206,10 @@
         <v>449</v>
       </c>
       <c r="D168" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E168" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5207,10 +5223,10 @@
         <v>449</v>
       </c>
       <c r="D169" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E169" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5224,10 +5240,10 @@
         <v>449</v>
       </c>
       <c r="D170" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E170" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5241,10 +5257,10 @@
         <v>446</v>
       </c>
       <c r="D171" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E171" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5258,10 +5274,10 @@
         <v>446</v>
       </c>
       <c r="D172" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5275,10 +5291,10 @@
         <v>460</v>
       </c>
       <c r="D173" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E173" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5292,10 +5308,10 @@
         <v>460</v>
       </c>
       <c r="D174" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E174" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5309,10 +5325,10 @@
         <v>460</v>
       </c>
       <c r="D175" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E175" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5326,10 +5342,10 @@
         <v>460</v>
       </c>
       <c r="D176" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E176" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5343,10 +5359,10 @@
         <v>460</v>
       </c>
       <c r="D177" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E177" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5360,10 +5376,10 @@
         <v>421</v>
       </c>
       <c r="D178" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E178" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5377,10 +5393,10 @@
         <v>421</v>
       </c>
       <c r="D179" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E179" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5394,10 +5410,10 @@
         <v>421</v>
       </c>
       <c r="D180" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E180" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5411,10 +5427,10 @@
         <v>477</v>
       </c>
       <c r="D181" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E181" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5428,10 +5444,10 @@
         <v>446</v>
       </c>
       <c r="D182" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E182" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5445,10 +5461,10 @@
         <v>446</v>
       </c>
       <c r="D183" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5462,10 +5478,10 @@
         <v>446</v>
       </c>
       <c r="D184" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5479,10 +5495,10 @@
         <v>364</v>
       </c>
       <c r="D185" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E185" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5496,10 +5512,10 @@
         <v>316</v>
       </c>
       <c r="D186" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E186" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5513,11 +5529,18 @@
         <v>316</v>
       </c>
       <c r="D187" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>12</v>
-      </c>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="16"/>
+      <c r="B188" s="16"/>
+      <c r="C188" s="16"/>
+      <c r="D188" s="16"/>
+      <c r="E188" s="17"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -5542,11 +5565,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="24.24609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.41796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="16" width="26.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="16" width="25.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="16" width="69.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="18" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="25.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="18" width="69.15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5564,17 +5587,17 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>490</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="20" t="s">
         <v>491</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="20" t="s">
         <v>492</v>
       </c>
-      <c r="D2" s="19" t="s">
-        <v>12</v>
+      <c r="D2" s="21" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -5600,7 +5623,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.24609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.41796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5633,7 +5656,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.24609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.41796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5666,7 +5689,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.24609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.41796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">

</xml_diff>

<commit_message>
added txnlist api instead of txnDetails api
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -60,637 +60,637 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
+    <t xml:space="preserve">False</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_SA_CheckStatus_After_Expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_HDFC_QR_Generation_Success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Expired_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_AXIS_DIRECT_QR_Generation_Success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_APB_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_075</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_084</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_226</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_227</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_QR_Generation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_SA_CheckStatus_KOTAK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_SA_CheckStatus_After_Expiry_KOTAK_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_166</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_221</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_224</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_QR_Generation_Success_via_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_AXIS_DIRECT_QR_Generation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_full_Refund_via-Portal_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_partial_Refund_via-Portal_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_HDFC _08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Expired_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_UPG_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_FAILED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUND_PENDING_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_before_qr_expiry_AutoRefund_Enabled_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_CheckStatus_API_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_partial_Refund_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Partial_Refund_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_CheckStatus_via_API_After_Expiry_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Success_Callback_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_failed_Callback_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_AXIS_DIRECT_AutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_AXIS_DIRECT_AutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Ref_ID_Val_Via_Pure_UPI_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AxisDirect_Ref_ID_Val_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AXIS_DIRECT_UPG_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_FAILED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_066</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Refund_UPG_AUTHORIZED_via_API_when_UPGRefund_&amp;_UPGAutoRefund_Disabled_AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_amount_mismatch_Via_Pure_UPI_Success_Callback_AXISDIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_071</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_REFUND_Failed_via_API_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_072</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Pure_UPI_REFUND_Posted_via_API_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_APB_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_074</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_077</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Success_Callback_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_APB_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Failed_Callback_APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_101_079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Disabled_APB</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">False</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_SA_CheckStatus_After_Expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_HDFC_QR_Generation_Success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Expired_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_AXIS_DIRECT_QR_Generation_Success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_068</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Success_Via_SA_CheckStatus_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_APB_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_069</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_075</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_SA_CheckStatus_After_Expiry_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_101_084</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_UPI_QR_Generation_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_225</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_226</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_227</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_QR_Generation_Success_via_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_Kotak_Atos_QR_Generation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_228</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Success_Via_SA_CheckStatus_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_BQR_Kotak_Atos_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_229</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_Failed_Via_SA_CheckStatus_KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_230</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_BQR_SA_CheckStatus_After_Expiry_KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_166</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Success_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_Failed_Via_SA_CheckStatus_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_UPI_SA_CheckStatus_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_224</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_QR_Generation_Success_via_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_PM_BQRV4_AXIS_DIRECT_QR_Generation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_full_Refund_via-Portal_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_PartialRefund_via_api_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_PartialRefund</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_partial_Refund_via-Portal_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_HDFC_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Callback_HDFC _08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_Expired_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_HDFC_UPG_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_FAILED_VIA_HDFC_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUND_PENDING_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_HDFC_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_before_qr_expiry_AutoRefund_Enabled_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_before_qr_expiry_HDFC_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AXIS_DIRECT_CheckStatus_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Expired_Via_CheckStatus_API_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_full_Refund_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_partial_Refund_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Partial_Refund_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_CheckStatus_via_API_After_Expiry_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Success_Callback_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_failed_Callback_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Failed_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_Refund_Posted_via_API_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_052</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Enabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_failed_callback_after_qr_expiry_AutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_057</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_058</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_failed_callback_after_qr_expiry_AXIS_DIRECT_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_060</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_AXIS_DIRECT_AutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_061</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_2_Pure_UPI_success_callback_before_qr_expiry_AXIS_DIRECT_AutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_AXIS_DIRECT_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_062</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Ref_ID_Val_Via_Pure_UPI_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AxisDirect_Ref_ID_Val_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_063</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_AXIS_DIRECT_UPG_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_064</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_FAILED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_065</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_UPG_AUTHORIZED_via_AXIS_DIRECT_when_UPGRefund_&amp;_UPGAutoRefund_Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_066</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Refund_UPG_AUTHORIZED_via_API_when_UPGRefund_&amp;_UPGAutoRefund_Disabled_AXIS_DIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_067</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_amount_mismatch_Via_Pure_UPI_Success_Callback_AXISDIRECT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_070</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Pure_UPI_Pending_Via_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Pending_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_071</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_REFUND_Failed_via_API_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_072</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Pure_UPI_REFUND_Posted_via_API_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_073</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Success_Via_CheckStatus_API_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Checkstatus_APB_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_074</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_UPI_qr_via_api_Failed_Via_CheckStatus_API_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_076</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_077</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Success_Via_Pure_UPI_Success_Callback_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Callback_APB_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_Failed_Via_Pure_UPI_Failed_Callback_APB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_101_079</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_UPI_success_callback_after_qr_expiry_AutoRefund_Disabled_APB</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_080</t>
@@ -1900,15 +1900,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -1917,347 +1917,347 @@
         <v>8</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="C19" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="C20" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>57</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C22" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="C23" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>64</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2283,7 +2283,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2316,7 +2316,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2378,1141 +2378,1141 @@
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>67</v>
-      </c>
       <c r="D2" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>71</v>
-      </c>
       <c r="D3" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="C4" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>76</v>
-      </c>
       <c r="D5" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="C6" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>81</v>
-      </c>
       <c r="D7" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>84</v>
-      </c>
       <c r="D8" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>86</v>
-      </c>
       <c r="C9" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>88</v>
-      </c>
       <c r="C10" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>90</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="C12" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>94</v>
-      </c>
       <c r="C13" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>96</v>
-      </c>
       <c r="C14" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>98</v>
-      </c>
       <c r="C15" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="C16" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>101</v>
-      </c>
       <c r="D16" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>103</v>
-      </c>
       <c r="C17" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="D18" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>108</v>
-      </c>
       <c r="C19" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>110</v>
-      </c>
       <c r="C20" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>112</v>
-      </c>
       <c r="C21" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="14" t="s">
-        <v>114</v>
-      </c>
       <c r="C22" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="B23" s="14" t="s">
-        <v>116</v>
-      </c>
       <c r="C23" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>118</v>
-      </c>
       <c r="C24" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>120</v>
-      </c>
       <c r="C25" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="C26" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>123</v>
-      </c>
       <c r="D26" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>125</v>
-      </c>
       <c r="C27" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="B28" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="C28" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="B29" s="15" t="s">
-        <v>129</v>
-      </c>
       <c r="C29" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B30" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>131</v>
-      </c>
       <c r="C30" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B31" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>133</v>
-      </c>
       <c r="C31" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="C32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>136</v>
-      </c>
       <c r="D32" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B33" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>138</v>
-      </c>
       <c r="C33" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>140</v>
-      </c>
       <c r="C34" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="C35" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>143</v>
-      </c>
       <c r="D35" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="C36" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C36" s="7" t="s">
-        <v>146</v>
-      </c>
       <c r="D36" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B37" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B37" s="15" t="s">
-        <v>148</v>
-      </c>
       <c r="C37" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="B38" s="15" t="s">
-        <v>150</v>
-      </c>
       <c r="C38" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="15" t="s">
-        <v>152</v>
-      </c>
       <c r="C39" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="B40" s="15" t="s">
+      <c r="C40" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="C40" s="7" t="s">
-        <v>155</v>
-      </c>
       <c r="D40" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B41" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="15" t="s">
-        <v>157</v>
-      </c>
       <c r="C41" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B42" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>159</v>
-      </c>
       <c r="C42" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>161</v>
-      </c>
       <c r="C43" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B44" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="C44" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="C44" s="7" t="s">
-        <v>164</v>
-      </c>
       <c r="D44" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B45" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>166</v>
-      </c>
       <c r="C45" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B46" s="7" t="s">
-        <v>168</v>
-      </c>
       <c r="C46" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="B47" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B47" s="7" t="s">
-        <v>170</v>
-      </c>
       <c r="C47" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B48" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="C48" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="C48" s="7" t="s">
-        <v>173</v>
-      </c>
       <c r="D48" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B49" s="7" t="s">
-        <v>175</v>
-      </c>
       <c r="C49" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B50" s="7" t="s">
-        <v>177</v>
-      </c>
       <c r="C50" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B51" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="B51" s="7" t="s">
-        <v>179</v>
-      </c>
       <c r="C51" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="B52" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="B52" s="7" t="s">
-        <v>181</v>
-      </c>
       <c r="C52" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B53" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="C53" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="C53" s="7" t="s">
-        <v>184</v>
-      </c>
       <c r="D53" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B54" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="C54" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="C54" s="7" t="s">
-        <v>187</v>
-      </c>
       <c r="D54" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="C55" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="C55" s="7" t="s">
-        <v>190</v>
-      </c>
       <c r="D55" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B56" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="B56" s="7" t="s">
-        <v>192</v>
-      </c>
       <c r="C56" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B57" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="C57" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="C57" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="D57" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
+      <c r="B58" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="B58" s="7" t="s">
-        <v>196</v>
-      </c>
       <c r="C58" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B59" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B59" s="7" t="s">
-        <v>198</v>
-      </c>
       <c r="C59" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B60" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="C60" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C60" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="D60" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B61" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="C61" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C61" s="1" t="s">
-        <v>204</v>
-      </c>
       <c r="D61" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="B62" s="7" t="s">
-        <v>206</v>
-      </c>
       <c r="C62" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B63" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="B63" s="7" t="s">
+      <c r="C63" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C63" s="1" t="s">
-        <v>209</v>
-      </c>
       <c r="D63" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B64" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>211</v>
-      </c>
       <c r="C64" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B66" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="C66" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C66" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="D66" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B67" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="B67" s="7" t="s">
-        <v>217</v>
-      </c>
       <c r="C67" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="B68" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="B68" s="7" t="s">
+      <c r="C68" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D68" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E68" s="6" t="s">
         <v>219</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="D68" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3523,13 +3523,13 @@
         <v>221</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3540,13 +3540,13 @@
         <v>223</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3560,10 +3560,10 @@
         <v>226</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3577,10 +3577,10 @@
         <v>226</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3594,10 +3594,10 @@
         <v>226</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3611,10 +3611,10 @@
         <v>226</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3628,10 +3628,10 @@
         <v>226</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3645,10 +3645,10 @@
         <v>237</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3662,10 +3662,10 @@
         <v>237</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3679,10 +3679,10 @@
         <v>237</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3696,10 +3696,10 @@
         <v>244</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3713,10 +3713,10 @@
         <v>244</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3730,10 +3730,10 @@
         <v>244</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3747,10 +3747,10 @@
         <v>244</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3764,10 +3764,10 @@
         <v>244</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3781,10 +3781,10 @@
         <v>255</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3798,10 +3798,10 @@
         <v>255</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3815,10 +3815,10 @@
         <v>255</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3832,10 +3832,10 @@
         <v>262</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3849,10 +3849,10 @@
         <v>265</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3866,10 +3866,10 @@
         <v>268</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3883,10 +3883,10 @@
         <v>271</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3900,10 +3900,10 @@
         <v>274</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3917,10 +3917,10 @@
         <v>271</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3934,10 +3934,10 @@
         <v>271</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3951,10 +3951,10 @@
         <v>271</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3968,10 +3968,10 @@
         <v>271</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3985,10 +3985,10 @@
         <v>285</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4002,10 +4002,10 @@
         <v>288</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4019,10 +4019,10 @@
         <v>288</v>
       </c>
       <c r="D98" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,10 +4036,10 @@
         <v>262</v>
       </c>
       <c r="D99" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4053,10 +4053,10 @@
         <v>262</v>
       </c>
       <c r="D100" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4070,10 +4070,10 @@
         <v>297</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4087,10 +4087,10 @@
         <v>297</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4104,10 +4104,10 @@
         <v>297</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4121,10 +4121,10 @@
         <v>297</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4138,10 +4138,10 @@
         <v>297</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4152,13 +4152,13 @@
         <v>307</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4172,10 +4172,10 @@
         <v>297</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4189,10 +4189,10 @@
         <v>312</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4206,10 +4206,10 @@
         <v>312</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4223,10 +4223,10 @@
         <v>317</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4240,10 +4240,10 @@
         <v>317</v>
       </c>
       <c r="D111" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4257,10 +4257,10 @@
         <v>322</v>
       </c>
       <c r="D112" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4274,10 +4274,10 @@
         <v>322</v>
       </c>
       <c r="D113" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4291,10 +4291,10 @@
         <v>262</v>
       </c>
       <c r="D114" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4305,13 +4305,13 @@
         <v>328</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4322,13 +4322,13 @@
         <v>330</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4339,13 +4339,13 @@
         <v>332</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4356,13 +4356,13 @@
         <v>334</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4373,13 +4373,13 @@
         <v>336</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4390,13 +4390,13 @@
         <v>338</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D120" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4410,10 +4410,10 @@
         <v>265</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4424,13 +4424,13 @@
         <v>342</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D122" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4441,13 +4441,13 @@
         <v>344</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D123" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,13 +4458,13 @@
         <v>346</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4478,10 +4478,10 @@
         <v>349</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4495,10 +4495,10 @@
         <v>349</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4512,10 +4512,10 @@
         <v>349</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4529,10 +4529,10 @@
         <v>349</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4546,10 +4546,10 @@
         <v>358</v>
       </c>
       <c r="D129" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4563,10 +4563,10 @@
         <v>358</v>
       </c>
       <c r="D130" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4580,10 +4580,10 @@
         <v>358</v>
       </c>
       <c r="D131" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4597,10 +4597,10 @@
         <v>365</v>
       </c>
       <c r="D132" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4614,10 +4614,10 @@
         <v>365</v>
       </c>
       <c r="D133" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4631,10 +4631,10 @@
         <v>370</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4648,10 +4648,10 @@
         <v>370</v>
       </c>
       <c r="D135" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4665,10 +4665,10 @@
         <v>375</v>
       </c>
       <c r="D136" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4682,10 +4682,10 @@
         <v>375</v>
       </c>
       <c r="D137" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E137" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4699,10 +4699,10 @@
         <v>375</v>
       </c>
       <c r="D138" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4716,10 +4716,10 @@
         <v>365</v>
       </c>
       <c r="D139" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E139" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4733,10 +4733,10 @@
         <v>384</v>
       </c>
       <c r="D140" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4750,10 +4750,10 @@
         <v>387</v>
       </c>
       <c r="D141" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4767,10 +4767,10 @@
         <v>390</v>
       </c>
       <c r="D142" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4784,10 +4784,10 @@
         <v>393</v>
       </c>
       <c r="D143" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4801,10 +4801,10 @@
         <v>396</v>
       </c>
       <c r="D144" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4818,10 +4818,10 @@
         <v>393</v>
       </c>
       <c r="D145" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4835,10 +4835,10 @@
         <v>401</v>
       </c>
       <c r="D146" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4852,10 +4852,10 @@
         <v>401</v>
       </c>
       <c r="D147" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4869,10 +4869,10 @@
         <v>393</v>
       </c>
       <c r="D148" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4886,10 +4886,10 @@
         <v>393</v>
       </c>
       <c r="D149" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E149" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4903,10 +4903,10 @@
         <v>396</v>
       </c>
       <c r="D150" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E150" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4920,10 +4920,10 @@
         <v>396</v>
       </c>
       <c r="D151" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E151" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4937,10 +4937,10 @@
         <v>390</v>
       </c>
       <c r="D152" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4954,10 +4954,10 @@
         <v>390</v>
       </c>
       <c r="D153" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4971,10 +4971,10 @@
         <v>396</v>
       </c>
       <c r="D154" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4988,10 +4988,10 @@
         <v>390</v>
       </c>
       <c r="D155" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E155" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5005,10 +5005,10 @@
         <v>422</v>
       </c>
       <c r="D156" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5022,10 +5022,10 @@
         <v>425</v>
       </c>
       <c r="D157" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E157" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5039,10 +5039,10 @@
         <v>428</v>
       </c>
       <c r="D158" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5056,10 +5056,10 @@
         <v>428</v>
       </c>
       <c r="D159" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E159" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5073,10 +5073,10 @@
         <v>428</v>
       </c>
       <c r="D160" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5090,10 +5090,10 @@
         <v>428</v>
       </c>
       <c r="D161" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E161" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5107,10 +5107,10 @@
         <v>428</v>
       </c>
       <c r="D162" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5124,10 +5124,10 @@
         <v>438</v>
       </c>
       <c r="D163" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5141,10 +5141,10 @@
         <v>438</v>
       </c>
       <c r="D164" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E164" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5158,10 +5158,10 @@
         <v>438</v>
       </c>
       <c r="D165" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E165" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,10 +5175,10 @@
         <v>438</v>
       </c>
       <c r="D166" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E166" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5192,10 +5192,10 @@
         <v>447</v>
       </c>
       <c r="D167" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E167" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5209,10 +5209,10 @@
         <v>450</v>
       </c>
       <c r="D168" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E168" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5226,10 +5226,10 @@
         <v>450</v>
       </c>
       <c r="D169" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E169" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5243,10 +5243,10 @@
         <v>450</v>
       </c>
       <c r="D170" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E170" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5260,10 +5260,10 @@
         <v>447</v>
       </c>
       <c r="D171" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E171" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5277,10 +5277,10 @@
         <v>447</v>
       </c>
       <c r="D172" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5294,10 +5294,10 @@
         <v>461</v>
       </c>
       <c r="D173" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E173" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5311,10 +5311,10 @@
         <v>461</v>
       </c>
       <c r="D174" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E174" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5328,10 +5328,10 @@
         <v>461</v>
       </c>
       <c r="D175" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E175" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5345,10 +5345,10 @@
         <v>461</v>
       </c>
       <c r="D176" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E176" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5362,10 +5362,10 @@
         <v>461</v>
       </c>
       <c r="D177" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E177" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5379,10 +5379,10 @@
         <v>422</v>
       </c>
       <c r="D178" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E178" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5396,10 +5396,10 @@
         <v>422</v>
       </c>
       <c r="D179" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E179" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5413,10 +5413,10 @@
         <v>422</v>
       </c>
       <c r="D180" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E180" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5430,10 +5430,10 @@
         <v>478</v>
       </c>
       <c r="D181" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E181" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5447,10 +5447,10 @@
         <v>447</v>
       </c>
       <c r="D182" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E182" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5464,10 +5464,10 @@
         <v>447</v>
       </c>
       <c r="D183" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5481,10 +5481,10 @@
         <v>447</v>
       </c>
       <c r="D184" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5498,10 +5498,10 @@
         <v>365</v>
       </c>
       <c r="D185" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E185" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5515,10 +5515,10 @@
         <v>317</v>
       </c>
       <c r="D186" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E186" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5532,10 +5532,10 @@
         <v>317</v>
       </c>
       <c r="D187" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5568,7 +5568,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="24.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="18" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="25.4"/>
@@ -5600,7 +5600,7 @@
         <v>493</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -5626,7 +5626,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5659,7 +5659,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5692,7 +5692,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">

</xml_diff>

<commit_message>
updated ssh un/filename in config.ini file
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -60,15 +60,18 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_101_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
+  </si>
+  <si>
     <t xml:space="preserve">False</t>
   </si>
   <si>
-    <t xml:space="preserve">test_sa_100_101_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_UPI_Failed_Via_SA_CheckStatus_HDFC</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_sa_100_101_003</t>
   </si>
   <si>
@@ -1045,9 +1048,6 @@
   </si>
   <si>
     <t xml:space="preserve">UI_Common_PM_UPI_AXIS_DIRECT_Amount_Mismatch_Upon_Check_Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_136</t>
@@ -1900,15 +1900,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -1917,347 +1917,347 @@
         <v>8</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>57</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>56</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2283,7 +2283,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2316,7 +2316,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2378,2025 +2378,2025 @@
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>70</v>
-      </c>
       <c r="D4" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>75</v>
-      </c>
       <c r="D6" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>100</v>
-      </c>
       <c r="D17" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>105</v>
-      </c>
       <c r="D19" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>122</v>
-      </c>
       <c r="D27" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>135</v>
-      </c>
       <c r="D33" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B41" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>154</v>
-      </c>
       <c r="D41" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="C49" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B49" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>172</v>
-      </c>
       <c r="D49" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C56" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="B56" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>189</v>
-      </c>
       <c r="D56" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B62" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>203</v>
-      </c>
       <c r="D62" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>208</v>
-      </c>
       <c r="D64" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B65" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="B65" s="7" t="s">
-        <v>210</v>
-      </c>
       <c r="C65" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C67" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B67" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>214</v>
-      </c>
       <c r="D67" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B72" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>225</v>
-      </c>
       <c r="D72" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C77" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B77" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>236</v>
-      </c>
       <c r="D77" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="B80" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>243</v>
-      </c>
       <c r="D80" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="B85" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B85" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>254</v>
-      </c>
       <c r="D85" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B96" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B98" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>287</v>
-      </c>
       <c r="D98" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D99" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D100" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B102" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>296</v>
-      </c>
       <c r="D102" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B105" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="C109" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B109" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>311</v>
-      </c>
       <c r="D109" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="B111" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>316</v>
-      </c>
       <c r="D111" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D112" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B113" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>321</v>
-      </c>
       <c r="D113" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D114" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B116" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="7" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="7" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D120" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>338</v>
+        <v>12</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4407,13 +4407,13 @@
         <v>340</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4424,13 +4424,13 @@
         <v>342</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D122" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4441,13 +4441,13 @@
         <v>344</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D123" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,13 +4458,13 @@
         <v>346</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4478,10 +4478,10 @@
         <v>349</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4495,10 +4495,10 @@
         <v>349</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4512,10 +4512,10 @@
         <v>349</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4529,10 +4529,10 @@
         <v>349</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4546,10 +4546,10 @@
         <v>358</v>
       </c>
       <c r="D129" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4563,10 +4563,10 @@
         <v>358</v>
       </c>
       <c r="D130" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4580,10 +4580,10 @@
         <v>358</v>
       </c>
       <c r="D131" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4597,10 +4597,10 @@
         <v>365</v>
       </c>
       <c r="D132" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4614,10 +4614,10 @@
         <v>365</v>
       </c>
       <c r="D133" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4631,10 +4631,10 @@
         <v>370</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4648,10 +4648,10 @@
         <v>370</v>
       </c>
       <c r="D135" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4665,10 +4665,10 @@
         <v>375</v>
       </c>
       <c r="D136" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4682,10 +4682,10 @@
         <v>375</v>
       </c>
       <c r="D137" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E137" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4699,10 +4699,10 @@
         <v>375</v>
       </c>
       <c r="D138" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4716,10 +4716,10 @@
         <v>365</v>
       </c>
       <c r="D139" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E139" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4733,10 +4733,10 @@
         <v>384</v>
       </c>
       <c r="D140" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4750,10 +4750,10 @@
         <v>387</v>
       </c>
       <c r="D141" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4767,10 +4767,10 @@
         <v>390</v>
       </c>
       <c r="D142" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4784,10 +4784,10 @@
         <v>393</v>
       </c>
       <c r="D143" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4801,10 +4801,10 @@
         <v>396</v>
       </c>
       <c r="D144" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4818,10 +4818,10 @@
         <v>393</v>
       </c>
       <c r="D145" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4835,10 +4835,10 @@
         <v>401</v>
       </c>
       <c r="D146" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4852,10 +4852,10 @@
         <v>401</v>
       </c>
       <c r="D147" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4869,10 +4869,10 @@
         <v>393</v>
       </c>
       <c r="D148" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4886,10 +4886,10 @@
         <v>393</v>
       </c>
       <c r="D149" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E149" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4903,10 +4903,10 @@
         <v>396</v>
       </c>
       <c r="D150" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E150" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4920,10 +4920,10 @@
         <v>396</v>
       </c>
       <c r="D151" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E151" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4937,10 +4937,10 @@
         <v>390</v>
       </c>
       <c r="D152" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4954,10 +4954,10 @@
         <v>390</v>
       </c>
       <c r="D153" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4971,10 +4971,10 @@
         <v>396</v>
       </c>
       <c r="D154" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4988,10 +4988,10 @@
         <v>390</v>
       </c>
       <c r="D155" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E155" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5005,10 +5005,10 @@
         <v>422</v>
       </c>
       <c r="D156" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5022,10 +5022,10 @@
         <v>425</v>
       </c>
       <c r="D157" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E157" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5039,10 +5039,10 @@
         <v>428</v>
       </c>
       <c r="D158" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5056,10 +5056,10 @@
         <v>428</v>
       </c>
       <c r="D159" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E159" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5073,10 +5073,10 @@
         <v>428</v>
       </c>
       <c r="D160" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5090,10 +5090,10 @@
         <v>428</v>
       </c>
       <c r="D161" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E161" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5107,10 +5107,10 @@
         <v>428</v>
       </c>
       <c r="D162" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5124,10 +5124,10 @@
         <v>438</v>
       </c>
       <c r="D163" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5141,10 +5141,10 @@
         <v>438</v>
       </c>
       <c r="D164" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E164" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5158,10 +5158,10 @@
         <v>438</v>
       </c>
       <c r="D165" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E165" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,10 +5175,10 @@
         <v>438</v>
       </c>
       <c r="D166" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E166" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5192,10 +5192,10 @@
         <v>447</v>
       </c>
       <c r="D167" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E167" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5209,10 +5209,10 @@
         <v>450</v>
       </c>
       <c r="D168" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E168" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5226,10 +5226,10 @@
         <v>450</v>
       </c>
       <c r="D169" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E169" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5243,10 +5243,10 @@
         <v>450</v>
       </c>
       <c r="D170" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E170" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5260,10 +5260,10 @@
         <v>447</v>
       </c>
       <c r="D171" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E171" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5277,10 +5277,10 @@
         <v>447</v>
       </c>
       <c r="D172" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5294,10 +5294,10 @@
         <v>461</v>
       </c>
       <c r="D173" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E173" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5311,10 +5311,10 @@
         <v>461</v>
       </c>
       <c r="D174" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E174" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5328,10 +5328,10 @@
         <v>461</v>
       </c>
       <c r="D175" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E175" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5345,10 +5345,10 @@
         <v>461</v>
       </c>
       <c r="D176" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E176" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5362,10 +5362,10 @@
         <v>461</v>
       </c>
       <c r="D177" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E177" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5379,10 +5379,10 @@
         <v>422</v>
       </c>
       <c r="D178" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E178" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5396,10 +5396,10 @@
         <v>422</v>
       </c>
       <c r="D179" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E179" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5413,10 +5413,10 @@
         <v>422</v>
       </c>
       <c r="D180" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E180" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5430,10 +5430,10 @@
         <v>478</v>
       </c>
       <c r="D181" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E181" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5447,10 +5447,10 @@
         <v>447</v>
       </c>
       <c r="D182" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E182" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5464,10 +5464,10 @@
         <v>447</v>
       </c>
       <c r="D183" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5481,10 +5481,10 @@
         <v>447</v>
       </c>
       <c r="D184" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5498,10 +5498,10 @@
         <v>365</v>
       </c>
       <c r="D185" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E185" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5512,13 +5512,13 @@
         <v>488</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D186" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E186" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5529,13 +5529,13 @@
         <v>490</v>
       </c>
       <c r="C187" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D187" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5568,7 +5568,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="24.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="18" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="25.4"/>
@@ -5600,7 +5600,7 @@
         <v>493</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -5626,7 +5626,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5659,7 +5659,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -5692,7 +5692,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="24.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">

</xml_diff>

<commit_message>
Added config Processor file
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -851,6 +851,9 @@
     <t xml:space="preserve">API_DB/Common</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_common_300_301_002</t>
   </si>
   <si>
@@ -1041,9 +1044,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/API_DB/Common/test_NonUI_Common_Ezewallet_Agency_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_200_201_002</t>
@@ -2723,7 +2723,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="26.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="26.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.87"/>
@@ -3202,7 +3202,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3235,7 +3235,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3268,7 +3268,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA83"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60.32"/>
@@ -4851,7 +4851,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.4"/>
@@ -4909,7 +4909,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -4942,7 +4942,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -4975,7 +4975,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F236"/>
-  <sheetFormatPr defaultColWidth="22.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="75.14"/>
@@ -5014,15 +5014,15 @@
         <v>249</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>248</v>
@@ -5031,15 +5031,15 @@
         <v>249</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>248</v>
@@ -5048,449 +5048,449 @@
         <v>249</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="B6" s="21" t="s">
-        <v>258</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>256</v>
-      </c>
       <c r="D6" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>270</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="B11" s="21" t="s">
-        <v>269</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>267</v>
-      </c>
       <c r="D11" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>281</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>280</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>278</v>
-      </c>
       <c r="D16" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
+        <v>287</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="B19" s="21" t="s">
-        <v>287</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>285</v>
-      </c>
       <c r="D19" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>302</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="B25" s="21" t="s">
-        <v>301</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>299</v>
-      </c>
       <c r="D25" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>8</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5501,13 +5501,13 @@
         <v>316</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5518,13 +5518,13 @@
         <v>318</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5535,13 +5535,13 @@
         <v>320</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5552,13 +5552,13 @@
         <v>322</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>249</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5575,7 +5575,7 @@
         <v>249</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5592,7 +5592,7 @@
         <v>249</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5609,7 +5609,7 @@
         <v>249</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5796,7 +5796,7 @@
         <v>249</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5813,7 +5813,7 @@
         <v>249</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5830,7 +5830,7 @@
         <v>249</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5847,7 +5847,7 @@
         <v>249</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5864,7 +5864,7 @@
         <v>249</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>314</v>
+        <v>250</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
detailed val updated tcs
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -128,391 +128,391 @@
     <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_QR_Generation_HDFC</t>
   </si>
   <si>
+    <t xml:space="preserve">test_sa_100_102_059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_Success_Via_CheckStatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_CheckStatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_BQRV4_QR_Generation_Success_YES_ATOS_59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_QR_Generation_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQRV4_AfterExpiry_Via_CheckStatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_BQRV4_Checkstatus_Success_AXIS_ATOS_078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_CheckStatus_AXIS_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_BQRV4_CheckStatus_Expired_AXIS_ATOS_079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_BQRV4_QR_Generation_Success_AXIS_ATOS_80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_QR_Generation_AXIS_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_PM_BQR_AXIS_ATOS_QR_Generation_Failed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_BQRV4_BQR_Checkstatus_Success_AXIS_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_AXIS_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_BQRV4_BQR_CheckStatus_After_Expired_AXIS_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_sa_100_102_205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_SA_BQRV4_QR_Generation_Success_AXIS_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Success_HDFC _01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/Common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Failed_HDFC _02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_AfterExpiry_HDFC _03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Success_HDFC _04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Failed_HDFC _05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_AfterExpiry_HDFC _06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_BQR_two_Callback_Success_AutoRefund_Disbaled_HDFC_11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_disabled_HDFC_12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_enabled_HDFC_13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_HDFC_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_HDFC_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_HDFC_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_Portal_HDFC_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Pending_HDFC _018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_Failed_AUTOREFUND_ENABLED_HDFC_21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_HDFC_22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_API_HDFC_23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Success_YES_ATOS_24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Callback_AfterExpiry_YES_ATOS_25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Success_YES_ATOS_30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_AfterExpiry_YES_ATOS _31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_two_Callback_Success_YES_ATOS _32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_disabled_YES_ATOS_33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_enabled_YES_ATOS_34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_YES_ATOS_35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_YES_ATOS_36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_YES_ATOS_37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_YES_ATOS_38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Pending_YES_ATOS_39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPGAutoRefund_Enabled_YES_ATOS _40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_YES_ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPGAutoRefund_Disabled_YES_ATOS _41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_API_YES_ATOS_42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_portal_YES_ATOS_43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_Posted_YES_ATOS_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQR_Refund_Failed_YES_ATOS_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Success_UPI_Callback_HDFC _046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Callback_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Failed_UPI_Callback_HDFC_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_BQRV4_Expired_UPI_ExpiredCallback_HDFC_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_PM_Initiate_BQRV4_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Checkstatus_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_BQRV4_Refund_via_HDFC_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Refund_HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_common_100_102_053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI_Common_BQRV4_Refund_UPI_via_API_HDFC _053</t>
+  </si>
+  <si>
     <t xml:space="preserve">True</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_Success_Via_CheckStatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_CheckStatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_060</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_BQRV4_QR_Generation_Success_YES_ATOS_59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_QR_Generation_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_073</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQRV4_AfterExpiry_Via_CheckStatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_BQRV4_Checkstatus_Success_AXIS_ATOS_078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_CheckStatus_AXIS_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_079</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_BQRV4_CheckStatus_Expired_AXIS_ATOS_079</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_080</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_BQRV4_QR_Generation_Success_AXIS_ATOS_80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQRV4_QR_Generation_AXIS_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_PM_BQR_AXIS_ATOS_QR_Generation_Failed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_BQRV4_BQR_Checkstatus_Success_AXIS_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/SA/test_UI_SA_BQR_CheckStatus_AXIS_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_BQRV4_BQR_CheckStatus_After_Expired_AXIS_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_sa_100_102_205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_SA_BQRV4_QR_Generation_Success_AXIS_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Success_HDFC _01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/Common</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Failed_HDFC _02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_AfterExpiry_HDFC _03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Success_HDFC _04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Failed_HDFC _05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_AfterExpiry_HDFC _06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_BQR_two_Callback_Success_AutoRefund_Disbaled_HDFC_11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_HDFC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_disabled_HDFC_12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_enabled_HDFC_13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_HDFC_014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_HDFC_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_HDFC_016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_Portal_HDFC_017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Pending_HDFC _018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_AUTOREFUND_ENABLED_HDFC_20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_Failed_AUTOREFUND_ENABLED_HDFC_21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_HDFC_22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_API_HDFC_23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_Success_YES_ATOS_24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Callback_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Callback_AfterExpiry_YES_ATOS_25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_Success_YES_ATOS_30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Checkstatus_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Checkstatus_AfterExpiry_YES_ATOS _31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_two_Callback_Success_YES_ATOS _32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_disabled_YES_ATOS_33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Expired_Callback_AutoRefund_enabled_YES_ATOS_34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_YES_ATOS_35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Refund_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_API_YES_ATOS_36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_YES_ATOS_37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Partial_Refund_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Partial_Refund_API_YES_ATOS_38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Pending_YES_ATOS_39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_Pending_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPGAutoRefund_Enabled_YES_ATOS _40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQR_UPG_YES_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPGAutoRefund_Disabled_YES_ATOS _41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_API_YES_ATOS_42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_UPG_REFUND_via_portal_YES_ATOS_43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_Posted_YES_ATOS_044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQR_Refund_Failed_YES_ATOS_045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_Success_UPI_Callback_HDFC _046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Callback_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_Failed_UPI_Callback_HDFC_047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_BQRV4_Expired_UPI_ExpiredCallback_HDFC_048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_PM_Initiate_BQRV4_qr_via_api_Success_Via_CheckStatus_API_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Checkstatus_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_052</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_BQRV4_Refund_via_HDFC_052</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional/UI/Common/test_UI_Common_BQRV4_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_common_100_102_053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI_Common_BQRV4_Refund_UPI_via_API_HDFC _053</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_102_054</t>
@@ -1891,18 +1891,18 @@
         <v>8</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>35</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>36</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>8</v>
@@ -1913,13 +1913,13 @@
     </row>
     <row r="13" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>39</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>8</v>
@@ -1930,13 +1930,13 @@
     </row>
     <row r="14" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>41</v>
-      </c>
       <c r="C14" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>8</v>
@@ -1947,13 +1947,13 @@
     </row>
     <row r="15" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>43</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>44</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>8</v>
@@ -1964,13 +1964,13 @@
     </row>
     <row r="16" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>46</v>
-      </c>
       <c r="C16" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>8</v>
@@ -1981,13 +1981,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="C17" s="10" t="s">
         <v>48</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>8</v>
@@ -3017,13 +3017,13 @@
     </row>
     <row r="18" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="C18" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>8</v>
@@ -3034,13 +3034,13 @@
     </row>
     <row r="19" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>8</v>
@@ -3051,13 +3051,13 @@
     </row>
     <row r="20" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="C20" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>8</v>
@@ -3068,13 +3068,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>58</v>
-      </c>
       <c r="C21" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>8</v>
@@ -4126,7 +4126,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="19.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
@@ -4159,7 +4159,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="19.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
@@ -4221,16 +4221,16 @@
     </row>
     <row r="2" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="18" t="s">
-        <v>61</v>
-      </c>
       <c r="D2" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>9</v>
@@ -4238,16 +4238,16 @@
     </row>
     <row r="3" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>64</v>
-      </c>
       <c r="C3" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>9</v>
@@ -4255,16 +4255,16 @@
     </row>
     <row r="4" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="C4" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>9</v>
@@ -4272,16 +4272,16 @@
     </row>
     <row r="5" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>69</v>
-      </c>
       <c r="D5" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E5" s="19" t="s">
         <v>9</v>
@@ -4289,16 +4289,16 @@
     </row>
     <row r="6" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="C6" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>9</v>
@@ -4306,16 +4306,16 @@
     </row>
     <row r="7" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>73</v>
-      </c>
       <c r="C7" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>9</v>
@@ -4323,16 +4323,16 @@
     </row>
     <row r="8" s="20" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>76</v>
-      </c>
       <c r="D8" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>9</v>
@@ -4340,16 +4340,16 @@
     </row>
     <row r="9" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>78</v>
-      </c>
       <c r="C9" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E9" s="19" t="s">
         <v>9</v>
@@ -4357,16 +4357,16 @@
     </row>
     <row r="10" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="C10" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>9</v>
@@ -4374,16 +4374,16 @@
     </row>
     <row r="11" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="20" t="s">
-        <v>83</v>
-      </c>
       <c r="D11" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E11" s="19" t="s">
         <v>9</v>
@@ -4391,16 +4391,16 @@
     </row>
     <row r="12" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>85</v>
-      </c>
       <c r="C12" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E12" s="19" t="s">
         <v>9</v>
@@ -4408,16 +4408,16 @@
     </row>
     <row r="13" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="20" t="s">
-        <v>88</v>
-      </c>
       <c r="D13" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>9</v>
@@ -4425,16 +4425,16 @@
     </row>
     <row r="14" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="C14" s="20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E14" s="19" t="s">
         <v>9</v>
@@ -4442,16 +4442,16 @@
     </row>
     <row r="15" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="C15" s="20" t="s">
-        <v>93</v>
-      </c>
       <c r="D15" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E15" s="19" t="s">
         <v>9</v>
@@ -4459,16 +4459,16 @@
     </row>
     <row r="16" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="20" t="s">
-        <v>96</v>
-      </c>
       <c r="D16" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>9</v>
@@ -4476,16 +4476,16 @@
     </row>
     <row r="17" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="C17" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>9</v>
@@ -4493,16 +4493,16 @@
     </row>
     <row r="18" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="C18" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E18" s="19" t="s">
         <v>9</v>
@@ -4510,16 +4510,16 @@
     </row>
     <row r="19" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>102</v>
-      </c>
       <c r="C19" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E19" s="19" t="s">
         <v>9</v>
@@ -4527,16 +4527,16 @@
     </row>
     <row r="20" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>104</v>
-      </c>
       <c r="C20" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E20" s="19" t="s">
         <v>9</v>
@@ -4544,16 +4544,16 @@
     </row>
     <row r="21" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="20" t="s">
-        <v>107</v>
-      </c>
       <c r="D21" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>9</v>
@@ -4561,16 +4561,16 @@
     </row>
     <row r="22" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>109</v>
-      </c>
       <c r="C22" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>9</v>
@@ -4578,16 +4578,16 @@
     </row>
     <row r="23" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="20" t="s">
-        <v>112</v>
-      </c>
       <c r="D23" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E23" s="19" t="s">
         <v>9</v>
@@ -4595,16 +4595,16 @@
     </row>
     <row r="24" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>114</v>
-      </c>
       <c r="C24" s="20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>9</v>
@@ -4612,16 +4612,16 @@
     </row>
     <row r="25" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="B25" s="20" t="s">
-        <v>116</v>
-      </c>
       <c r="C25" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>9</v>
@@ -4629,16 +4629,16 @@
     </row>
     <row r="26" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>118</v>
-      </c>
       <c r="C26" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E26" s="19" t="s">
         <v>9</v>
@@ -4646,16 +4646,16 @@
     </row>
     <row r="27" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="C27" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>9</v>
@@ -4663,16 +4663,16 @@
     </row>
     <row r="28" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="C28" s="20" t="s">
-        <v>123</v>
-      </c>
       <c r="D28" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>9</v>
@@ -4680,16 +4680,16 @@
     </row>
     <row r="29" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="C29" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>9</v>
@@ -4697,16 +4697,16 @@
     </row>
     <row r="30" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C30" s="20" t="s">
-        <v>128</v>
-      </c>
       <c r="D30" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>9</v>
@@ -4714,16 +4714,16 @@
     </row>
     <row r="31" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="C31" s="20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>9</v>
@@ -4731,16 +4731,16 @@
     </row>
     <row r="32" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="C32" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="20" t="s">
-        <v>133</v>
-      </c>
       <c r="D32" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E32" s="19" t="s">
         <v>9</v>
@@ -4748,16 +4748,16 @@
     </row>
     <row r="33" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="C33" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="C33" s="20" t="s">
-        <v>136</v>
-      </c>
       <c r="D33" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>9</v>
@@ -4765,16 +4765,16 @@
     </row>
     <row r="34" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>138</v>
-      </c>
       <c r="C34" s="20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>9</v>
@@ -4782,16 +4782,16 @@
     </row>
     <row r="35" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>140</v>
-      </c>
       <c r="C35" s="20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E35" s="19" t="s">
         <v>9</v>
@@ -4799,16 +4799,16 @@
     </row>
     <row r="36" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="C36" s="20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E36" s="19" t="s">
         <v>9</v>
@@ -4816,16 +4816,16 @@
     </row>
     <row r="37" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>144</v>
-      </c>
       <c r="C37" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>9</v>
@@ -4833,16 +4833,16 @@
     </row>
     <row r="38" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="C38" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>9</v>
@@ -4850,16 +4850,16 @@
     </row>
     <row r="39" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="B39" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="C39" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="C39" s="20" t="s">
-        <v>149</v>
-      </c>
       <c r="D39" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>9</v>
@@ -4867,16 +4867,16 @@
     </row>
     <row r="40" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B40" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B40" s="22" t="s">
-        <v>151</v>
-      </c>
       <c r="C40" s="20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>9</v>
@@ -4884,16 +4884,16 @@
     </row>
     <row r="41" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="B41" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="B41" s="22" t="s">
-        <v>153</v>
-      </c>
       <c r="C41" s="20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E41" s="19" t="s">
         <v>9</v>
@@ -4901,16 +4901,16 @@
     </row>
     <row r="42" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B42" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="C42" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="C42" s="20" t="s">
-        <v>156</v>
-      </c>
       <c r="D42" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E42" s="19" t="s">
         <v>9</v>
@@ -4918,16 +4918,16 @@
     </row>
     <row r="43" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="C43" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="C43" s="20" t="s">
-        <v>159</v>
-      </c>
       <c r="D43" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E43" s="19" t="s">
         <v>9</v>
@@ -4935,19 +4935,19 @@
     </row>
     <row r="44" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="B44" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="C44" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" s="19" t="s">
         <v>161</v>
-      </c>
-      <c r="C44" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="D44" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E44" s="19" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="45" s="20" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4961,7 +4961,7 @@
         <v>164</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>9</v>
@@ -4978,7 +4978,7 @@
         <v>164</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E46" s="19" t="s">
         <v>9</v>
@@ -4992,10 +4992,10 @@
         <v>168</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>9</v>
@@ -5009,10 +5009,10 @@
         <v>170</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D48" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>9</v>
@@ -5029,7 +5029,7 @@
         <v>173</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E49" s="19" t="s">
         <v>9</v>
@@ -5046,7 +5046,7 @@
         <v>176</v>
       </c>
       <c r="D50" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>9</v>
@@ -5063,7 +5063,7 @@
         <v>176</v>
       </c>
       <c r="D51" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>9</v>
@@ -5080,7 +5080,7 @@
         <v>181</v>
       </c>
       <c r="D52" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E52" s="19" t="s">
         <v>9</v>
@@ -5097,7 +5097,7 @@
         <v>173</v>
       </c>
       <c r="D53" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E53" s="19" t="s">
         <v>9</v>
@@ -5114,7 +5114,7 @@
         <v>186</v>
       </c>
       <c r="D54" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E54" s="19" t="s">
         <v>9</v>
@@ -5131,7 +5131,7 @@
         <v>189</v>
       </c>
       <c r="D55" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E55" s="19" t="s">
         <v>9</v>
@@ -5148,7 +5148,7 @@
         <v>189</v>
       </c>
       <c r="D56" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E56" s="19" t="s">
         <v>9</v>
@@ -5165,7 +5165,7 @@
         <v>189</v>
       </c>
       <c r="D57" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E57" s="19" t="s">
         <v>9</v>
@@ -5182,7 +5182,7 @@
         <v>173</v>
       </c>
       <c r="D58" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E58" s="19" t="s">
         <v>9</v>
@@ -5199,7 +5199,7 @@
         <v>176</v>
       </c>
       <c r="D59" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E59" s="19" t="s">
         <v>9</v>
@@ -5216,7 +5216,7 @@
         <v>173</v>
       </c>
       <c r="D60" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E60" s="19" t="s">
         <v>9</v>
@@ -5233,7 +5233,7 @@
         <v>173</v>
       </c>
       <c r="D61" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E61" s="19" t="s">
         <v>9</v>
@@ -5250,7 +5250,7 @@
         <v>204</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E62" s="19" t="s">
         <v>9</v>
@@ -5267,7 +5267,7 @@
         <v>204</v>
       </c>
       <c r="D63" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E63" s="19" t="s">
         <v>9</v>
@@ -6303,7 +6303,7 @@
         <v>209</v>
       </c>
       <c r="D64" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E64" s="19" t="s">
         <v>9</v>
@@ -7339,7 +7339,7 @@
         <v>209</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E65" s="19" t="s">
         <v>9</v>
@@ -8375,7 +8375,7 @@
         <v>214</v>
       </c>
       <c r="D66" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E66" s="19" t="s">
         <v>9</v>
@@ -9411,7 +9411,7 @@
         <v>214</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E67" s="19" t="s">
         <v>9</v>
@@ -9425,10 +9425,10 @@
         <v>218</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D68" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E68" s="19" t="s">
         <v>9</v>
@@ -9442,10 +9442,10 @@
         <v>220</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D69" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E69" s="19" t="s">
         <v>9</v>
@@ -9459,10 +9459,10 @@
         <v>222</v>
       </c>
       <c r="C70" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D70" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E70" s="19" t="s">
         <v>9</v>
@@ -9476,10 +9476,10 @@
         <v>224</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D71" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E71" s="19" t="s">
         <v>9</v>
@@ -9493,10 +9493,10 @@
         <v>226</v>
       </c>
       <c r="C72" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D72" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E72" s="19" t="s">
         <v>9</v>
@@ -9510,10 +9510,10 @@
         <v>228</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E73" s="19" t="s">
         <v>9</v>
@@ -9530,7 +9530,7 @@
         <v>231</v>
       </c>
       <c r="D74" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E74" s="19" t="s">
         <v>9</v>
@@ -9547,7 +9547,7 @@
         <v>231</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E75" s="19" t="s">
         <v>9</v>
@@ -9564,7 +9564,7 @@
         <v>231</v>
       </c>
       <c r="D76" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E76" s="19" t="s">
         <v>9</v>
@@ -9581,7 +9581,7 @@
         <v>238</v>
       </c>
       <c r="D77" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E77" s="19" t="s">
         <v>9</v>
@@ -9598,7 +9598,7 @@
         <v>238</v>
       </c>
       <c r="D78" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E78" s="19" t="s">
         <v>9</v>
@@ -9615,7 +9615,7 @@
         <v>238</v>
       </c>
       <c r="D79" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E79" s="19" t="s">
         <v>9</v>
@@ -9632,7 +9632,7 @@
         <v>231</v>
       </c>
       <c r="D80" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E80" s="19" t="s">
         <v>9</v>
@@ -9649,7 +9649,7 @@
         <v>231</v>
       </c>
       <c r="D81" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E81" s="19" t="s">
         <v>9</v>
@@ -9666,10 +9666,10 @@
         <v>249</v>
       </c>
       <c r="D82" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E82" s="19" t="s">
-        <v>9</v>
+        <v>161</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9683,7 +9683,7 @@
         <v>249</v>
       </c>
       <c r="D83" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E83" s="19" t="s">
         <v>9</v>
@@ -9700,7 +9700,7 @@
         <v>249</v>
       </c>
       <c r="D84" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E84" s="19" t="s">
         <v>9</v>
@@ -9717,7 +9717,7 @@
         <v>249</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E85" s="19" t="s">
         <v>9</v>
@@ -9734,7 +9734,7 @@
         <v>258</v>
       </c>
       <c r="D86" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E86" s="19" t="s">
         <v>9</v>
@@ -9751,7 +9751,7 @@
         <v>261</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E87" s="19" t="s">
         <v>9</v>
@@ -9768,7 +9768,7 @@
         <v>258</v>
       </c>
       <c r="D88" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E88" s="19" t="s">
         <v>9</v>
@@ -9785,7 +9785,7 @@
         <v>258</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E89" s="19" t="s">
         <v>9</v>
@@ -9802,7 +9802,7 @@
         <v>268</v>
       </c>
       <c r="D90" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E90" s="19" t="s">
         <v>9</v>
@@ -9819,7 +9819,7 @@
         <v>238</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E91" s="19" t="s">
         <v>9</v>
@@ -9836,7 +9836,7 @@
         <v>261</v>
       </c>
       <c r="D92" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E92" s="19" t="s">
         <v>9</v>
@@ -9853,7 +9853,7 @@
         <v>261</v>
       </c>
       <c r="D93" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E93" s="19" t="s">
         <v>9</v>
@@ -9870,7 +9870,7 @@
         <v>261</v>
       </c>
       <c r="D94" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E94" s="19" t="s">
         <v>9</v>
@@ -9887,7 +9887,7 @@
         <v>279</v>
       </c>
       <c r="D95" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E95" s="19" t="s">
         <v>9</v>
@@ -9904,7 +9904,7 @@
         <v>279</v>
       </c>
       <c r="D96" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E96" s="19" t="s">
         <v>9</v>
@@ -9921,7 +9921,7 @@
         <v>284</v>
       </c>
       <c r="D97" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E97" s="19" t="s">
         <v>9</v>
@@ -9938,7 +9938,7 @@
         <v>279</v>
       </c>
       <c r="D98" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E98" s="19" t="s">
         <v>9</v>
@@ -9955,7 +9955,7 @@
         <v>279</v>
       </c>
       <c r="D99" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E99" s="19" t="s">
         <v>9</v>
@@ -9972,7 +9972,7 @@
         <v>291</v>
       </c>
       <c r="D100" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E100" s="19" t="s">
         <v>9</v>
@@ -9989,7 +9989,7 @@
         <v>291</v>
       </c>
       <c r="D101" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E101" s="19" t="s">
         <v>9</v>
@@ -10006,7 +10006,7 @@
         <v>291</v>
       </c>
       <c r="D102" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E102" s="19" t="s">
         <v>9</v>
@@ -10023,7 +10023,7 @@
         <v>291</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E103" s="19" t="s">
         <v>9</v>
@@ -10040,7 +10040,7 @@
         <v>300</v>
       </c>
       <c r="D104" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E104" s="19" t="s">
         <v>9</v>
@@ -10057,7 +10057,7 @@
         <v>303</v>
       </c>
       <c r="D105" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E105" s="19" t="s">
         <v>9</v>
@@ -10074,7 +10074,7 @@
         <v>303</v>
       </c>
       <c r="D106" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E106" s="19" t="s">
         <v>9</v>
@@ -10091,7 +10091,7 @@
         <v>303</v>
       </c>
       <c r="D107" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E107" s="19" t="s">
         <v>9</v>
@@ -10108,7 +10108,7 @@
         <v>303</v>
       </c>
       <c r="D108" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E108" s="19" t="s">
         <v>9</v>
@@ -10125,7 +10125,7 @@
         <v>284</v>
       </c>
       <c r="D109" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E109" s="19" t="s">
         <v>9</v>
@@ -10142,7 +10142,7 @@
         <v>291</v>
       </c>
       <c r="D110" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E110" s="19" t="s">
         <v>9</v>
@@ -10159,7 +10159,7 @@
         <v>316</v>
       </c>
       <c r="D111" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E111" s="19" t="s">
         <v>9</v>
@@ -10176,7 +10176,7 @@
         <v>316</v>
       </c>
       <c r="D112" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E112" s="19" t="s">
         <v>9</v>
@@ -10193,7 +10193,7 @@
         <v>316</v>
       </c>
       <c r="D113" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E113" s="19" t="s">
         <v>9</v>
@@ -10210,7 +10210,7 @@
         <v>316</v>
       </c>
       <c r="D114" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E114" s="19" t="s">
         <v>9</v>
@@ -10227,7 +10227,7 @@
         <v>316</v>
       </c>
       <c r="D115" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E115" s="19" t="s">
         <v>9</v>
@@ -10241,10 +10241,10 @@
         <v>326</v>
       </c>
       <c r="C116" s="20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D116" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E116" s="19" t="s">
         <v>9</v>
@@ -10261,7 +10261,7 @@
         <v>164</v>
       </c>
       <c r="D117" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E117" s="19" t="s">
         <v>9</v>
@@ -10278,7 +10278,7 @@
         <v>164</v>
       </c>
       <c r="D118" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E118" s="19" t="s">
         <v>9</v>
@@ -10295,7 +10295,7 @@
         <v>164</v>
       </c>
       <c r="D119" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E119" s="19" t="s">
         <v>9</v>
@@ -10309,10 +10309,10 @@
         <v>334</v>
       </c>
       <c r="C120" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D120" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E120" s="19" t="s">
         <v>9</v>
@@ -10329,7 +10329,7 @@
         <v>337</v>
       </c>
       <c r="D121" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E121" s="19" t="s">
         <v>9</v>
@@ -10343,10 +10343,10 @@
         <v>339</v>
       </c>
       <c r="C122" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D122" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E122" s="19" t="s">
         <v>9</v>
@@ -10360,10 +10360,10 @@
         <v>341</v>
       </c>
       <c r="C123" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D123" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E123" s="19" t="s">
         <v>9</v>
@@ -10377,10 +10377,10 @@
         <v>343</v>
       </c>
       <c r="C124" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D124" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E124" s="19" t="s">
         <v>9</v>
@@ -10394,10 +10394,10 @@
         <v>345</v>
       </c>
       <c r="C125" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D125" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E125" s="19" t="s">
         <v>9</v>
@@ -10414,7 +10414,7 @@
         <v>249</v>
       </c>
       <c r="D126" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E126" s="19" t="s">
         <v>9</v>
@@ -10431,7 +10431,7 @@
         <v>279</v>
       </c>
       <c r="D127" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E127" s="19" t="s">
         <v>9</v>
@@ -10448,7 +10448,7 @@
         <v>204</v>
       </c>
       <c r="D128" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E128" s="19" t="s">
         <v>9</v>
@@ -10465,7 +10465,7 @@
         <v>204</v>
       </c>
       <c r="D129" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E129" s="19" t="s">
         <v>9</v>
@@ -10482,7 +10482,7 @@
         <v>204</v>
       </c>
       <c r="D130" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E130" s="19" t="s">
         <v>9</v>
@@ -10499,7 +10499,7 @@
         <v>209</v>
       </c>
       <c r="D131" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E131" s="19" t="s">
         <v>9</v>
@@ -10516,7 +10516,7 @@
         <v>360</v>
       </c>
       <c r="D132" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E132" s="19" t="s">
         <v>9</v>
@@ -10533,7 +10533,7 @@
         <v>360</v>
       </c>
       <c r="D133" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E133" s="19" t="s">
         <v>9</v>
@@ -10550,7 +10550,7 @@
         <v>360</v>
       </c>
       <c r="D134" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E134" s="19" t="s">
         <v>9</v>
@@ -10567,7 +10567,7 @@
         <v>367</v>
       </c>
       <c r="D135" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E135" s="19" t="s">
         <v>9</v>
@@ -10584,7 +10584,7 @@
         <v>367</v>
       </c>
       <c r="D136" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E136" s="19" t="s">
         <v>9</v>
@@ -10601,7 +10601,7 @@
         <v>367</v>
       </c>
       <c r="D137" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E137" s="19" t="s">
         <v>9</v>
@@ -10618,7 +10618,7 @@
         <v>367</v>
       </c>
       <c r="D138" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E138" s="19" t="s">
         <v>9</v>
@@ -10635,7 +10635,7 @@
         <v>376</v>
       </c>
       <c r="D139" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E139" s="19" t="s">
         <v>9</v>
@@ -10652,7 +10652,7 @@
         <v>379</v>
       </c>
       <c r="D140" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E140" s="19" t="s">
         <v>9</v>
@@ -10669,7 +10669,7 @@
         <v>379</v>
       </c>
       <c r="D141" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E141" s="19" t="s">
         <v>9</v>
@@ -10686,7 +10686,7 @@
         <v>384</v>
       </c>
       <c r="D142" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E142" s="19" t="s">
         <v>9</v>
@@ -10703,7 +10703,7 @@
         <v>384</v>
       </c>
       <c r="D143" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E143" s="19" t="s">
         <v>9</v>
@@ -10720,7 +10720,7 @@
         <v>379</v>
       </c>
       <c r="D144" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E144" s="19" t="s">
         <v>9</v>
@@ -10737,7 +10737,7 @@
         <v>390</v>
       </c>
       <c r="D145" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E145" s="19" t="s">
         <v>9</v>
@@ -10754,7 +10754,7 @@
         <v>390</v>
       </c>
       <c r="D146" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E146" s="19" t="s">
         <v>9</v>
@@ -10771,7 +10771,7 @@
         <v>376</v>
       </c>
       <c r="D147" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E147" s="19" t="s">
         <v>9</v>
@@ -10788,7 +10788,7 @@
         <v>397</v>
       </c>
       <c r="D148" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E148" s="19" t="s">
         <v>9</v>
@@ -10805,7 +10805,7 @@
         <v>400</v>
       </c>
       <c r="D149" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E149" s="19" t="s">
         <v>9</v>
@@ -10822,7 +10822,7 @@
         <v>400</v>
       </c>
       <c r="D150" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E150" s="19" t="s">
         <v>9</v>
@@ -10839,7 +10839,7 @@
         <v>400</v>
       </c>
       <c r="D151" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E151" s="19" t="s">
         <v>9</v>
@@ -10856,7 +10856,7 @@
         <v>400</v>
       </c>
       <c r="D152" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E152" s="19" t="s">
         <v>9</v>
@@ -10873,7 +10873,7 @@
         <v>400</v>
       </c>
       <c r="D153" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E153" s="19" t="s">
         <v>9</v>
@@ -10890,7 +10890,7 @@
         <v>411</v>
       </c>
       <c r="D154" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E154" s="19" t="s">
         <v>9</v>
@@ -10907,7 +10907,7 @@
         <v>411</v>
       </c>
       <c r="D155" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E155" s="19" t="s">
         <v>9</v>
@@ -10924,7 +10924,7 @@
         <v>411</v>
       </c>
       <c r="D156" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E156" s="19" t="s">
         <v>9</v>
@@ -10992,7 +10992,7 @@
         <v>425</v>
       </c>
       <c r="D160" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E160" s="19" t="s">
         <v>9</v>
@@ -11009,7 +11009,7 @@
         <v>384</v>
       </c>
       <c r="D161" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E161" s="19" t="s">
         <v>9</v>
@@ -11026,7 +11026,7 @@
         <v>429</v>
       </c>
       <c r="D162" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E162" s="19" t="s">
         <v>9</v>
@@ -11043,7 +11043,7 @@
         <v>429</v>
       </c>
       <c r="D163" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E163" s="19" t="s">
         <v>9</v>
@@ -11060,7 +11060,7 @@
         <v>429</v>
       </c>
       <c r="D164" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E164" s="19" t="s">
         <v>9</v>
@@ -12235,7 +12235,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="19.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
@@ -12268,7 +12268,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="19.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="10" width="25.4"/>
@@ -12326,7 +12326,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="19.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
@@ -12359,7 +12359,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="19.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="19.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">

</xml_diff>

<commit_message>
updated detailed validation for cnp hdfc pg
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -338,9 +338,6 @@
     <t xml:space="preserve">UI_Common_PM_RP_UPI_UPG_REFUNDED_VIA_HDFC_when_UPGRefund_Enabled_&amp;_UPGAutoRefund_Enabled_REFUND_via_API</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
     <t xml:space="preserve">test_common_100_103_036</t>
   </si>
   <si>
@@ -480,6 +477,9 @@
       </rPr>
       <t xml:space="preserve">test_UI_Common_PM_RP_UPI_HDFC_UPG</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_050</t>
@@ -2010,7 +2010,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
@@ -2043,7 +2043,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
@@ -2695,15 +2695,15 @@
         <v>8</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>85</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="24" t="s">
         <v>86</v>
-      </c>
-      <c r="B37" s="24" t="s">
-        <v>87</v>
       </c>
       <c r="C37" s="24" t="s">
         <v>80</v>
@@ -2717,10 +2717,10 @@
     </row>
     <row r="38" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="24" t="s">
         <v>88</v>
-      </c>
-      <c r="B38" s="24" t="s">
-        <v>89</v>
       </c>
       <c r="C38" s="24" t="s">
         <v>80</v>
@@ -2734,13 +2734,13 @@
     </row>
     <row r="39" s="26" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B39" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B39" s="24" t="s">
+      <c r="C39" s="24" t="s">
         <v>91</v>
-      </c>
-      <c r="C39" s="24" t="s">
-        <v>92</v>
       </c>
       <c r="D39" s="25" t="s">
         <v>8</v>
@@ -2751,13 +2751,13 @@
     </row>
     <row r="40" s="26" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="B40" s="24" t="s">
-        <v>94</v>
-      </c>
       <c r="C40" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D40" s="25" t="s">
         <v>8</v>
@@ -2768,13 +2768,13 @@
     </row>
     <row r="41" s="26" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="24" t="s">
-        <v>96</v>
-      </c>
       <c r="C41" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D41" s="25" t="s">
         <v>8</v>
@@ -2785,13 +2785,13 @@
     </row>
     <row r="42" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B42" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="24" t="s">
+      <c r="C42" s="24" t="s">
         <v>98</v>
-      </c>
-      <c r="C42" s="24" t="s">
-        <v>99</v>
       </c>
       <c r="D42" s="25" t="s">
         <v>8</v>
@@ -2802,13 +2802,13 @@
     </row>
     <row r="43" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="B43" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="B43" s="24" t="s">
-        <v>101</v>
-      </c>
       <c r="C43" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D43" s="25" t="s">
         <v>8</v>
@@ -2819,13 +2819,13 @@
     </row>
     <row r="44" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="B44" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="B44" s="24" t="s">
-        <v>103</v>
-      </c>
       <c r="C44" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D44" s="25" t="s">
         <v>8</v>
@@ -2836,13 +2836,13 @@
     </row>
     <row r="45" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="B45" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="B45" s="24" t="s">
-        <v>105</v>
-      </c>
       <c r="C45" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D45" s="25" t="s">
         <v>8</v>
@@ -2853,13 +2853,13 @@
     </row>
     <row r="46" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="B46" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="24" t="s">
-        <v>107</v>
-      </c>
       <c r="C46" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D46" s="25" t="s">
         <v>8</v>
@@ -2870,13 +2870,13 @@
     </row>
     <row r="47" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B47" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="B47" s="24" t="s">
+      <c r="C47" s="24" t="s">
         <v>109</v>
-      </c>
-      <c r="C47" s="24" t="s">
-        <v>110</v>
       </c>
       <c r="D47" s="25" t="s">
         <v>8</v>
@@ -2887,7 +2887,7 @@
     </row>
     <row r="48" s="26" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B48" s="27" t="s">
         <v>13</v>
@@ -2904,7 +2904,7 @@
     </row>
     <row r="49" s="26" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B49" s="27" t="s">
         <v>13</v>
@@ -2921,19 +2921,19 @@
     </row>
     <row r="50" s="26" customFormat="true" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B50" s="24" t="s">
         <v>13</v>
       </c>
       <c r="C50" s="24" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D50" s="25" t="s">
         <v>8</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>9</v>
+        <v>114</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2944,7 +2944,7 @@
         <v>13</v>
       </c>
       <c r="C51" s="24" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D51" s="25" t="s">
         <v>8</v>
@@ -3009,7 +3009,7 @@
         <v>123</v>
       </c>
       <c r="B55" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C55" s="24" t="s">
         <v>118</v>
@@ -3026,7 +3026,7 @@
         <v>124</v>
       </c>
       <c r="B56" s="24" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C56" s="24" t="s">
         <v>118</v>
@@ -22747,7 +22747,7 @@
         <v>126</v>
       </c>
       <c r="C77" s="24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D77" s="25" t="s">
         <v>8</v>
@@ -33384,7 +33384,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="25.4"/>
@@ -33442,7 +33442,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
@@ -33475,7 +33475,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
@@ -33508,7 +33508,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">

</xml_diff>

<commit_message>
fixed issues related to cnp
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -59,7 +59,7 @@
     <t xml:space="preserve">UI/SA</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
+    <t xml:space="preserve">False</t>
   </si>
   <si>
     <t xml:space="preserve">test_sa_100_102_008</t>
@@ -450,6 +450,9 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_CNP_Cyber_Card_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_103_008</t>
@@ -1699,9 +1702,6 @@
   </si>
   <si>
     <t xml:space="preserve">Functional/UI/Common/test_UI_Common_PM_UPI_Refund_HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">False</t>
   </si>
   <si>
     <t xml:space="preserve">test_common_100_101_011</t>
@@ -6898,7 +6898,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -6931,7 +6931,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -7107,15 +7107,15 @@
         <v>118</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>133</v>
@@ -7124,15 +7124,15 @@
         <v>118</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>117</v>
@@ -7146,10 +7146,10 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>117</v>
@@ -7163,10 +7163,10 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>133</v>
@@ -7180,10 +7180,10 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>117</v>
@@ -7197,10 +7197,10 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>133</v>
@@ -7214,13 +7214,13 @@
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>118</v>
@@ -7231,13 +7231,13 @@
     </row>
     <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>149</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>148</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>118</v>
@@ -7248,13 +7248,13 @@
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>118</v>
@@ -7265,13 +7265,13 @@
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>118</v>
@@ -7282,13 +7282,13 @@
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>118</v>
@@ -7299,13 +7299,13 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>118</v>
@@ -7316,13 +7316,13 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>159</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>158</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>118</v>
@@ -7333,13 +7333,13 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>118</v>
@@ -7350,13 +7350,13 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D23" s="21" t="s">
         <v>118</v>
@@ -7367,13 +7367,13 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>118</v>
@@ -7384,13 +7384,13 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>118</v>
@@ -7401,13 +7401,13 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>170</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>169</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>118</v>
@@ -7418,13 +7418,13 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>118</v>
@@ -7435,13 +7435,13 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>118</v>
@@ -7452,13 +7452,13 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>118</v>
@@ -7469,13 +7469,13 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>118</v>
@@ -7486,13 +7486,13 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="C31" s="13" t="s">
         <v>181</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>180</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>118</v>
@@ -7503,13 +7503,13 @@
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>118</v>
@@ -7520,13 +7520,13 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D33" s="21" t="s">
         <v>118</v>
@@ -7537,13 +7537,13 @@
     </row>
     <row r="34" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D34" s="21" t="s">
         <v>118</v>
@@ -7554,13 +7554,13 @@
     </row>
     <row r="35" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="C35" s="13" t="s">
         <v>190</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>189</v>
       </c>
       <c r="D35" s="21" t="s">
         <v>118</v>
@@ -7571,13 +7571,13 @@
     </row>
     <row r="36" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D36" s="21" t="s">
         <v>118</v>
@@ -7588,13 +7588,13 @@
     </row>
     <row r="37" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D37" s="21" t="s">
         <v>118</v>
@@ -7605,13 +7605,13 @@
     </row>
     <row r="38" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>118</v>
@@ -7622,13 +7622,13 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D39" s="21" t="s">
         <v>118</v>
@@ -7639,13 +7639,13 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>200</v>
       </c>
       <c r="D40" s="21" t="s">
         <v>118</v>
@@ -7656,13 +7656,13 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D41" s="21" t="s">
         <v>118</v>
@@ -7673,13 +7673,13 @@
     </row>
     <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D42" s="21" t="s">
         <v>118</v>
@@ -7690,13 +7690,13 @@
     </row>
     <row r="43" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>208</v>
-      </c>
-      <c r="B43" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>207</v>
       </c>
       <c r="D43" s="21" t="s">
         <v>118</v>
@@ -7707,13 +7707,13 @@
     </row>
     <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D44" s="21" t="s">
         <v>118</v>
@@ -7724,13 +7724,13 @@
     </row>
     <row r="45" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D45" s="21" t="s">
         <v>118</v>
@@ -7741,13 +7741,13 @@
     </row>
     <row r="46" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D46" s="21" t="s">
         <v>118</v>
@@ -7758,13 +7758,13 @@
     </row>
     <row r="47" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D47" s="21" t="s">
         <v>118</v>
@@ -7775,7 +7775,7 @@
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B48" s="23" t="s">
         <v>122</v>
@@ -7792,7 +7792,7 @@
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B49" s="23" t="s">
         <v>122</v>
@@ -7809,13 +7809,13 @@
     </row>
     <row r="50" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B50" s="13" t="s">
         <v>122</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D50" s="21" t="s">
         <v>118</v>
@@ -7826,13 +7826,13 @@
     </row>
     <row r="51" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B51" s="13" t="s">
         <v>122</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D51" s="21" t="s">
         <v>118</v>
@@ -7843,13 +7843,13 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D52" s="21" t="s">
         <v>118</v>
@@ -7860,13 +7860,13 @@
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="C53" s="13" t="s">
         <v>227</v>
-      </c>
-      <c r="B53" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>226</v>
       </c>
       <c r="D53" s="21" t="s">
         <v>118</v>
@@ -7877,13 +7877,13 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D54" s="21" t="s">
         <v>118</v>
@@ -7894,13 +7894,13 @@
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D55" s="21" t="s">
         <v>118</v>
@@ -7911,13 +7911,13 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>118</v>
@@ -7928,13 +7928,13 @@
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>118</v>
@@ -7945,13 +7945,13 @@
     </row>
     <row r="58" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C58" s="25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>118</v>
@@ -7962,13 +7962,13 @@
     </row>
     <row r="59" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="C59" s="25" t="s">
         <v>239</v>
-      </c>
-      <c r="B59" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="C59" s="25" t="s">
-        <v>238</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>118</v>
@@ -7979,13 +7979,13 @@
     </row>
     <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C60" s="25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>118</v>
@@ -7996,13 +7996,13 @@
     </row>
     <row r="61" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C61" s="25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>118</v>
@@ -8013,13 +8013,13 @@
     </row>
     <row r="62" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C62" s="25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D62" s="21" t="s">
         <v>118</v>
@@ -8030,13 +8030,13 @@
     </row>
     <row r="63" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C63" s="25" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D63" s="21" t="s">
         <v>118</v>
@@ -8047,13 +8047,13 @@
     </row>
     <row r="64" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="C64" s="25" t="s">
         <v>250</v>
-      </c>
-      <c r="B64" s="13" t="s">
-        <v>251</v>
-      </c>
-      <c r="C64" s="25" t="s">
-        <v>249</v>
       </c>
       <c r="D64" s="21" t="s">
         <v>118</v>
@@ -8064,13 +8064,13 @@
     </row>
     <row r="65" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C65" s="25" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D65" s="21" t="s">
         <v>118</v>
@@ -8081,13 +8081,13 @@
     </row>
     <row r="66" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C66" s="25" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D66" s="21" t="s">
         <v>118</v>
@@ -8098,13 +8098,13 @@
     </row>
     <row r="67" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C67" s="25" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D67" s="21" t="s">
         <v>118</v>
@@ -8115,13 +8115,13 @@
     </row>
     <row r="68" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C68" s="25" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D68" s="21" t="s">
         <v>118</v>
@@ -8132,13 +8132,13 @@
     </row>
     <row r="69" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="B69" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="C69" s="25" t="s">
         <v>261</v>
-      </c>
-      <c r="B69" s="13" t="s">
-        <v>262</v>
-      </c>
-      <c r="C69" s="25" t="s">
-        <v>260</v>
       </c>
       <c r="D69" s="21" t="s">
         <v>118</v>
@@ -8149,13 +8149,13 @@
     </row>
     <row r="70" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C70" s="25" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D70" s="21" t="s">
         <v>118</v>
@@ -8166,13 +8166,13 @@
     </row>
     <row r="71" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B71" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="B71" s="13" t="s">
-        <v>264</v>
-      </c>
       <c r="C71" s="25" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D71" s="21" t="s">
         <v>118</v>
@@ -8183,13 +8183,13 @@
     </row>
     <row r="72" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C72" s="25" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D72" s="21" t="s">
         <v>118</v>
@@ -8200,13 +8200,13 @@
     </row>
     <row r="73" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C73" s="25" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D73" s="21" t="s">
         <v>118</v>
@@ -8217,13 +8217,13 @@
     </row>
     <row r="74" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="B74" s="13" t="s">
+        <v>272</v>
+      </c>
+      <c r="C74" s="25" t="s">
         <v>270</v>
-      </c>
-      <c r="B74" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="C74" s="25" t="s">
-        <v>269</v>
       </c>
       <c r="D74" s="21" t="s">
         <v>118</v>
@@ -8234,13 +8234,13 @@
     </row>
     <row r="75" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="13" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C75" s="25" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D75" s="21" t="s">
         <v>118</v>
@@ -8251,13 +8251,13 @@
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D76" s="21" t="s">
         <v>118</v>
@@ -8268,13 +8268,13 @@
     </row>
     <row r="77" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D77" s="21" t="s">
         <v>118</v>
@@ -8285,13 +8285,13 @@
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="13" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C78" s="25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D78" s="21" t="s">
         <v>118</v>
@@ -8302,13 +8302,13 @@
     </row>
     <row r="79" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C79" s="25" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D79" s="21" t="s">
         <v>118</v>
@@ -8319,13 +8319,13 @@
     </row>
     <row r="80" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="B80" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="C80" s="25" t="s">
         <v>282</v>
-      </c>
-      <c r="B80" s="13" t="s">
-        <v>283</v>
-      </c>
-      <c r="C80" s="25" t="s">
-        <v>281</v>
       </c>
       <c r="D80" s="21" t="s">
         <v>118</v>
@@ -8336,13 +8336,13 @@
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C81" s="25" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D81" s="21" t="s">
         <v>118</v>
@@ -8353,13 +8353,13 @@
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="B82" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="C82" s="25" t="s">
         <v>287</v>
-      </c>
-      <c r="B82" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="C82" s="25" t="s">
-        <v>286</v>
       </c>
       <c r="D82" s="21" t="s">
         <v>118</v>
@@ -8370,13 +8370,13 @@
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="13" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C83" s="25" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D83" s="21" t="s">
         <v>118</v>
@@ -8387,13 +8387,13 @@
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="B84" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="B84" s="13" t="s">
-        <v>290</v>
-      </c>
       <c r="C84" s="25" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D84" s="21" t="s">
         <v>118</v>
@@ -8404,13 +8404,13 @@
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="13" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C85" s="25" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D85" s="21" t="s">
         <v>118</v>
@@ -8421,13 +8421,13 @@
     </row>
     <row r="86" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="26" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B86" s="27" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C86" s="25" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D86" s="21" t="s">
         <v>118</v>
@@ -8438,13 +8438,13 @@
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="13" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C87" s="25" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D87" s="21" t="s">
         <v>118</v>
@@ -8455,13 +8455,13 @@
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="B88" s="13" t="s">
+        <v>301</v>
+      </c>
+      <c r="C88" s="25" t="s">
         <v>299</v>
-      </c>
-      <c r="B88" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="C88" s="25" t="s">
-        <v>298</v>
       </c>
       <c r="D88" s="21" t="s">
         <v>118</v>
@@ -8472,13 +8472,13 @@
     </row>
     <row r="89" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="13" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C89" s="25" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D89" s="21" t="s">
         <v>118</v>
@@ -8489,13 +8489,13 @@
     </row>
     <row r="90" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="13" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B90" s="13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C90" s="25" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D90" s="21" t="s">
         <v>118</v>
@@ -8506,13 +8506,13 @@
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="13" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C91" s="25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D91" s="21" t="s">
         <v>118</v>
@@ -8523,13 +8523,13 @@
     </row>
     <row r="92" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="13" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C92" s="25" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D92" s="21" t="s">
         <v>118</v>
@@ -8540,13 +8540,13 @@
     </row>
     <row r="93" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="B93" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="C93" s="25" t="s">
         <v>311</v>
-      </c>
-      <c r="B93" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="C93" s="25" t="s">
-        <v>310</v>
       </c>
       <c r="D93" s="21" t="s">
         <v>118</v>
@@ -8557,13 +8557,13 @@
     </row>
     <row r="94" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="13" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C94" s="25" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D94" s="21" t="s">
         <v>118</v>
@@ -8574,13 +8574,13 @@
     </row>
     <row r="95" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="13" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C95" s="25" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D95" s="21" t="s">
         <v>118</v>
@@ -8591,13 +8591,13 @@
     </row>
     <row r="96" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C96" s="25" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D96" s="21" t="s">
         <v>118</v>
@@ -8608,13 +8608,13 @@
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C97" s="25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D97" s="21" t="s">
         <v>118</v>
@@ -8625,13 +8625,13 @@
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="13" t="s">
+        <v>322</v>
+      </c>
+      <c r="B98" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="C98" s="25" t="s">
         <v>321</v>
-      </c>
-      <c r="B98" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="C98" s="25" t="s">
-        <v>320</v>
       </c>
       <c r="D98" s="21" t="s">
         <v>118</v>
@@ -8642,13 +8642,13 @@
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="13" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B99" s="13" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C99" s="25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D99" s="21" t="s">
         <v>118</v>
@@ -8659,13 +8659,13 @@
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="13" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B100" s="13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D100" s="21" t="s">
         <v>118</v>
@@ -8676,13 +8676,13 @@
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B101" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C101" s="25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D101" s="21" t="s">
         <v>118</v>
@@ -8693,13 +8693,13 @@
     </row>
     <row r="102" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="13" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C102" s="25" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D102" s="21" t="s">
         <v>118</v>
@@ -8710,13 +8710,13 @@
     </row>
     <row r="103" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="B103" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="C103" s="25" t="s">
         <v>328</v>
-      </c>
-      <c r="B103" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="C103" s="25" t="s">
-        <v>327</v>
       </c>
       <c r="D103" s="21" t="s">
         <v>118</v>
@@ -8727,13 +8727,13 @@
     </row>
     <row r="104" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="13" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B104" s="13" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C104" s="25" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D104" s="21" t="s">
         <v>118</v>
@@ -8744,13 +8744,13 @@
     </row>
     <row r="105" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C105" s="25" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D105" s="21" t="s">
         <v>118</v>
@@ -8761,13 +8761,13 @@
     </row>
     <row r="106" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B106" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C106" s="25" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D106" s="21" t="s">
         <v>118</v>
@@ -8778,13 +8778,13 @@
     </row>
     <row r="107" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="B107" s="25" t="s">
         <v>336</v>
       </c>
-      <c r="B107" s="25" t="s">
-        <v>335</v>
-      </c>
       <c r="C107" s="25" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D107" s="21" t="s">
         <v>118</v>
@@ -8795,13 +8795,13 @@
     </row>
     <row r="108" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="B108" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="C108" s="25" t="s">
         <v>338</v>
-      </c>
-      <c r="B108" s="25" t="s">
-        <v>339</v>
-      </c>
-      <c r="C108" s="25" t="s">
-        <v>337</v>
       </c>
       <c r="D108" s="21" t="s">
         <v>118</v>
@@ -8812,13 +8812,13 @@
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="13" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B109" s="25" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C109" s="25" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D109" s="21" t="s">
         <v>118</v>
@@ -8829,13 +8829,13 @@
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="B110" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="C110" s="25" t="s">
         <v>343</v>
-      </c>
-      <c r="B110" s="25" t="s">
-        <v>344</v>
-      </c>
-      <c r="C110" s="25" t="s">
-        <v>342</v>
       </c>
       <c r="D110" s="21" t="s">
         <v>118</v>
@@ -8846,13 +8846,13 @@
     </row>
     <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="13" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B111" s="25" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C111" s="25" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D111" s="21" t="s">
         <v>118</v>
@@ -8863,13 +8863,13 @@
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="13" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B112" s="25" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C112" s="25" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D112" s="21" t="s">
         <v>118</v>
@@ -8880,13 +8880,13 @@
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="13" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B113" s="25" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C113" s="25" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D113" s="21" t="s">
         <v>118</v>
@@ -8897,13 +8897,13 @@
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="13" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B114" s="25" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C114" s="25" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D114" s="21" t="s">
         <v>118</v>
@@ -8914,13 +8914,13 @@
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="B115" s="25" t="s">
+        <v>356</v>
+      </c>
+      <c r="C115" s="25" t="s">
         <v>354</v>
-      </c>
-      <c r="B115" s="25" t="s">
-        <v>355</v>
-      </c>
-      <c r="C115" s="25" t="s">
-        <v>353</v>
       </c>
       <c r="D115" s="21" t="s">
         <v>118</v>
@@ -8931,13 +8931,13 @@
     </row>
     <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="13" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B116" s="25" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C116" s="25" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D116" s="21" t="s">
         <v>118</v>
@@ -8948,13 +8948,13 @@
     </row>
     <row r="117" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="13" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B117" s="25" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C117" s="25" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D117" s="21" t="s">
         <v>118</v>
@@ -8965,13 +8965,13 @@
     </row>
     <row r="118" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="B118" s="25" t="s">
+        <v>364</v>
+      </c>
+      <c r="C118" s="25" t="s">
         <v>362</v>
-      </c>
-      <c r="B118" s="25" t="s">
-        <v>363</v>
-      </c>
-      <c r="C118" s="25" t="s">
-        <v>361</v>
       </c>
       <c r="D118" s="21" t="s">
         <v>118</v>
@@ -8982,13 +8982,13 @@
     </row>
     <row r="119" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B119" s="25" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C119" s="25" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D119" s="21" t="s">
         <v>118</v>
@@ -8999,13 +8999,13 @@
     </row>
     <row r="120" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="B120" s="25" t="s">
         <v>366</v>
       </c>
-      <c r="B120" s="25" t="s">
-        <v>365</v>
-      </c>
       <c r="C120" s="25" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D120" s="21" t="s">
         <v>118</v>
@@ -9016,13 +9016,13 @@
     </row>
     <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="B121" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="C121" s="25" t="s">
         <v>368</v>
-      </c>
-      <c r="B121" s="25" t="s">
-        <v>369</v>
-      </c>
-      <c r="C121" s="25" t="s">
-        <v>367</v>
       </c>
       <c r="D121" s="21" t="s">
         <v>118</v>
@@ -9033,13 +9033,13 @@
     </row>
     <row r="122" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="13" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B122" s="25" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C122" s="25" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D122" s="21" t="s">
         <v>118</v>
@@ -9050,13 +9050,13 @@
     </row>
     <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="13" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B123" s="25" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C123" s="25" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D123" s="21" t="s">
         <v>118</v>
@@ -9067,13 +9067,13 @@
     </row>
     <row r="124" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="13" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B124" s="25" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C124" s="25" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D124" s="21" t="s">
         <v>118</v>
@@ -9084,13 +9084,13 @@
     </row>
     <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="13" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B125" s="25" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C125" s="25" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D125" s="21" t="s">
         <v>118</v>
@@ -9101,13 +9101,13 @@
     </row>
     <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="B126" s="25" t="s">
+        <v>381</v>
+      </c>
+      <c r="C126" s="25" t="s">
         <v>379</v>
-      </c>
-      <c r="B126" s="25" t="s">
-        <v>380</v>
-      </c>
-      <c r="C126" s="25" t="s">
-        <v>378</v>
       </c>
       <c r="D126" s="21" t="s">
         <v>118</v>
@@ -9118,13 +9118,13 @@
     </row>
     <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="13" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B127" s="25" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C127" s="25" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D127" s="21" t="s">
         <v>118</v>
@@ -9135,13 +9135,13 @@
     </row>
     <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="28" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B128" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C128" s="29" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>118</v>
@@ -9152,13 +9152,13 @@
     </row>
     <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="28" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B129" s="10" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C129" s="29" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>118</v>
@@ -9169,13 +9169,13 @@
     </row>
     <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="28" t="s">
+        <v>390</v>
+      </c>
+      <c r="B130" s="10" t="s">
+        <v>391</v>
+      </c>
+      <c r="C130" s="29" t="s">
         <v>389</v>
-      </c>
-      <c r="B130" s="10" t="s">
-        <v>390</v>
-      </c>
-      <c r="C130" s="29" t="s">
-        <v>388</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>118</v>
@@ -9186,13 +9186,13 @@
     </row>
     <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="28" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C131" s="29" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>118</v>
@@ -9203,13 +9203,13 @@
     </row>
     <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="28" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C132" s="29" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>118</v>
@@ -9220,13 +9220,13 @@
     </row>
     <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="28" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C133" s="29" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>118</v>
@@ -9237,13 +9237,13 @@
     </row>
     <row r="134" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="28" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>118</v>
@@ -9254,13 +9254,13 @@
     </row>
     <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="28" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C135" s="29" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>118</v>
@@ -9271,13 +9271,13 @@
     </row>
     <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="28" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C136" s="29" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>118</v>
@@ -9288,13 +9288,13 @@
     </row>
     <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="28" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C137" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>118</v>
@@ -9305,13 +9305,13 @@
     </row>
     <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="28" t="s">
+        <v>407</v>
+      </c>
+      <c r="B138" s="10" t="s">
+        <v>408</v>
+      </c>
+      <c r="C138" s="10" t="s">
         <v>406</v>
-      </c>
-      <c r="B138" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="C138" s="10" t="s">
-        <v>405</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>118</v>
@@ -9322,13 +9322,13 @@
     </row>
     <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="28" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B139" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C139" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>118</v>
@@ -9339,13 +9339,13 @@
     </row>
     <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="28" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B140" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C140" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>118</v>
@@ -9356,13 +9356,13 @@
     </row>
     <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="28" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>118</v>
@@ -9373,13 +9373,13 @@
     </row>
     <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="28" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>118</v>
@@ -9390,13 +9390,13 @@
     </row>
     <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="28" t="s">
+        <v>418</v>
+      </c>
+      <c r="B143" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="C143" s="10" t="s">
         <v>417</v>
-      </c>
-      <c r="B143" s="10" t="s">
-        <v>418</v>
-      </c>
-      <c r="C143" s="10" t="s">
-        <v>416</v>
       </c>
       <c r="D143" s="30" t="s">
         <v>118</v>
@@ -9407,13 +9407,13 @@
     </row>
     <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="28" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D144" s="30" t="s">
         <v>118</v>
@@ -9424,13 +9424,13 @@
     </row>
     <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="28" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C145" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D145" s="30" t="s">
         <v>118</v>
@@ -9441,13 +9441,13 @@
     </row>
     <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="28" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B146" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C146" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D146" s="30" t="s">
         <v>118</v>
@@ -9458,13 +9458,13 @@
     </row>
     <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="28" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C147" s="10" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D147" s="30" t="s">
         <v>118</v>
@@ -9475,13 +9475,13 @@
     </row>
     <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="28" t="s">
+        <v>429</v>
+      </c>
+      <c r="B148" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="C148" s="10" t="s">
         <v>428</v>
-      </c>
-      <c r="B148" s="10" t="s">
-        <v>429</v>
-      </c>
-      <c r="C148" s="10" t="s">
-        <v>427</v>
       </c>
       <c r="D148" s="30" t="s">
         <v>118</v>
@@ -9492,13 +9492,13 @@
     </row>
     <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="28" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C149" s="10" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D149" s="30" t="s">
         <v>118</v>
@@ -9509,13 +9509,13 @@
     </row>
     <row r="150" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="8" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D150" s="31" t="s">
         <v>118</v>
@@ -9526,19 +9526,19 @@
     </row>
     <row r="151" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="8" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D151" s="31" t="s">
         <v>118</v>
       </c>
       <c r="E151" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9549,7 +9549,7 @@
         <v>440</v>
       </c>
       <c r="C152" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D152" s="31" t="s">
         <v>118</v>
@@ -9589,7 +9589,7 @@
         <v>118</v>
       </c>
       <c r="E154" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9835,7 +9835,7 @@
         <v>478</v>
       </c>
       <c r="B169" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C169" s="8" t="s">
         <v>473</v>
@@ -9861,7 +9861,7 @@
         <v>118</v>
       </c>
       <c r="E170" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9988,7 +9988,7 @@
         <v>496</v>
       </c>
       <c r="B178" s="33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C178" s="8" t="s">
         <v>489</v>
@@ -10127,7 +10127,7 @@
         <v>515</v>
       </c>
       <c r="C186" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D186" s="31" t="s">
         <v>118</v>
@@ -10144,7 +10144,7 @@
         <v>517</v>
       </c>
       <c r="C187" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D187" s="31" t="s">
         <v>118</v>
@@ -10430,7 +10430,7 @@
         <v>555</v>
       </c>
       <c r="B204" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C204" s="8" t="s">
         <v>554</v>
@@ -10464,7 +10464,7 @@
         <v>558</v>
       </c>
       <c r="B206" s="8" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C206" s="8" t="s">
         <v>554</v>
@@ -10481,7 +10481,7 @@
         <v>559</v>
       </c>
       <c r="B207" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C207" s="8" t="s">
         <v>554</v>
@@ -11952,7 +11952,7 @@
         <v>118</v>
       </c>
       <c r="E293" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="294" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12836,7 +12836,7 @@
         <v>118</v>
       </c>
       <c r="E345" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="346" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12887,7 +12887,7 @@
         <v>118</v>
       </c>
       <c r="E348" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="349" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12972,7 +12972,7 @@
         <v>118</v>
       </c>
       <c r="E353" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="354" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13125,7 +13125,7 @@
         <v>118</v>
       </c>
       <c r="E362" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="363" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13159,7 +13159,7 @@
         <v>118</v>
       </c>
       <c r="E364" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="365" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13261,7 +13261,7 @@
         <v>118</v>
       </c>
       <c r="E370" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="371" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13380,7 +13380,7 @@
         <v>118</v>
       </c>
       <c r="E377" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="378" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13431,7 +13431,7 @@
         <v>118</v>
       </c>
       <c r="E380" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="381" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15465,7 +15465,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="23.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="38" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="38" width="25.4"/>
@@ -15497,7 +15497,7 @@
         <v>1228</v>
       </c>
       <c r="D2" s="41" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -15523,7 +15523,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -15556,7 +15556,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="23.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="24.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
@@ -15589,7 +15589,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E497"/>
-  <sheetFormatPr defaultColWidth="57.00390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="57.3828125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="69.46"/>
@@ -15628,7 +15628,7 @@
         <v>1232</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15645,7 +15645,7 @@
         <v>1232</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15662,7 +15662,7 @@
         <v>1232</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15679,7 +15679,7 @@
         <v>1232</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15696,7 +15696,7 @@
         <v>1232</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15713,7 +15713,7 @@
         <v>1232</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15730,7 +15730,7 @@
         <v>1232</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15747,7 +15747,7 @@
         <v>1232</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15764,7 +15764,7 @@
         <v>1232</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15781,7 +15781,7 @@
         <v>1232</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15798,7 +15798,7 @@
         <v>1232</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15815,7 +15815,7 @@
         <v>1232</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15832,7 +15832,7 @@
         <v>1232</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15849,7 +15849,7 @@
         <v>1232</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15866,7 +15866,7 @@
         <v>1232</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15883,7 +15883,7 @@
         <v>1232</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15900,7 +15900,7 @@
         <v>1232</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15917,7 +15917,7 @@
         <v>1232</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15934,7 +15934,7 @@
         <v>1232</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15951,7 +15951,7 @@
         <v>1232</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15968,7 +15968,7 @@
         <v>1232</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15985,7 +15985,7 @@
         <v>1232</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16002,7 +16002,7 @@
         <v>1232</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16019,7 +16019,7 @@
         <v>1232</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16036,7 +16036,7 @@
         <v>1232</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16053,7 +16053,7 @@
         <v>1232</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16070,7 +16070,7 @@
         <v>1232</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16087,7 +16087,7 @@
         <v>1232</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16104,7 +16104,7 @@
         <v>1232</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16121,7 +16121,7 @@
         <v>1232</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16138,7 +16138,7 @@
         <v>1232</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16155,7 +16155,7 @@
         <v>1232</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16172,7 +16172,7 @@
         <v>1232</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16189,7 +16189,7 @@
         <v>1232</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16206,7 +16206,7 @@
         <v>1232</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16223,7 +16223,7 @@
         <v>1232</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16240,7 +16240,7 @@
         <v>1232</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16257,7 +16257,7 @@
         <v>1232</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16274,7 +16274,7 @@
         <v>1232</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16291,7 +16291,7 @@
         <v>1232</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16308,7 +16308,7 @@
         <v>1232</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16325,7 +16325,7 @@
         <v>1232</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16342,7 +16342,7 @@
         <v>1232</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16359,7 +16359,7 @@
         <v>1232</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16376,7 +16376,7 @@
         <v>1232</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16393,7 +16393,7 @@
         <v>1232</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16410,7 +16410,7 @@
         <v>1232</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16427,7 +16427,7 @@
         <v>1232</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16444,7 +16444,7 @@
         <v>1232</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16461,7 +16461,7 @@
         <v>1232</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16478,7 +16478,7 @@
         <v>1232</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16495,7 +16495,7 @@
         <v>1232</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16512,7 +16512,7 @@
         <v>1232</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16529,7 +16529,7 @@
         <v>1232</v>
       </c>
       <c r="E55" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16546,7 +16546,7 @@
         <v>1232</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16563,7 +16563,7 @@
         <v>1232</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16580,7 +16580,7 @@
         <v>1232</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16597,7 +16597,7 @@
         <v>1232</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16614,7 +16614,7 @@
         <v>1232</v>
       </c>
       <c r="E60" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16631,7 +16631,7 @@
         <v>1232</v>
       </c>
       <c r="E61" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16648,7 +16648,7 @@
         <v>1232</v>
       </c>
       <c r="E62" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16665,7 +16665,7 @@
         <v>1232</v>
       </c>
       <c r="E63" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16682,7 +16682,7 @@
         <v>1232</v>
       </c>
       <c r="E64" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16699,7 +16699,7 @@
         <v>1232</v>
       </c>
       <c r="E65" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16716,7 +16716,7 @@
         <v>1232</v>
       </c>
       <c r="E66" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16733,7 +16733,7 @@
         <v>1232</v>
       </c>
       <c r="E67" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16750,7 +16750,7 @@
         <v>1232</v>
       </c>
       <c r="E68" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16767,7 +16767,7 @@
         <v>1232</v>
       </c>
       <c r="E69" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16784,7 +16784,7 @@
         <v>1232</v>
       </c>
       <c r="E70" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16801,7 +16801,7 @@
         <v>1232</v>
       </c>
       <c r="E71" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16818,7 +16818,7 @@
         <v>1232</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16835,7 +16835,7 @@
         <v>1232</v>
       </c>
       <c r="E73" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16852,7 +16852,7 @@
         <v>1232</v>
       </c>
       <c r="E74" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16869,7 +16869,7 @@
         <v>1232</v>
       </c>
       <c r="E75" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16886,7 +16886,7 @@
         <v>1232</v>
       </c>
       <c r="E76" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16903,7 +16903,7 @@
         <v>1232</v>
       </c>
       <c r="E77" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16920,7 +16920,7 @@
         <v>1232</v>
       </c>
       <c r="E78" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16937,7 +16937,7 @@
         <v>1232</v>
       </c>
       <c r="E79" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16954,7 +16954,7 @@
         <v>1232</v>
       </c>
       <c r="E80" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16971,7 +16971,7 @@
         <v>1232</v>
       </c>
       <c r="E81" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16988,7 +16988,7 @@
         <v>1232</v>
       </c>
       <c r="E82" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17005,7 +17005,7 @@
         <v>1232</v>
       </c>
       <c r="E83" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17022,7 +17022,7 @@
         <v>1232</v>
       </c>
       <c r="E84" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17039,7 +17039,7 @@
         <v>1232</v>
       </c>
       <c r="E85" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17056,7 +17056,7 @@
         <v>1232</v>
       </c>
       <c r="E86" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17073,7 +17073,7 @@
         <v>1232</v>
       </c>
       <c r="E87" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17090,7 +17090,7 @@
         <v>1232</v>
       </c>
       <c r="E88" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17107,7 +17107,7 @@
         <v>1232</v>
       </c>
       <c r="E89" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17124,7 +17124,7 @@
         <v>1232</v>
       </c>
       <c r="E90" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17141,7 +17141,7 @@
         <v>1232</v>
       </c>
       <c r="E91" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17158,7 +17158,7 @@
         <v>1232</v>
       </c>
       <c r="E92" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17175,7 +17175,7 @@
         <v>1232</v>
       </c>
       <c r="E93" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17192,7 +17192,7 @@
         <v>1232</v>
       </c>
       <c r="E94" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17209,7 +17209,7 @@
         <v>1232</v>
       </c>
       <c r="E95" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17226,7 +17226,7 @@
         <v>1232</v>
       </c>
       <c r="E96" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17243,7 +17243,7 @@
         <v>1232</v>
       </c>
       <c r="E97" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17260,7 +17260,7 @@
         <v>1232</v>
       </c>
       <c r="E98" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17277,7 +17277,7 @@
         <v>1232</v>
       </c>
       <c r="E99" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17294,7 +17294,7 @@
         <v>1232</v>
       </c>
       <c r="E100" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17311,7 +17311,7 @@
         <v>1232</v>
       </c>
       <c r="E101" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17328,7 +17328,7 @@
         <v>1232</v>
       </c>
       <c r="E102" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17345,7 +17345,7 @@
         <v>1232</v>
       </c>
       <c r="E103" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17362,7 +17362,7 @@
         <v>1232</v>
       </c>
       <c r="E104" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17379,7 +17379,7 @@
         <v>1232</v>
       </c>
       <c r="E105" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17396,7 +17396,7 @@
         <v>1232</v>
       </c>
       <c r="E106" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17413,7 +17413,7 @@
         <v>1232</v>
       </c>
       <c r="E107" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17430,7 +17430,7 @@
         <v>1232</v>
       </c>
       <c r="E108" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17447,7 +17447,7 @@
         <v>1232</v>
       </c>
       <c r="E109" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17464,7 +17464,7 @@
         <v>1232</v>
       </c>
       <c r="E110" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17481,7 +17481,7 @@
         <v>1232</v>
       </c>
       <c r="E111" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17498,7 +17498,7 @@
         <v>1232</v>
       </c>
       <c r="E112" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17515,7 +17515,7 @@
         <v>1232</v>
       </c>
       <c r="E113" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17532,7 +17532,7 @@
         <v>1232</v>
       </c>
       <c r="E114" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17549,7 +17549,7 @@
         <v>1232</v>
       </c>
       <c r="E115" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17566,7 +17566,7 @@
         <v>1232</v>
       </c>
       <c r="E116" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17583,7 +17583,7 @@
         <v>1232</v>
       </c>
       <c r="E117" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17600,7 +17600,7 @@
         <v>1232</v>
       </c>
       <c r="E118" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17617,7 +17617,7 @@
         <v>1232</v>
       </c>
       <c r="E119" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17634,7 +17634,7 @@
         <v>1232</v>
       </c>
       <c r="E120" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17651,7 +17651,7 @@
         <v>1232</v>
       </c>
       <c r="E121" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17668,7 +17668,7 @@
         <v>1232</v>
       </c>
       <c r="E122" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17685,7 +17685,7 @@
         <v>1232</v>
       </c>
       <c r="E123" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17702,7 +17702,7 @@
         <v>1232</v>
       </c>
       <c r="E124" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17719,7 +17719,7 @@
         <v>1232</v>
       </c>
       <c r="E125" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17736,7 +17736,7 @@
         <v>1232</v>
       </c>
       <c r="E126" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17753,7 +17753,7 @@
         <v>1232</v>
       </c>
       <c r="E127" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17770,7 +17770,7 @@
         <v>1232</v>
       </c>
       <c r="E128" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17787,7 +17787,7 @@
         <v>1232</v>
       </c>
       <c r="E129" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17804,7 +17804,7 @@
         <v>1232</v>
       </c>
       <c r="E130" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17821,7 +17821,7 @@
         <v>1232</v>
       </c>
       <c r="E131" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17838,7 +17838,7 @@
         <v>1232</v>
       </c>
       <c r="E132" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17855,7 +17855,7 @@
         <v>1232</v>
       </c>
       <c r="E133" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17872,7 +17872,7 @@
         <v>1232</v>
       </c>
       <c r="E134" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17889,7 +17889,7 @@
         <v>1232</v>
       </c>
       <c r="E135" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17906,7 +17906,7 @@
         <v>1232</v>
       </c>
       <c r="E136" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17923,7 +17923,7 @@
         <v>1232</v>
       </c>
       <c r="E137" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17940,7 +17940,7 @@
         <v>1232</v>
       </c>
       <c r="E138" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17957,7 +17957,7 @@
         <v>1232</v>
       </c>
       <c r="E139" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17974,7 +17974,7 @@
         <v>1232</v>
       </c>
       <c r="E140" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17991,7 +17991,7 @@
         <v>1232</v>
       </c>
       <c r="E141" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18008,7 +18008,7 @@
         <v>1232</v>
       </c>
       <c r="E142" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18025,7 +18025,7 @@
         <v>1232</v>
       </c>
       <c r="E143" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18042,7 +18042,7 @@
         <v>1232</v>
       </c>
       <c r="E144" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18059,7 +18059,7 @@
         <v>1232</v>
       </c>
       <c r="E145" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18076,7 +18076,7 @@
         <v>1232</v>
       </c>
       <c r="E146" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18093,7 +18093,7 @@
         <v>1232</v>
       </c>
       <c r="E147" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18110,7 +18110,7 @@
         <v>1232</v>
       </c>
       <c r="E148" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18127,7 +18127,7 @@
         <v>1232</v>
       </c>
       <c r="E149" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18144,7 +18144,7 @@
         <v>1232</v>
       </c>
       <c r="E150" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18161,7 +18161,7 @@
         <v>1232</v>
       </c>
       <c r="E151" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18178,7 +18178,7 @@
         <v>1232</v>
       </c>
       <c r="E152" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18195,7 +18195,7 @@
         <v>1232</v>
       </c>
       <c r="E153" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18212,7 +18212,7 @@
         <v>1232</v>
       </c>
       <c r="E154" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18229,7 +18229,7 @@
         <v>1232</v>
       </c>
       <c r="E155" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18246,7 +18246,7 @@
         <v>1232</v>
       </c>
       <c r="E156" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18263,7 +18263,7 @@
         <v>1232</v>
       </c>
       <c r="E157" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18280,7 +18280,7 @@
         <v>1232</v>
       </c>
       <c r="E158" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18297,7 +18297,7 @@
         <v>1232</v>
       </c>
       <c r="E159" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18314,7 +18314,7 @@
         <v>1232</v>
       </c>
       <c r="E160" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18331,7 +18331,7 @@
         <v>1232</v>
       </c>
       <c r="E161" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18348,7 +18348,7 @@
         <v>1232</v>
       </c>
       <c r="E162" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18365,7 +18365,7 @@
         <v>1232</v>
       </c>
       <c r="E163" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18382,7 +18382,7 @@
         <v>1232</v>
       </c>
       <c r="E164" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18399,7 +18399,7 @@
         <v>1232</v>
       </c>
       <c r="E165" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18416,7 +18416,7 @@
         <v>1232</v>
       </c>
       <c r="E166" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18433,7 +18433,7 @@
         <v>1232</v>
       </c>
       <c r="E167" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18450,7 +18450,7 @@
         <v>1232</v>
       </c>
       <c r="E168" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18467,7 +18467,7 @@
         <v>1232</v>
       </c>
       <c r="E169" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18484,7 +18484,7 @@
         <v>1232</v>
       </c>
       <c r="E170" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18501,7 +18501,7 @@
         <v>1232</v>
       </c>
       <c r="E171" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18518,7 +18518,7 @@
         <v>1232</v>
       </c>
       <c r="E172" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18535,7 +18535,7 @@
         <v>1232</v>
       </c>
       <c r="E173" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18552,7 +18552,7 @@
         <v>1232</v>
       </c>
       <c r="E174" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18569,7 +18569,7 @@
         <v>1232</v>
       </c>
       <c r="E175" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18586,7 +18586,7 @@
         <v>1232</v>
       </c>
       <c r="E176" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18603,7 +18603,7 @@
         <v>1232</v>
       </c>
       <c r="E177" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18620,7 +18620,7 @@
         <v>1232</v>
       </c>
       <c r="E178" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18637,7 +18637,7 @@
         <v>1232</v>
       </c>
       <c r="E179" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18654,7 +18654,7 @@
         <v>1232</v>
       </c>
       <c r="E180" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18671,7 +18671,7 @@
         <v>1232</v>
       </c>
       <c r="E181" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18688,7 +18688,7 @@
         <v>1232</v>
       </c>
       <c r="E182" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18705,7 +18705,7 @@
         <v>1232</v>
       </c>
       <c r="E183" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18722,7 +18722,7 @@
         <v>1232</v>
       </c>
       <c r="E184" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18739,7 +18739,7 @@
         <v>1232</v>
       </c>
       <c r="E185" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18756,7 +18756,7 @@
         <v>1232</v>
       </c>
       <c r="E186" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18773,7 +18773,7 @@
         <v>1232</v>
       </c>
       <c r="E187" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18790,7 +18790,7 @@
         <v>1232</v>
       </c>
       <c r="E188" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18807,7 +18807,7 @@
         <v>1232</v>
       </c>
       <c r="E189" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18824,7 +18824,7 @@
         <v>1232</v>
       </c>
       <c r="E190" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18841,7 +18841,7 @@
         <v>1232</v>
       </c>
       <c r="E191" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18858,7 +18858,7 @@
         <v>1232</v>
       </c>
       <c r="E192" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18875,7 +18875,7 @@
         <v>1232</v>
       </c>
       <c r="E193" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18892,7 +18892,7 @@
         <v>1232</v>
       </c>
       <c r="E194" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18909,7 +18909,7 @@
         <v>1232</v>
       </c>
       <c r="E195" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18926,7 +18926,7 @@
         <v>1232</v>
       </c>
       <c r="E196" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18943,7 +18943,7 @@
         <v>1232</v>
       </c>
       <c r="E197" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18960,7 +18960,7 @@
         <v>1232</v>
       </c>
       <c r="E198" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18977,7 +18977,7 @@
         <v>1232</v>
       </c>
       <c r="E199" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18994,7 +18994,7 @@
         <v>1232</v>
       </c>
       <c r="E200" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19011,7 +19011,7 @@
         <v>1232</v>
       </c>
       <c r="E201" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19028,7 +19028,7 @@
         <v>1232</v>
       </c>
       <c r="E202" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19045,7 +19045,7 @@
         <v>1232</v>
       </c>
       <c r="E203" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19062,7 +19062,7 @@
         <v>1232</v>
       </c>
       <c r="E204" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19079,7 +19079,7 @@
         <v>1232</v>
       </c>
       <c r="E205" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19096,7 +19096,7 @@
         <v>1232</v>
       </c>
       <c r="E206" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19113,7 +19113,7 @@
         <v>1232</v>
       </c>
       <c r="E207" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19130,7 +19130,7 @@
         <v>1232</v>
       </c>
       <c r="E208" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19147,7 +19147,7 @@
         <v>1232</v>
       </c>
       <c r="E209" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19164,7 +19164,7 @@
         <v>1232</v>
       </c>
       <c r="E210" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19181,7 +19181,7 @@
         <v>1232</v>
       </c>
       <c r="E211" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19198,7 +19198,7 @@
         <v>1232</v>
       </c>
       <c r="E212" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19215,7 +19215,7 @@
         <v>1232</v>
       </c>
       <c r="E213" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19232,7 +19232,7 @@
         <v>1232</v>
       </c>
       <c r="E214" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19249,7 +19249,7 @@
         <v>1232</v>
       </c>
       <c r="E215" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19266,7 +19266,7 @@
         <v>1232</v>
       </c>
       <c r="E216" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19283,7 +19283,7 @@
         <v>1232</v>
       </c>
       <c r="E217" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19300,7 +19300,7 @@
         <v>1232</v>
       </c>
       <c r="E218" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19317,7 +19317,7 @@
         <v>1232</v>
       </c>
       <c r="E219" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19334,7 +19334,7 @@
         <v>1232</v>
       </c>
       <c r="E220" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19351,7 +19351,7 @@
         <v>1232</v>
       </c>
       <c r="E221" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19368,7 +19368,7 @@
         <v>1232</v>
       </c>
       <c r="E222" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19385,7 +19385,7 @@
         <v>1232</v>
       </c>
       <c r="E223" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19402,7 +19402,7 @@
         <v>1232</v>
       </c>
       <c r="E224" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19419,7 +19419,7 @@
         <v>1232</v>
       </c>
       <c r="E225" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19436,7 +19436,7 @@
         <v>1232</v>
       </c>
       <c r="E226" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19453,7 +19453,7 @@
         <v>1232</v>
       </c>
       <c r="E227" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19470,7 +19470,7 @@
         <v>1232</v>
       </c>
       <c r="E228" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19487,7 +19487,7 @@
         <v>1232</v>
       </c>
       <c r="E229" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19504,7 +19504,7 @@
         <v>1232</v>
       </c>
       <c r="E230" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19521,7 +19521,7 @@
         <v>1232</v>
       </c>
       <c r="E231" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19538,7 +19538,7 @@
         <v>1232</v>
       </c>
       <c r="E232" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19555,7 +19555,7 @@
         <v>1232</v>
       </c>
       <c r="E233" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19572,7 +19572,7 @@
         <v>1232</v>
       </c>
       <c r="E234" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19589,7 +19589,7 @@
         <v>1232</v>
       </c>
       <c r="E235" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19606,7 +19606,7 @@
         <v>1232</v>
       </c>
       <c r="E236" s="22" t="s">
-        <v>438</v>
+        <v>9</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
added few changes in conftest
</commit_message>
<xml_diff>
--- a/DataProvider/TestCasesDetail.xlsx
+++ b/DataProvider/TestCasesDetail.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UI_SA" sheetId="1" state="visible" r:id="rId2"/>
@@ -2387,7 +2387,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
@@ -2420,7 +2420,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
@@ -5716,7 +5716,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="26.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="25.4"/>
@@ -5774,7 +5774,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
@@ -5807,7 +5807,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
@@ -5840,7 +5840,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">

</xml_diff>